<commit_message>
refactor: integrate player numbers into spreadsheet data, bracket cells, and tags with updated layout formatting
</commit_message>
<xml_diff>
--- a/playoffs-example-large-seeded.xlsx
+++ b/playoffs-example-large-seeded.xlsx
@@ -1453,11 +1453,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col customWidth="true" max="1" min="1" width="15"/>
-    <col customWidth="true" max="26" min="2" width="30"/>
+    <col customWidth="true" max="1" min="1" width="9"/>
+    <col customWidth="true" max="3" min="2" width="20"/>
+    <col customWidth="true" max="26" min="4" width="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2760,7 +2764,8 @@
       </c>
     </row>
   </sheetData>
-  <pageSetup orientation="landscape"/>
+  <printOptions horizontalCentered="true" verticalCentered="true"/>
+  <pageSetup fitToHeight="0" fitToWidth="1" orientation="portrait" paperSize="9"/>
 </worksheet>
 </file>
 
@@ -2768,7 +2773,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>
   <cols>
-    <col customWidth="true" max="1" min="1" width="20.83"/>
+    <col customWidth="true" max="1" min="1" width="25"/>
     <col customWidth="true" max="2" min="2" width="10"/>
     <col customWidth="true" max="26" min="3" width="3.5"/>
   </cols>
@@ -2991,7 +2996,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>
   <cols>
-    <col customWidth="true" max="1" min="1" width="20.83"/>
+    <col customWidth="true" max="1" min="1" width="25"/>
     <col customWidth="true" max="2" min="2" width="10"/>
     <col customWidth="true" max="26" min="3" width="3.5"/>
   </cols>
@@ -3223,7 +3228,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>
   <cols>
-    <col customWidth="true" max="1" min="1" width="20.83"/>
+    <col customWidth="true" max="1" min="1" width="25"/>
     <col customWidth="true" max="2" min="2" width="10"/>
     <col customWidth="true" max="26" min="3" width="3.5"/>
   </cols>
@@ -3446,7 +3451,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>
   <cols>
-    <col customWidth="true" max="1" min="1" width="20.83"/>
+    <col customWidth="true" max="1" min="1" width="25"/>
     <col customWidth="true" max="2" min="2" width="10"/>
     <col customWidth="true" max="26" min="3" width="3.5"/>
   </cols>
@@ -3678,7 +3683,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>
   <cols>
-    <col customWidth="true" max="1" min="1" width="20.83"/>
+    <col customWidth="true" max="1" min="1" width="25"/>
     <col customWidth="true" max="2" min="2" width="10"/>
     <col customWidth="true" max="26" min="3" width="3.5"/>
   </cols>
@@ -3901,7 +3906,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>
   <cols>
-    <col customWidth="true" max="1" min="1" width="20.83"/>
+    <col customWidth="true" max="1" min="1" width="25"/>
     <col customWidth="true" max="2" min="2" width="10"/>
     <col customWidth="true" max="26" min="3" width="3.5"/>
   </cols>
@@ -9131,7 +9136,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>
   <cols>
-    <col customWidth="true" max="1" min="1" width="20.83"/>
+    <col customWidth="true" max="1" min="1" width="25"/>
     <col customWidth="true" max="2" min="2" width="10"/>
     <col customWidth="true" max="26" min="3" width="3.5"/>
   </cols>
@@ -9354,7 +9359,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>
   <cols>
-    <col customWidth="true" max="1" min="1" width="20.83"/>
+    <col customWidth="true" max="1" min="1" width="25"/>
     <col customWidth="true" max="2" min="2" width="10"/>
     <col customWidth="true" max="26" min="3" width="3.5"/>
   </cols>

</xml_diff>

<commit_message>
feat: refactor output to support per-court sheets for player names and improve multi-page bracket match numbering
</commit_message>
<xml_diff>
--- a/playoffs-example-large-seeded.xlsx
+++ b/playoffs-example-large-seeded.xlsx
@@ -10,7 +10,6 @@
     <sheet name="data" sheetId="1" r:id="rId1"/>
     <sheet name="Time Estimator" sheetId="2" r:id="rId4"/>
     <sheet name="Elimination Matches" sheetId="5" r:id="rId7"/>
-    <sheet name="Names to Print" sheetId="6" r:id="rId8"/>
     <sheet name="Tree 1" sheetId="8" r:id="rId11"/>
     <sheet name="Tree 2" sheetId="9" r:id="rId12"/>
     <sheet name="Tree 3" sheetId="10" r:id="rId13"/>
@@ -19,9 +18,12 @@
     <sheet name="Tree 6" sheetId="13" r:id="rId16"/>
     <sheet name="Tree 7" sheetId="14" r:id="rId17"/>
     <sheet name="Tree 8" sheetId="15" r:id="rId18"/>
+    <sheet name="Names to Print A" sheetId="16" r:id="rId19"/>
+    <sheet name="Names to Print B" sheetId="17" r:id="rId20"/>
   </sheets>
   <definedNames>
-    <definedName localSheetId="3" name="_xlnm.Print_Area">'Names to Print'!$A$1:$B$91</definedName>
+    <definedName localSheetId="11" name="_xlnm.Print_Area">'Names to Print A'!$A$1:$B$46</definedName>
+    <definedName localSheetId="12" name="_xlnm.Print_Area">'Names to Print B'!$A$1:$B$45</definedName>
     <definedName localSheetId="2" name="_xlnm.Print_Area">'Elimination Matches'!$A$1:$O$404</definedName>
   </definedNames>
   <calcPr calcId="122211"/>
@@ -29,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="306">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="310">
   <si>
     <t>Number of pools</t>
   </si>
@@ -919,13 +921,25 @@
     <t>Round 4 - Match 83</t>
   </si>
   <si>
-    <t>Round 5 - Match 0</t>
-  </si>
-  <si>
-    <t>Round 6 - Match 0</t>
-  </si>
-  <si>
-    <t>Round 7 - Match 0</t>
+    <t>Round 5 - Match 84</t>
+  </si>
+  <si>
+    <t>Round 5 - Match 86</t>
+  </si>
+  <si>
+    <t>Round 5 - Match 85</t>
+  </si>
+  <si>
+    <t>Round 5 - Match 87</t>
+  </si>
+  <si>
+    <t>Round 6 - Match 88</t>
+  </si>
+  <si>
+    <t>Round 6 - Match 89</t>
+  </si>
+  <si>
+    <t>Round 7 - Match 90</t>
   </si>
   <si>
     <t>Tournament Summary</t>
@@ -4134,6 +4148,798 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <cols>
+    <col customWidth="true" max="1" min="1" width="30"/>
+    <col customWidth="true" max="2" min="2" width="160"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="270" customHeight="true">
+      <c r="A1" s="17">
+        <v>0</v>
+      </c>
+      <c r="B1" s="18" t="str">
+        <f>data!D3</f>
+      </c>
+    </row>
+    <row r="2" ht="270" customHeight="true">
+      <c r="A2" s="17">
+        <v>4</v>
+      </c>
+      <c r="B2" s="18" t="str">
+        <f>data!D7</f>
+      </c>
+    </row>
+    <row r="3" ht="270" customHeight="true">
+      <c r="A3" s="17">
+        <v>5</v>
+      </c>
+      <c r="B3" s="18" t="str">
+        <f>data!D8</f>
+      </c>
+    </row>
+    <row r="4" ht="270" customHeight="true">
+      <c r="A4" s="17">
+        <v>6</v>
+      </c>
+      <c r="B4" s="18" t="str">
+        <f>data!D9</f>
+      </c>
+    </row>
+    <row r="5" ht="270" customHeight="true">
+      <c r="A5" s="17">
+        <v>7</v>
+      </c>
+      <c r="B5" s="18" t="str">
+        <f>data!D10</f>
+      </c>
+    </row>
+    <row r="6" ht="270" customHeight="true">
+      <c r="A6" s="17">
+        <v>8</v>
+      </c>
+      <c r="B6" s="18" t="str">
+        <f>data!D11</f>
+      </c>
+    </row>
+    <row r="7" ht="270" customHeight="true">
+      <c r="A7" s="17">
+        <v>9</v>
+      </c>
+      <c r="B7" s="18" t="str">
+        <f>data!D12</f>
+      </c>
+    </row>
+    <row r="8" ht="270" customHeight="true">
+      <c r="A8" s="17">
+        <v>10</v>
+      </c>
+      <c r="B8" s="18" t="str">
+        <f>data!D13</f>
+      </c>
+    </row>
+    <row r="9" ht="270" customHeight="true">
+      <c r="A9" s="17">
+        <v>11</v>
+      </c>
+      <c r="B9" s="18" t="str">
+        <f>data!D14</f>
+      </c>
+    </row>
+    <row r="10" ht="270" customHeight="true">
+      <c r="A10" s="17">
+        <v>12</v>
+      </c>
+      <c r="B10" s="18" t="str">
+        <f>data!D15</f>
+      </c>
+    </row>
+    <row r="11" ht="270" customHeight="true">
+      <c r="A11" s="17">
+        <v>13</v>
+      </c>
+      <c r="B11" s="18" t="str">
+        <f>data!D16</f>
+      </c>
+    </row>
+    <row r="12" ht="270" customHeight="true">
+      <c r="A12" s="17">
+        <v>14</v>
+      </c>
+      <c r="B12" s="18" t="str">
+        <f>data!D17</f>
+      </c>
+    </row>
+    <row r="13" ht="270" customHeight="true">
+      <c r="A13" s="17">
+        <v>15</v>
+      </c>
+      <c r="B13" s="18" t="str">
+        <f>data!D18</f>
+      </c>
+    </row>
+    <row r="14" ht="270" customHeight="true">
+      <c r="A14" s="17">
+        <v>16</v>
+      </c>
+      <c r="B14" s="18" t="str">
+        <f>data!D19</f>
+      </c>
+    </row>
+    <row r="15" ht="270" customHeight="true">
+      <c r="A15" s="17">
+        <v>17</v>
+      </c>
+      <c r="B15" s="18" t="str">
+        <f>data!D20</f>
+      </c>
+    </row>
+    <row r="16" ht="270" customHeight="true">
+      <c r="A16" s="17">
+        <v>18</v>
+      </c>
+      <c r="B16" s="18" t="str">
+        <f>data!D21</f>
+      </c>
+    </row>
+    <row r="17" ht="270" customHeight="true">
+      <c r="A17" s="17">
+        <v>19</v>
+      </c>
+      <c r="B17" s="18" t="str">
+        <f>data!D22</f>
+      </c>
+    </row>
+    <row r="18" ht="270" customHeight="true">
+      <c r="A18" s="17">
+        <v>20</v>
+      </c>
+      <c r="B18" s="18" t="str">
+        <f>data!D23</f>
+      </c>
+    </row>
+    <row r="19" ht="270" customHeight="true">
+      <c r="A19" s="17">
+        <v>21</v>
+      </c>
+      <c r="B19" s="18" t="str">
+        <f>data!D24</f>
+      </c>
+    </row>
+    <row r="20" ht="270" customHeight="true">
+      <c r="A20" s="17">
+        <v>22</v>
+      </c>
+      <c r="B20" s="18" t="str">
+        <f>data!D25</f>
+      </c>
+    </row>
+    <row r="21" ht="270" customHeight="true">
+      <c r="A21" s="17">
+        <v>23</v>
+      </c>
+      <c r="B21" s="18" t="str">
+        <f>data!D26</f>
+      </c>
+    </row>
+    <row r="22" ht="270" customHeight="true">
+      <c r="A22" s="17">
+        <v>24</v>
+      </c>
+      <c r="B22" s="18" t="str">
+        <f>data!D27</f>
+      </c>
+    </row>
+    <row r="23" ht="270" customHeight="true">
+      <c r="A23" s="17">
+        <v>25</v>
+      </c>
+      <c r="B23" s="18" t="str">
+        <f>data!D28</f>
+      </c>
+    </row>
+    <row r="24" ht="270" customHeight="true">
+      <c r="A24" s="17">
+        <v>26</v>
+      </c>
+      <c r="B24" s="18" t="str">
+        <f>data!D29</f>
+      </c>
+    </row>
+    <row r="25" ht="270" customHeight="true">
+      <c r="A25" s="17">
+        <v>27</v>
+      </c>
+      <c r="B25" s="18" t="str">
+        <f>data!D30</f>
+      </c>
+    </row>
+    <row r="26" ht="270" customHeight="true">
+      <c r="A26" s="17">
+        <v>28</v>
+      </c>
+      <c r="B26" s="18" t="str">
+        <f>data!D31</f>
+      </c>
+    </row>
+    <row r="27" ht="270" customHeight="true">
+      <c r="A27" s="17">
+        <v>29</v>
+      </c>
+      <c r="B27" s="18" t="str">
+        <f>data!D32</f>
+      </c>
+    </row>
+    <row r="28" ht="270" customHeight="true">
+      <c r="A28" s="17">
+        <v>30</v>
+      </c>
+      <c r="B28" s="18" t="str">
+        <f>data!D33</f>
+      </c>
+    </row>
+    <row r="29" ht="270" customHeight="true">
+      <c r="A29" s="17">
+        <v>31</v>
+      </c>
+      <c r="B29" s="18" t="str">
+        <f>data!D34</f>
+      </c>
+    </row>
+    <row r="30" ht="270" customHeight="true">
+      <c r="A30" s="17">
+        <v>32</v>
+      </c>
+      <c r="B30" s="18" t="str">
+        <f>data!D35</f>
+      </c>
+    </row>
+    <row r="31" ht="270" customHeight="true">
+      <c r="A31" s="17">
+        <v>33</v>
+      </c>
+      <c r="B31" s="18" t="str">
+        <f>data!D36</f>
+      </c>
+    </row>
+    <row r="32" ht="270" customHeight="true">
+      <c r="A32" s="17">
+        <v>34</v>
+      </c>
+      <c r="B32" s="18" t="str">
+        <f>data!D37</f>
+      </c>
+    </row>
+    <row r="33" ht="270" customHeight="true">
+      <c r="A33" s="17">
+        <v>3</v>
+      </c>
+      <c r="B33" s="18" t="str">
+        <f>data!D6</f>
+      </c>
+    </row>
+    <row r="34" ht="270" customHeight="true">
+      <c r="A34" s="17">
+        <v>35</v>
+      </c>
+      <c r="B34" s="18" t="str">
+        <f>data!D38</f>
+      </c>
+    </row>
+    <row r="35" ht="270" customHeight="true">
+      <c r="A35" s="17">
+        <v>36</v>
+      </c>
+      <c r="B35" s="18" t="str">
+        <f>data!D39</f>
+      </c>
+    </row>
+    <row r="36" ht="270" customHeight="true">
+      <c r="A36" s="17">
+        <v>37</v>
+      </c>
+      <c r="B36" s="18" t="str">
+        <f>data!D40</f>
+      </c>
+    </row>
+    <row r="37" ht="270" customHeight="true">
+      <c r="A37" s="17">
+        <v>38</v>
+      </c>
+      <c r="B37" s="18" t="str">
+        <f>data!D41</f>
+      </c>
+    </row>
+    <row r="38" ht="270" customHeight="true">
+      <c r="A38" s="17">
+        <v>39</v>
+      </c>
+      <c r="B38" s="18" t="str">
+        <f>data!D42</f>
+      </c>
+    </row>
+    <row r="39" ht="270" customHeight="true">
+      <c r="A39" s="17">
+        <v>40</v>
+      </c>
+      <c r="B39" s="18" t="str">
+        <f>data!D43</f>
+      </c>
+    </row>
+    <row r="40" ht="270" customHeight="true">
+      <c r="A40" s="17">
+        <v>41</v>
+      </c>
+      <c r="B40" s="18" t="str">
+        <f>data!D44</f>
+      </c>
+    </row>
+    <row r="41" ht="270" customHeight="true">
+      <c r="A41" s="17">
+        <v>42</v>
+      </c>
+      <c r="B41" s="18" t="str">
+        <f>data!D45</f>
+      </c>
+    </row>
+    <row r="42" ht="270" customHeight="true">
+      <c r="A42" s="17">
+        <v>43</v>
+      </c>
+      <c r="B42" s="18" t="str">
+        <f>data!D46</f>
+      </c>
+    </row>
+    <row r="43" ht="270" customHeight="true">
+      <c r="A43" s="17">
+        <v>44</v>
+      </c>
+      <c r="B43" s="18" t="str">
+        <f>data!D47</f>
+      </c>
+    </row>
+    <row r="44" ht="270" customHeight="true">
+      <c r="A44" s="17">
+        <v>45</v>
+      </c>
+      <c r="B44" s="18" t="str">
+        <f>data!D48</f>
+      </c>
+    </row>
+    <row r="45" ht="270" customHeight="true">
+      <c r="A45" s="17">
+        <v>46</v>
+      </c>
+      <c r="B45" s="18" t="str">
+        <f>data!D49</f>
+      </c>
+    </row>
+    <row r="46" ht="270" customHeight="true">
+      <c r="A46" s="17">
+        <v>47</v>
+      </c>
+      <c r="B46" s="18" t="str">
+        <f>data!D50</f>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.1" right="0.1" top="0.1" bottom="0.1" header="0.1" footer="0.1"/>
+  <pageSetup orientation="landscape" paperSize="8"/>
+  <rowBreaks count="15" manualBreakCount="15">
+    <brk id="3" max="16383" man="true"/>
+    <brk id="6" max="16383" man="true"/>
+    <brk id="9" max="16383" man="true"/>
+    <brk id="12" max="16383" man="true"/>
+    <brk id="15" max="16383" man="true"/>
+    <brk id="18" max="16383" man="true"/>
+    <brk id="21" max="16383" man="true"/>
+    <brk id="24" max="16383" man="true"/>
+    <brk id="27" max="16383" man="true"/>
+    <brk id="30" max="16383" man="true"/>
+    <brk id="33" max="16383" man="true"/>
+    <brk id="36" max="16383" man="true"/>
+    <brk id="39" max="16383" man="true"/>
+    <brk id="42" max="16383" man="true"/>
+    <brk id="45" max="16383" man="true"/>
+  </rowBreaks>
+  <colBreaks/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <cols>
+    <col customWidth="true" max="1" min="1" width="30"/>
+    <col customWidth="true" max="2" min="2" width="160"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="270" customHeight="true">
+      <c r="A1" s="17">
+        <v>48</v>
+      </c>
+      <c r="B1" s="18" t="str">
+        <f>data!D51</f>
+      </c>
+    </row>
+    <row r="2" ht="270" customHeight="true">
+      <c r="A2" s="17">
+        <v>49</v>
+      </c>
+      <c r="B2" s="18" t="str">
+        <f>data!D52</f>
+      </c>
+    </row>
+    <row r="3" ht="270" customHeight="true">
+      <c r="A3" s="17">
+        <v>50</v>
+      </c>
+      <c r="B3" s="18" t="str">
+        <f>data!D53</f>
+      </c>
+    </row>
+    <row r="4" ht="270" customHeight="true">
+      <c r="A4" s="17">
+        <v>51</v>
+      </c>
+      <c r="B4" s="18" t="str">
+        <f>data!D54</f>
+      </c>
+    </row>
+    <row r="5" ht="270" customHeight="true">
+      <c r="A5" s="17">
+        <v>52</v>
+      </c>
+      <c r="B5" s="18" t="str">
+        <f>data!D55</f>
+      </c>
+    </row>
+    <row r="6" ht="270" customHeight="true">
+      <c r="A6" s="17">
+        <v>53</v>
+      </c>
+      <c r="B6" s="18" t="str">
+        <f>data!D56</f>
+      </c>
+    </row>
+    <row r="7" ht="270" customHeight="true">
+      <c r="A7" s="17">
+        <v>54</v>
+      </c>
+      <c r="B7" s="18" t="str">
+        <f>data!D57</f>
+      </c>
+    </row>
+    <row r="8" ht="270" customHeight="true">
+      <c r="A8" s="17">
+        <v>55</v>
+      </c>
+      <c r="B8" s="18" t="str">
+        <f>data!D58</f>
+      </c>
+    </row>
+    <row r="9" ht="270" customHeight="true">
+      <c r="A9" s="17">
+        <v>56</v>
+      </c>
+      <c r="B9" s="18" t="str">
+        <f>data!D59</f>
+      </c>
+    </row>
+    <row r="10" ht="270" customHeight="true">
+      <c r="A10" s="17">
+        <v>57</v>
+      </c>
+      <c r="B10" s="18" t="str">
+        <f>data!D60</f>
+      </c>
+    </row>
+    <row r="11" ht="270" customHeight="true">
+      <c r="A11" s="17">
+        <v>58</v>
+      </c>
+      <c r="B11" s="18" t="str">
+        <f>data!D61</f>
+      </c>
+    </row>
+    <row r="12" ht="270" customHeight="true">
+      <c r="A12" s="17">
+        <v>59</v>
+      </c>
+      <c r="B12" s="18" t="str">
+        <f>data!D62</f>
+      </c>
+    </row>
+    <row r="13" ht="270" customHeight="true">
+      <c r="A13" s="17">
+        <v>60</v>
+      </c>
+      <c r="B13" s="18" t="str">
+        <f>data!D63</f>
+      </c>
+    </row>
+    <row r="14" ht="270" customHeight="true">
+      <c r="A14" s="17">
+        <v>61</v>
+      </c>
+      <c r="B14" s="18" t="str">
+        <f>data!D64</f>
+      </c>
+    </row>
+    <row r="15" ht="270" customHeight="true">
+      <c r="A15" s="17">
+        <v>62</v>
+      </c>
+      <c r="B15" s="18" t="str">
+        <f>data!D65</f>
+      </c>
+    </row>
+    <row r="16" ht="270" customHeight="true">
+      <c r="A16" s="17">
+        <v>63</v>
+      </c>
+      <c r="B16" s="18" t="str">
+        <f>data!D66</f>
+      </c>
+    </row>
+    <row r="17" ht="270" customHeight="true">
+      <c r="A17" s="17">
+        <v>64</v>
+      </c>
+      <c r="B17" s="18" t="str">
+        <f>data!D67</f>
+      </c>
+    </row>
+    <row r="18" ht="270" customHeight="true">
+      <c r="A18" s="17">
+        <v>65</v>
+      </c>
+      <c r="B18" s="18" t="str">
+        <f>data!D68</f>
+      </c>
+    </row>
+    <row r="19" ht="270" customHeight="true">
+      <c r="A19" s="17">
+        <v>1</v>
+      </c>
+      <c r="B19" s="18" t="str">
+        <f>data!D4</f>
+      </c>
+    </row>
+    <row r="20" ht="270" customHeight="true">
+      <c r="A20" s="17">
+        <v>66</v>
+      </c>
+      <c r="B20" s="18" t="str">
+        <f>data!D69</f>
+      </c>
+    </row>
+    <row r="21" ht="270" customHeight="true">
+      <c r="A21" s="17">
+        <v>67</v>
+      </c>
+      <c r="B21" s="18" t="str">
+        <f>data!D70</f>
+      </c>
+    </row>
+    <row r="22" ht="270" customHeight="true">
+      <c r="A22" s="17">
+        <v>68</v>
+      </c>
+      <c r="B22" s="18" t="str">
+        <f>data!D71</f>
+      </c>
+    </row>
+    <row r="23" ht="270" customHeight="true">
+      <c r="A23" s="17">
+        <v>69</v>
+      </c>
+      <c r="B23" s="18" t="str">
+        <f>data!D72</f>
+      </c>
+    </row>
+    <row r="24" ht="270" customHeight="true">
+      <c r="A24" s="17">
+        <v>70</v>
+      </c>
+      <c r="B24" s="18" t="str">
+        <f>data!D73</f>
+      </c>
+    </row>
+    <row r="25" ht="270" customHeight="true">
+      <c r="A25" s="17">
+        <v>71</v>
+      </c>
+      <c r="B25" s="18" t="str">
+        <f>data!D74</f>
+      </c>
+    </row>
+    <row r="26" ht="270" customHeight="true">
+      <c r="A26" s="17">
+        <v>72</v>
+      </c>
+      <c r="B26" s="18" t="str">
+        <f>data!D75</f>
+      </c>
+    </row>
+    <row r="27" ht="270" customHeight="true">
+      <c r="A27" s="17">
+        <v>73</v>
+      </c>
+      <c r="B27" s="18" t="str">
+        <f>data!D76</f>
+      </c>
+    </row>
+    <row r="28" ht="270" customHeight="true">
+      <c r="A28" s="17">
+        <v>74</v>
+      </c>
+      <c r="B28" s="18" t="str">
+        <f>data!D77</f>
+      </c>
+    </row>
+    <row r="29" ht="270" customHeight="true">
+      <c r="A29" s="17">
+        <v>75</v>
+      </c>
+      <c r="B29" s="18" t="str">
+        <f>data!D78</f>
+      </c>
+    </row>
+    <row r="30" ht="270" customHeight="true">
+      <c r="A30" s="17">
+        <v>76</v>
+      </c>
+      <c r="B30" s="18" t="str">
+        <f>data!D79</f>
+      </c>
+    </row>
+    <row r="31" ht="270" customHeight="true">
+      <c r="A31" s="17">
+        <v>77</v>
+      </c>
+      <c r="B31" s="18" t="str">
+        <f>data!D80</f>
+      </c>
+    </row>
+    <row r="32" ht="270" customHeight="true">
+      <c r="A32" s="17">
+        <v>78</v>
+      </c>
+      <c r="B32" s="18" t="str">
+        <f>data!D81</f>
+      </c>
+    </row>
+    <row r="33" ht="270" customHeight="true">
+      <c r="A33" s="17">
+        <v>79</v>
+      </c>
+      <c r="B33" s="18" t="str">
+        <f>data!D82</f>
+      </c>
+    </row>
+    <row r="34" ht="270" customHeight="true">
+      <c r="A34" s="17">
+        <v>80</v>
+      </c>
+      <c r="B34" s="18" t="str">
+        <f>data!D83</f>
+      </c>
+    </row>
+    <row r="35" ht="270" customHeight="true">
+      <c r="A35" s="17">
+        <v>81</v>
+      </c>
+      <c r="B35" s="18" t="str">
+        <f>data!D84</f>
+      </c>
+    </row>
+    <row r="36" ht="270" customHeight="true">
+      <c r="A36" s="17">
+        <v>82</v>
+      </c>
+      <c r="B36" s="18" t="str">
+        <f>data!D85</f>
+      </c>
+    </row>
+    <row r="37" ht="270" customHeight="true">
+      <c r="A37" s="17">
+        <v>83</v>
+      </c>
+      <c r="B37" s="18" t="str">
+        <f>data!D86</f>
+      </c>
+    </row>
+    <row r="38" ht="270" customHeight="true">
+      <c r="A38" s="17">
+        <v>84</v>
+      </c>
+      <c r="B38" s="18" t="str">
+        <f>data!D87</f>
+      </c>
+    </row>
+    <row r="39" ht="270" customHeight="true">
+      <c r="A39" s="17">
+        <v>85</v>
+      </c>
+      <c r="B39" s="18" t="str">
+        <f>data!D88</f>
+      </c>
+    </row>
+    <row r="40" ht="270" customHeight="true">
+      <c r="A40" s="17">
+        <v>86</v>
+      </c>
+      <c r="B40" s="18" t="str">
+        <f>data!D89</f>
+      </c>
+    </row>
+    <row r="41" ht="270" customHeight="true">
+      <c r="A41" s="17">
+        <v>87</v>
+      </c>
+      <c r="B41" s="18" t="str">
+        <f>data!D90</f>
+      </c>
+    </row>
+    <row r="42" ht="270" customHeight="true">
+      <c r="A42" s="17">
+        <v>88</v>
+      </c>
+      <c r="B42" s="18" t="str">
+        <f>data!D91</f>
+      </c>
+    </row>
+    <row r="43" ht="270" customHeight="true">
+      <c r="A43" s="17">
+        <v>89</v>
+      </c>
+      <c r="B43" s="18" t="str">
+        <f>data!D92</f>
+      </c>
+    </row>
+    <row r="44" ht="270" customHeight="true">
+      <c r="A44" s="17">
+        <v>90</v>
+      </c>
+      <c r="B44" s="18" t="str">
+        <f>data!D93</f>
+      </c>
+    </row>
+    <row r="45" ht="270" customHeight="true">
+      <c r="A45" s="17">
+        <v>2</v>
+      </c>
+      <c r="B45" s="18" t="str">
+        <f>data!D5</f>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.1" right="0.1" top="0.1" bottom="0.1" header="0.1" footer="0.1"/>
+  <pageSetup orientation="landscape" paperSize="8"/>
+  <rowBreaks count="15" manualBreakCount="15">
+    <brk id="3" max="16383" man="true"/>
+    <brk id="6" max="16383" man="true"/>
+    <brk id="9" max="16383" man="true"/>
+    <brk id="12" max="16383" man="true"/>
+    <brk id="15" max="16383" man="true"/>
+    <brk id="18" max="16383" man="true"/>
+    <brk id="21" max="16383" man="true"/>
+    <brk id="24" max="16383" man="true"/>
+    <brk id="27" max="16383" man="true"/>
+    <brk id="30" max="16383" man="true"/>
+    <brk id="33" max="16383" man="true"/>
+    <brk id="36" max="16383" man="true"/>
+    <brk id="39" max="16383" man="true"/>
+    <brk id="42" max="16383" man="true"/>
+    <brk id="45" max="16383" man="true"/>
+  </rowBreaks>
+  <colBreaks/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>
@@ -4334,7 +5140,7 @@
     </row>
     <row r="13">
       <c r="E13" s="11" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="F13" s="11"/>
       <c r="G13" s="11"/>
@@ -4345,7 +5151,7 @@
         <v>2</v>
       </c>
       <c r="E14" s="19" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="F14" s="19"/>
       <c r="G14" s="19"/>
@@ -4355,7 +5161,7 @@
     </row>
     <row r="15">
       <c r="E15" s="19" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="F15" s="19"/>
       <c r="G15" s="19"/>
@@ -4365,7 +5171,7 @@
     </row>
     <row r="16">
       <c r="E16" s="19" t="s">
-        <v>302</v>
+        <v>306</v>
       </c>
       <c r="F16" s="19"/>
       <c r="G16" s="19"/>
@@ -4375,7 +5181,7 @@
     </row>
     <row r="17">
       <c r="E17" s="19" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="F17" s="19"/>
       <c r="G17" s="19"/>
@@ -4385,7 +5191,7 @@
     </row>
     <row r="18">
       <c r="E18" s="11" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="F18" s="11"/>
       <c r="G18" s="11"/>
@@ -4395,7 +5201,7 @@
     </row>
     <row r="19">
       <c r="E19" s="11" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="F19" s="11"/>
       <c r="G19" s="11"/>
@@ -7955,7 +8761,7 @@
       <c r="F358" s="11"/>
       <c r="G358" s="11"/>
       <c r="I358" s="11" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="J358" s="11"/>
       <c r="K358" s="11"/>
@@ -8030,7 +8836,7 @@
     </row>
     <row r="366">
       <c r="A366" s="11" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B366" s="11"/>
       <c r="C366" s="11"/>
@@ -8039,7 +8845,7 @@
       <c r="F366" s="11"/>
       <c r="G366" s="11"/>
       <c r="I366" s="11" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="J366" s="11"/>
       <c r="K366" s="11"/>
@@ -8114,7 +8920,7 @@
     </row>
     <row r="379">
       <c r="A379" s="11" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="B379" s="11"/>
       <c r="C379" s="11"/>
@@ -8123,7 +8929,7 @@
       <c r="F379" s="11"/>
       <c r="G379" s="11"/>
       <c r="I379" s="11" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
       <c r="J379" s="11"/>
       <c r="K379" s="11"/>
@@ -8154,7 +8960,7 @@
     </row>
     <row r="381">
       <c r="A381" s="19" t="str">
-        <f>CONCATENATE("M 0 ",O370)</f>
+        <f>CONCATENATE("M 85 ",G370)</f>
       </c>
       <c r="B381" s="19"/>
       <c r="C381" s="19"/>
@@ -8162,10 +8968,10 @@
       <c r="E381" s="19"/>
       <c r="F381" s="19"/>
       <c r="G381" s="19" t="str">
-        <f>CONCATENATE("M 0 ",O370)</f>
+        <f>CONCATENATE("M 84 ",G362)</f>
       </c>
       <c r="I381" s="19" t="str">
-        <f>CONCATENATE("M 0 ",G383)</f>
+        <f>CONCATENATE("M 87 ",O370)</f>
       </c>
       <c r="J381" s="19"/>
       <c r="K381" s="19"/>
@@ -8173,7 +8979,7 @@
       <c r="M381" s="19"/>
       <c r="N381" s="19"/>
       <c r="O381" s="19" t="str">
-        <f>CONCATENATE("M 0 ",G383)</f>
+        <f>CONCATENATE("M 86 ",O362)</f>
       </c>
     </row>
     <row r="383">
@@ -8198,7 +9004,7 @@
     </row>
     <row r="392">
       <c r="A392" s="11" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="B392" s="11"/>
       <c r="C392" s="11"/>
@@ -8220,7 +9026,7 @@
     </row>
     <row r="394">
       <c r="A394" s="19" t="str">
-        <f>CONCATENATE("M 0 ",O383)</f>
+        <f>CONCATENATE("M 89 ",O383)</f>
       </c>
       <c r="B394" s="19"/>
       <c r="C394" s="19"/>
@@ -8228,7 +9034,7 @@
       <c r="E394" s="19"/>
       <c r="F394" s="19"/>
       <c r="G394" s="19" t="str">
-        <f>CONCATENATE("M 0 ",O383)</f>
+        <f>CONCATENATE("M 88 ",G383)</f>
       </c>
     </row>
     <row r="396">
@@ -8357,781 +9163,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1"/>
-  <cols>
-    <col customWidth="true" max="1" min="1" style="9" width="30"/>
-    <col customWidth="true" max="2" min="2" style="10" width="160"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="270" customHeight="true">
-      <c r="A1" s="17">
-        <v>0</v>
-      </c>
-      <c r="B1" s="18" t="str">
-        <f>data!D3</f>
-      </c>
-    </row>
-    <row r="2" ht="270" customHeight="true">
-      <c r="A2" s="17">
-        <v>4</v>
-      </c>
-      <c r="B2" s="18" t="str">
-        <f>data!D7</f>
-      </c>
-    </row>
-    <row r="3" ht="270" customHeight="true">
-      <c r="A3" s="17">
-        <v>5</v>
-      </c>
-      <c r="B3" s="18" t="str">
-        <f>data!D8</f>
-      </c>
-    </row>
-    <row r="4" ht="270" customHeight="true">
-      <c r="A4" s="17">
-        <v>6</v>
-      </c>
-      <c r="B4" s="18" t="str">
-        <f>data!D9</f>
-      </c>
-    </row>
-    <row r="5" ht="270" customHeight="true">
-      <c r="A5" s="17">
-        <v>7</v>
-      </c>
-      <c r="B5" s="18" t="str">
-        <f>data!D10</f>
-      </c>
-    </row>
-    <row r="6" ht="270" customHeight="true">
-      <c r="A6" s="17">
-        <v>8</v>
-      </c>
-      <c r="B6" s="18" t="str">
-        <f>data!D11</f>
-      </c>
-    </row>
-    <row r="7" ht="270" customHeight="true">
-      <c r="A7" s="17">
-        <v>9</v>
-      </c>
-      <c r="B7" s="18" t="str">
-        <f>data!D12</f>
-      </c>
-    </row>
-    <row r="8" ht="270" customHeight="true">
-      <c r="A8" s="17">
-        <v>10</v>
-      </c>
-      <c r="B8" s="18" t="str">
-        <f>data!D13</f>
-      </c>
-    </row>
-    <row r="9" ht="270" customHeight="true">
-      <c r="A9" s="17">
-        <v>11</v>
-      </c>
-      <c r="B9" s="18" t="str">
-        <f>data!D14</f>
-      </c>
-    </row>
-    <row r="10" ht="270" customHeight="true">
-      <c r="A10" s="17">
-        <v>12</v>
-      </c>
-      <c r="B10" s="18" t="str">
-        <f>data!D15</f>
-      </c>
-    </row>
-    <row r="11" ht="270" customHeight="true">
-      <c r="A11" s="17">
-        <v>13</v>
-      </c>
-      <c r="B11" s="18" t="str">
-        <f>data!D16</f>
-      </c>
-    </row>
-    <row r="12" ht="270" customHeight="true">
-      <c r="A12" s="17">
-        <v>14</v>
-      </c>
-      <c r="B12" s="18" t="str">
-        <f>data!D17</f>
-      </c>
-    </row>
-    <row r="13" ht="270" customHeight="true">
-      <c r="A13" s="17">
-        <v>15</v>
-      </c>
-      <c r="B13" s="18" t="str">
-        <f>data!D18</f>
-      </c>
-    </row>
-    <row r="14" ht="270" customHeight="true">
-      <c r="A14" s="17">
-        <v>16</v>
-      </c>
-      <c r="B14" s="18" t="str">
-        <f>data!D19</f>
-      </c>
-    </row>
-    <row r="15" ht="270" customHeight="true">
-      <c r="A15" s="17">
-        <v>17</v>
-      </c>
-      <c r="B15" s="18" t="str">
-        <f>data!D20</f>
-      </c>
-    </row>
-    <row r="16" ht="270" customHeight="true">
-      <c r="A16" s="17">
-        <v>18</v>
-      </c>
-      <c r="B16" s="18" t="str">
-        <f>data!D21</f>
-      </c>
-    </row>
-    <row r="17" ht="270" customHeight="true">
-      <c r="A17" s="17">
-        <v>19</v>
-      </c>
-      <c r="B17" s="18" t="str">
-        <f>data!D22</f>
-      </c>
-    </row>
-    <row r="18" ht="270" customHeight="true">
-      <c r="A18" s="17">
-        <v>20</v>
-      </c>
-      <c r="B18" s="18" t="str">
-        <f>data!D23</f>
-      </c>
-    </row>
-    <row r="19" ht="270" customHeight="true">
-      <c r="A19" s="17">
-        <v>21</v>
-      </c>
-      <c r="B19" s="18" t="str">
-        <f>data!D24</f>
-      </c>
-    </row>
-    <row r="20" ht="270" customHeight="true">
-      <c r="A20" s="17">
-        <v>22</v>
-      </c>
-      <c r="B20" s="18" t="str">
-        <f>data!D25</f>
-      </c>
-    </row>
-    <row r="21" ht="270" customHeight="true">
-      <c r="A21" s="17">
-        <v>23</v>
-      </c>
-      <c r="B21" s="18" t="str">
-        <f>data!D26</f>
-      </c>
-    </row>
-    <row r="22" ht="270" customHeight="true">
-      <c r="A22" s="17">
-        <v>24</v>
-      </c>
-      <c r="B22" s="18" t="str">
-        <f>data!D27</f>
-      </c>
-    </row>
-    <row r="23" ht="270" customHeight="true">
-      <c r="A23" s="17">
-        <v>25</v>
-      </c>
-      <c r="B23" s="18" t="str">
-        <f>data!D28</f>
-      </c>
-    </row>
-    <row r="24" ht="270" customHeight="true">
-      <c r="A24" s="17">
-        <v>26</v>
-      </c>
-      <c r="B24" s="18" t="str">
-        <f>data!D29</f>
-      </c>
-    </row>
-    <row r="25" ht="270" customHeight="true">
-      <c r="A25" s="17">
-        <v>27</v>
-      </c>
-      <c r="B25" s="18" t="str">
-        <f>data!D30</f>
-      </c>
-    </row>
-    <row r="26" ht="270" customHeight="true">
-      <c r="A26" s="17">
-        <v>28</v>
-      </c>
-      <c r="B26" s="18" t="str">
-        <f>data!D31</f>
-      </c>
-    </row>
-    <row r="27" ht="270" customHeight="true">
-      <c r="A27" s="17">
-        <v>29</v>
-      </c>
-      <c r="B27" s="18" t="str">
-        <f>data!D32</f>
-      </c>
-    </row>
-    <row r="28" ht="270" customHeight="true">
-      <c r="A28" s="17">
-        <v>30</v>
-      </c>
-      <c r="B28" s="18" t="str">
-        <f>data!D33</f>
-      </c>
-    </row>
-    <row r="29" ht="270" customHeight="true">
-      <c r="A29" s="17">
-        <v>31</v>
-      </c>
-      <c r="B29" s="18" t="str">
-        <f>data!D34</f>
-      </c>
-    </row>
-    <row r="30" ht="270" customHeight="true">
-      <c r="A30" s="17">
-        <v>32</v>
-      </c>
-      <c r="B30" s="18" t="str">
-        <f>data!D35</f>
-      </c>
-    </row>
-    <row r="31" ht="270" customHeight="true">
-      <c r="A31" s="17">
-        <v>33</v>
-      </c>
-      <c r="B31" s="18" t="str">
-        <f>data!D36</f>
-      </c>
-    </row>
-    <row r="32" ht="270" customHeight="true">
-      <c r="A32" s="17">
-        <v>34</v>
-      </c>
-      <c r="B32" s="18" t="str">
-        <f>data!D37</f>
-      </c>
-    </row>
-    <row r="33" ht="270" customHeight="true">
-      <c r="A33" s="17">
-        <v>3</v>
-      </c>
-      <c r="B33" s="18" t="str">
-        <f>data!D6</f>
-      </c>
-    </row>
-    <row r="34" ht="270" customHeight="true">
-      <c r="A34" s="17">
-        <v>35</v>
-      </c>
-      <c r="B34" s="18" t="str">
-        <f>data!D38</f>
-      </c>
-    </row>
-    <row r="35" ht="270" customHeight="true">
-      <c r="A35" s="17">
-        <v>36</v>
-      </c>
-      <c r="B35" s="18" t="str">
-        <f>data!D39</f>
-      </c>
-    </row>
-    <row r="36" ht="270" customHeight="true">
-      <c r="A36" s="17">
-        <v>37</v>
-      </c>
-      <c r="B36" s="18" t="str">
-        <f>data!D40</f>
-      </c>
-    </row>
-    <row r="37" ht="270" customHeight="true">
-      <c r="A37" s="17">
-        <v>38</v>
-      </c>
-      <c r="B37" s="18" t="str">
-        <f>data!D41</f>
-      </c>
-    </row>
-    <row r="38" ht="270" customHeight="true">
-      <c r="A38" s="17">
-        <v>39</v>
-      </c>
-      <c r="B38" s="18" t="str">
-        <f>data!D42</f>
-      </c>
-    </row>
-    <row r="39" ht="270" customHeight="true">
-      <c r="A39" s="17">
-        <v>40</v>
-      </c>
-      <c r="B39" s="18" t="str">
-        <f>data!D43</f>
-      </c>
-    </row>
-    <row r="40" ht="270" customHeight="true">
-      <c r="A40" s="17">
-        <v>41</v>
-      </c>
-      <c r="B40" s="18" t="str">
-        <f>data!D44</f>
-      </c>
-    </row>
-    <row r="41" ht="270" customHeight="true">
-      <c r="A41" s="17">
-        <v>42</v>
-      </c>
-      <c r="B41" s="18" t="str">
-        <f>data!D45</f>
-      </c>
-    </row>
-    <row r="42" ht="270" customHeight="true">
-      <c r="A42" s="17">
-        <v>43</v>
-      </c>
-      <c r="B42" s="18" t="str">
-        <f>data!D46</f>
-      </c>
-    </row>
-    <row r="43" ht="270" customHeight="true">
-      <c r="A43" s="17">
-        <v>44</v>
-      </c>
-      <c r="B43" s="18" t="str">
-        <f>data!D47</f>
-      </c>
-    </row>
-    <row r="44" ht="270" customHeight="true">
-      <c r="A44" s="17">
-        <v>45</v>
-      </c>
-      <c r="B44" s="18" t="str">
-        <f>data!D48</f>
-      </c>
-    </row>
-    <row r="45" ht="270" customHeight="true">
-      <c r="A45" s="17">
-        <v>46</v>
-      </c>
-      <c r="B45" s="18" t="str">
-        <f>data!D49</f>
-      </c>
-    </row>
-    <row r="46" ht="270" customHeight="true">
-      <c r="A46" s="17">
-        <v>47</v>
-      </c>
-      <c r="B46" s="18" t="str">
-        <f>data!D50</f>
-      </c>
-    </row>
-    <row r="47" ht="270" customHeight="true">
-      <c r="A47" s="17">
-        <v>48</v>
-      </c>
-      <c r="B47" s="18" t="str">
-        <f>data!D51</f>
-      </c>
-    </row>
-    <row r="48" ht="270" customHeight="true">
-      <c r="A48" s="17">
-        <v>49</v>
-      </c>
-      <c r="B48" s="18" t="str">
-        <f>data!D52</f>
-      </c>
-    </row>
-    <row r="49" ht="270" customHeight="true">
-      <c r="A49" s="17">
-        <v>50</v>
-      </c>
-      <c r="B49" s="18" t="str">
-        <f>data!D53</f>
-      </c>
-    </row>
-    <row r="50" ht="270" customHeight="true">
-      <c r="A50" s="17">
-        <v>51</v>
-      </c>
-      <c r="B50" s="18" t="str">
-        <f>data!D54</f>
-      </c>
-    </row>
-    <row r="51" ht="270" customHeight="true">
-      <c r="A51" s="17">
-        <v>52</v>
-      </c>
-      <c r="B51" s="18" t="str">
-        <f>data!D55</f>
-      </c>
-    </row>
-    <row r="52" ht="270" customHeight="true">
-      <c r="A52" s="17">
-        <v>53</v>
-      </c>
-      <c r="B52" s="18" t="str">
-        <f>data!D56</f>
-      </c>
-    </row>
-    <row r="53" ht="270" customHeight="true">
-      <c r="A53" s="17">
-        <v>54</v>
-      </c>
-      <c r="B53" s="18" t="str">
-        <f>data!D57</f>
-      </c>
-    </row>
-    <row r="54" ht="270" customHeight="true">
-      <c r="A54" s="17">
-        <v>55</v>
-      </c>
-      <c r="B54" s="18" t="str">
-        <f>data!D58</f>
-      </c>
-    </row>
-    <row r="55" ht="270" customHeight="true">
-      <c r="A55" s="17">
-        <v>56</v>
-      </c>
-      <c r="B55" s="18" t="str">
-        <f>data!D59</f>
-      </c>
-    </row>
-    <row r="56" ht="270" customHeight="true">
-      <c r="A56" s="17">
-        <v>57</v>
-      </c>
-      <c r="B56" s="18" t="str">
-        <f>data!D60</f>
-      </c>
-    </row>
-    <row r="57" ht="270" customHeight="true">
-      <c r="A57" s="17">
-        <v>58</v>
-      </c>
-      <c r="B57" s="18" t="str">
-        <f>data!D61</f>
-      </c>
-    </row>
-    <row r="58" ht="270" customHeight="true">
-      <c r="A58" s="17">
-        <v>59</v>
-      </c>
-      <c r="B58" s="18" t="str">
-        <f>data!D62</f>
-      </c>
-    </row>
-    <row r="59" ht="270" customHeight="true">
-      <c r="A59" s="17">
-        <v>60</v>
-      </c>
-      <c r="B59" s="18" t="str">
-        <f>data!D63</f>
-      </c>
-    </row>
-    <row r="60" ht="270" customHeight="true">
-      <c r="A60" s="17">
-        <v>61</v>
-      </c>
-      <c r="B60" s="18" t="str">
-        <f>data!D64</f>
-      </c>
-    </row>
-    <row r="61" ht="270" customHeight="true">
-      <c r="A61" s="17">
-        <v>62</v>
-      </c>
-      <c r="B61" s="18" t="str">
-        <f>data!D65</f>
-      </c>
-    </row>
-    <row r="62" ht="270" customHeight="true">
-      <c r="A62" s="17">
-        <v>63</v>
-      </c>
-      <c r="B62" s="18" t="str">
-        <f>data!D66</f>
-      </c>
-    </row>
-    <row r="63" ht="270" customHeight="true">
-      <c r="A63" s="17">
-        <v>64</v>
-      </c>
-      <c r="B63" s="18" t="str">
-        <f>data!D67</f>
-      </c>
-    </row>
-    <row r="64" ht="270" customHeight="true">
-      <c r="A64" s="17">
-        <v>65</v>
-      </c>
-      <c r="B64" s="18" t="str">
-        <f>data!D68</f>
-      </c>
-    </row>
-    <row r="65" ht="270" customHeight="true">
-      <c r="A65" s="17">
-        <v>1</v>
-      </c>
-      <c r="B65" s="18" t="str">
-        <f>data!D4</f>
-      </c>
-    </row>
-    <row r="66" ht="270" customHeight="true">
-      <c r="A66" s="17">
-        <v>66</v>
-      </c>
-      <c r="B66" s="18" t="str">
-        <f>data!D69</f>
-      </c>
-    </row>
-    <row r="67" ht="270" customHeight="true">
-      <c r="A67" s="17">
-        <v>67</v>
-      </c>
-      <c r="B67" s="18" t="str">
-        <f>data!D70</f>
-      </c>
-    </row>
-    <row r="68" ht="270" customHeight="true">
-      <c r="A68" s="17">
-        <v>68</v>
-      </c>
-      <c r="B68" s="18" t="str">
-        <f>data!D71</f>
-      </c>
-    </row>
-    <row r="69" ht="270" customHeight="true">
-      <c r="A69" s="17">
-        <v>69</v>
-      </c>
-      <c r="B69" s="18" t="str">
-        <f>data!D72</f>
-      </c>
-    </row>
-    <row r="70" ht="270" customHeight="true">
-      <c r="A70" s="17">
-        <v>70</v>
-      </c>
-      <c r="B70" s="18" t="str">
-        <f>data!D73</f>
-      </c>
-    </row>
-    <row r="71" ht="270" customHeight="true">
-      <c r="A71" s="17">
-        <v>71</v>
-      </c>
-      <c r="B71" s="18" t="str">
-        <f>data!D74</f>
-      </c>
-    </row>
-    <row r="72" ht="270" customHeight="true">
-      <c r="A72" s="17">
-        <v>72</v>
-      </c>
-      <c r="B72" s="18" t="str">
-        <f>data!D75</f>
-      </c>
-    </row>
-    <row r="73" ht="270" customHeight="true">
-      <c r="A73" s="17">
-        <v>73</v>
-      </c>
-      <c r="B73" s="18" t="str">
-        <f>data!D76</f>
-      </c>
-    </row>
-    <row r="74" ht="270" customHeight="true">
-      <c r="A74" s="17">
-        <v>74</v>
-      </c>
-      <c r="B74" s="18" t="str">
-        <f>data!D77</f>
-      </c>
-    </row>
-    <row r="75" ht="270" customHeight="true">
-      <c r="A75" s="17">
-        <v>75</v>
-      </c>
-      <c r="B75" s="18" t="str">
-        <f>data!D78</f>
-      </c>
-    </row>
-    <row r="76" ht="270" customHeight="true">
-      <c r="A76" s="17">
-        <v>76</v>
-      </c>
-      <c r="B76" s="18" t="str">
-        <f>data!D79</f>
-      </c>
-    </row>
-    <row r="77" ht="270" customHeight="true">
-      <c r="A77" s="17">
-        <v>77</v>
-      </c>
-      <c r="B77" s="18" t="str">
-        <f>data!D80</f>
-      </c>
-    </row>
-    <row r="78" ht="270" customHeight="true">
-      <c r="A78" s="17">
-        <v>78</v>
-      </c>
-      <c r="B78" s="18" t="str">
-        <f>data!D81</f>
-      </c>
-    </row>
-    <row r="79" ht="270" customHeight="true">
-      <c r="A79" s="17">
-        <v>79</v>
-      </c>
-      <c r="B79" s="18" t="str">
-        <f>data!D82</f>
-      </c>
-    </row>
-    <row r="80" ht="270" customHeight="true">
-      <c r="A80" s="17">
-        <v>80</v>
-      </c>
-      <c r="B80" s="18" t="str">
-        <f>data!D83</f>
-      </c>
-    </row>
-    <row r="81" ht="270" customHeight="true">
-      <c r="A81" s="17">
-        <v>81</v>
-      </c>
-      <c r="B81" s="18" t="str">
-        <f>data!D84</f>
-      </c>
-    </row>
-    <row r="82" ht="270" customHeight="true">
-      <c r="A82" s="17">
-        <v>82</v>
-      </c>
-      <c r="B82" s="18" t="str">
-        <f>data!D85</f>
-      </c>
-    </row>
-    <row r="83" ht="270" customHeight="true">
-      <c r="A83" s="17">
-        <v>83</v>
-      </c>
-      <c r="B83" s="18" t="str">
-        <f>data!D86</f>
-      </c>
-    </row>
-    <row r="84" ht="270" customHeight="true">
-      <c r="A84" s="17">
-        <v>84</v>
-      </c>
-      <c r="B84" s="18" t="str">
-        <f>data!D87</f>
-      </c>
-    </row>
-    <row r="85" ht="270" customHeight="true">
-      <c r="A85" s="17">
-        <v>85</v>
-      </c>
-      <c r="B85" s="18" t="str">
-        <f>data!D88</f>
-      </c>
-    </row>
-    <row r="86" ht="270" customHeight="true">
-      <c r="A86" s="17">
-        <v>86</v>
-      </c>
-      <c r="B86" s="18" t="str">
-        <f>data!D89</f>
-      </c>
-    </row>
-    <row r="87" ht="270" customHeight="true">
-      <c r="A87" s="17">
-        <v>87</v>
-      </c>
-      <c r="B87" s="18" t="str">
-        <f>data!D90</f>
-      </c>
-    </row>
-    <row r="88" ht="270" customHeight="true">
-      <c r="A88" s="17">
-        <v>88</v>
-      </c>
-      <c r="B88" s="18" t="str">
-        <f>data!D91</f>
-      </c>
-    </row>
-    <row r="89" ht="270" customHeight="true">
-      <c r="A89" s="17">
-        <v>89</v>
-      </c>
-      <c r="B89" s="18" t="str">
-        <f>data!D92</f>
-      </c>
-    </row>
-    <row r="90" ht="270" customHeight="true">
-      <c r="A90" s="17">
-        <v>90</v>
-      </c>
-      <c r="B90" s="18" t="str">
-        <f>data!D93</f>
-      </c>
-    </row>
-    <row r="91" ht="270" customHeight="true">
-      <c r="A91" s="17">
-        <v>2</v>
-      </c>
-      <c r="B91" s="18" t="str">
-        <f>data!D5</f>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.1" right="0.1" top="0.1" bottom="0.1" header="0.1" footer="0.1"/>
-  <pageSetup orientation="landscape" paperSize="8"/>
-  <rowBreaks count="30" manualBreakCount="30">
-    <brk id="3" max="16383" man="true"/>
-    <brk id="6" max="16383" man="true"/>
-    <brk id="9" max="16383" man="true"/>
-    <brk id="12" max="16383" man="true"/>
-    <brk id="15" max="16383" man="true"/>
-    <brk id="18" max="16383" man="true"/>
-    <brk id="21" max="16383" man="true"/>
-    <brk id="24" max="16383" man="true"/>
-    <brk id="27" max="16383" man="true"/>
-    <brk id="30" max="16383" man="true"/>
-    <brk id="33" max="16383" man="true"/>
-    <brk id="36" max="16383" man="true"/>
-    <brk id="39" max="16383" man="true"/>
-    <brk id="42" max="16383" man="true"/>
-    <brk id="45" max="16383" man="true"/>
-    <brk id="48" max="16383" man="true"/>
-    <brk id="51" max="16383" man="true"/>
-    <brk id="54" max="16383" man="true"/>
-    <brk id="57" max="16383" man="true"/>
-    <brk id="60" max="16383" man="true"/>
-    <brk id="63" max="16383" man="true"/>
-    <brk id="66" max="16383" man="true"/>
-    <brk id="69" max="16383" man="true"/>
-    <brk id="72" max="16383" man="true"/>
-    <brk id="75" max="16383" man="true"/>
-    <brk id="78" max="16383" man="true"/>
-    <brk id="81" max="16383" man="true"/>
-    <brk id="84" max="16383" man="true"/>
-    <brk id="87" max="16383" man="true"/>
-    <brk id="90" max="16383" man="true"/>
-  </rowBreaks>
-  <colBreaks/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>

</xml_diff>

<commit_message>
feat: implement mobile application server with REST API handlers and state management. Also added a more official way to record pool results.
</commit_message>
<xml_diff>
--- a/playoffs-example-large-seeded.xlsx
+++ b/playoffs-example-large-seeded.xlsx
@@ -1048,12 +1048,17 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEFEFEF"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -1129,7 +1134,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center" wrapText="true"/>
@@ -1176,7 +1181,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="true" applyAlignment="false">
       <alignment/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
@@ -1185,16 +1190,27 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="6" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="6" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center"/>
+      <protection hidden="false" locked="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="true" applyAlignment="false" applyProtection="true">
+      <alignment/>
+      <protection hidden="false" locked="false"/>
+    </xf>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="6" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="20" fontId="2" fillId="0" borderId="6" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
@@ -3000,6 +3016,7 @@
       <c r="E35" s="12"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="true" objects="true" scenarios="true" formatCells="true" formatColumns="true" formatRows="true" insertColumns="true" insertRows="true" insertHyperlinks="true" deleteColumns="true" deleteRows="true" selectLockedCells="false" sort="true" autoFilter="true" pivotTables="true" selectUnlockedCells="false"/>
   <mergeCells count="1">
     <mergeCell ref="A1:P1"/>
   </mergeCells>
@@ -3232,6 +3249,7 @@
       <c r="E35" s="12"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="true" objects="true" scenarios="true" formatCells="true" formatColumns="true" formatRows="true" insertColumns="true" insertRows="true" insertHyperlinks="true" deleteColumns="true" deleteRows="true" selectLockedCells="false" sort="true" autoFilter="true" pivotTables="true" selectUnlockedCells="false"/>
   <mergeCells count="1">
     <mergeCell ref="A1:P1"/>
   </mergeCells>
@@ -3455,6 +3473,7 @@
       <c r="E35" s="12"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="true" objects="true" scenarios="true" formatCells="true" formatColumns="true" formatRows="true" insertColumns="true" insertRows="true" insertHyperlinks="true" deleteColumns="true" deleteRows="true" selectLockedCells="false" sort="true" autoFilter="true" pivotTables="true" selectUnlockedCells="false"/>
   <mergeCells count="1">
     <mergeCell ref="A1:P1"/>
   </mergeCells>
@@ -3687,6 +3706,7 @@
       <c r="E35" s="12"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="true" objects="true" scenarios="true" formatCells="true" formatColumns="true" formatRows="true" insertColumns="true" insertRows="true" insertHyperlinks="true" deleteColumns="true" deleteRows="true" selectLockedCells="false" sort="true" autoFilter="true" pivotTables="true" selectUnlockedCells="false"/>
   <mergeCells count="1">
     <mergeCell ref="A1:P1"/>
   </mergeCells>
@@ -3910,6 +3930,7 @@
       <c r="E35" s="12"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="true" objects="true" scenarios="true" formatCells="true" formatColumns="true" formatRows="true" insertColumns="true" insertRows="true" insertHyperlinks="true" deleteColumns="true" deleteRows="true" selectLockedCells="false" sort="true" autoFilter="true" pivotTables="true" selectUnlockedCells="false"/>
   <mergeCells count="1">
     <mergeCell ref="A1:P1"/>
   </mergeCells>
@@ -4142,6 +4163,7 @@
       <c r="E35" s="12"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="true" objects="true" scenarios="true" formatCells="true" formatColumns="true" formatRows="true" insertColumns="true" insertRows="true" insertHyperlinks="true" deleteColumns="true" deleteRows="true" selectLockedCells="false" sort="true" autoFilter="true" pivotTables="true" selectUnlockedCells="false"/>
   <mergeCells count="1">
     <mergeCell ref="A1:P1"/>
   </mergeCells>
@@ -4525,6 +4547,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection sheet="true" objects="true" scenarios="true" formatCells="true" formatColumns="true" formatRows="true" insertColumns="true" insertRows="true" insertHyperlinks="true" deleteColumns="true" deleteRows="true" selectLockedCells="false" sort="true" autoFilter="true" pivotTables="true" selectUnlockedCells="false"/>
   <pageMargins left="0.1" right="0.1" top="0.1" bottom="0.1" header="0.1" footer="0.1"/>
   <pageSetup orientation="landscape" paperSize="8"/>
   <rowBreaks count="15" manualBreakCount="15">
@@ -4917,6 +4940,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection sheet="true" objects="true" scenarios="true" formatCells="true" formatColumns="true" formatRows="true" insertColumns="true" insertRows="true" insertHyperlinks="true" deleteColumns="true" deleteRows="true" selectLockedCells="false" sort="true" autoFilter="true" pivotTables="true" selectUnlockedCells="false"/>
   <pageMargins left="0.1" right="0.1" top="0.1" bottom="0.1" header="0.1" footer="0.1"/>
   <pageSetup orientation="landscape" paperSize="8"/>
   <rowBreaks count="15" manualBreakCount="15">
@@ -5000,7 +5024,7 @@
       <c r="G2" s="3">
         <v>0.020833333333333332</v>
       </c>
-      <c r="H2" s="22" t="str">
+      <c r="H2" s="24" t="str">
         <f>C2*I2+J2</f>
       </c>
     </row>
@@ -5104,7 +5128,7 @@
       <c r="G8" s="3">
         <v>0.020833333333333332</v>
       </c>
-      <c r="H8" s="22" t="str">
+      <c r="H8" s="24" t="str">
         <f>E8+(A8*F8)+G8</f>
       </c>
     </row>
@@ -5150,42 +5174,42 @@
       <c r="A14">
         <v>2</v>
       </c>
-      <c r="E14" s="19" t="s">
+      <c r="E14" s="25" t="s">
         <v>304</v>
       </c>
-      <c r="F14" s="19"/>
-      <c r="G14" s="19"/>
-      <c r="H14" s="22" t="str">
+      <c r="F14" s="25"/>
+      <c r="G14" s="25"/>
+      <c r="H14" s="24" t="str">
         <f>H2</f>
       </c>
     </row>
     <row r="15">
-      <c r="E15" s="19" t="s">
+      <c r="E15" s="25" t="s">
         <v>305</v>
       </c>
-      <c r="F15" s="19"/>
-      <c r="G15" s="19"/>
-      <c r="H15" s="22" t="str">
+      <c r="F15" s="25"/>
+      <c r="G15" s="25"/>
+      <c r="H15" s="24" t="str">
         <f>H8</f>
       </c>
     </row>
     <row r="16">
-      <c r="E16" s="19" t="s">
+      <c r="E16" s="25" t="s">
         <v>306</v>
       </c>
-      <c r="F16" s="19"/>
-      <c r="G16" s="19"/>
-      <c r="H16" s="22" t="str">
+      <c r="F16" s="25"/>
+      <c r="G16" s="25"/>
+      <c r="H16" s="24" t="str">
         <f>H14+H15</f>
       </c>
     </row>
     <row r="17">
-      <c r="E17" s="19" t="s">
+      <c r="E17" s="25" t="s">
         <v>307</v>
       </c>
-      <c r="F17" s="19"/>
-      <c r="G17" s="19"/>
-      <c r="H17" s="22" t="str">
+      <c r="F17" s="25"/>
+      <c r="G17" s="25"/>
+      <c r="H17" s="24" t="str">
         <f>H16/A14</f>
       </c>
     </row>
@@ -5195,7 +5219,7 @@
       </c>
       <c r="F18" s="11"/>
       <c r="G18" s="11"/>
-      <c r="H18" s="23">
+      <c r="H18" s="26">
         <v>0.375</v>
       </c>
     </row>
@@ -5205,7 +5229,7 @@
       </c>
       <c r="F19" s="11"/>
       <c r="G19" s="11"/>
-      <c r="H19" s="23" t="str">
+      <c r="H19" s="26" t="str">
         <f>H18+H17</f>
       </c>
     </row>
@@ -5229,14 +5253,15 @@
     <col customWidth="true" max="4" min="4" width="3"/>
     <col customWidth="true" max="6" min="5" width="5"/>
     <col customWidth="true" max="7" min="7" width="30"/>
-    <col customWidth="true" max="8" min="8" width="2"/>
+    <col customWidth="true" max="8" min="8" width="5"/>
     <col customWidth="true" max="9" min="9" width="30"/>
     <col customWidth="true" max="11" min="10" width="5"/>
     <col customWidth="true" max="12" min="12" width="3"/>
     <col customWidth="true" max="14" min="13" width="5"/>
     <col customWidth="true" max="15" min="15" width="30"/>
-    <col customWidth="true" max="16" min="16" width="2"/>
-    <col customWidth="true" max="20" min="17" width="10.83"/>
+    <col customWidth="true" max="18" min="16" width="5"/>
+    <col customWidth="true" max="19" min="19" width="30"/>
+    <col customWidth="true" max="20" min="20" width="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5303,22 +5328,22 @@
       <c r="A4" s="19" t="str">
         <f>'data'!$B$38</f>
       </c>
-      <c r="B4" s="19"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
       <c r="G4" s="19" t="str">
         <f>'data'!$B$37</f>
       </c>
       <c r="I4" s="19" t="str">
         <f>'data'!$B$54</f>
       </c>
-      <c r="J4" s="19"/>
-      <c r="K4" s="19"/>
-      <c r="L4" s="19"/>
-      <c r="M4" s="19"/>
-      <c r="N4" s="19"/>
+      <c r="J4" s="22"/>
+      <c r="K4" s="22"/>
+      <c r="L4" s="22"/>
+      <c r="M4" s="22"/>
+      <c r="N4" s="22"/>
       <c r="O4" s="19" t="str">
         <f>'data'!$B$53</f>
       </c>
@@ -5327,21 +5352,21 @@
       <c r="F6" t="s">
         <v>212</v>
       </c>
-      <c r="G6" s="15"/>
+      <c r="G6" s="23"/>
       <c r="N6" t="s">
         <v>212</v>
       </c>
-      <c r="O6" s="15"/>
+      <c r="O6" s="23"/>
     </row>
     <row r="7">
       <c r="F7" t="s">
         <v>213</v>
       </c>
-      <c r="G7" s="15"/>
+      <c r="G7" s="23"/>
       <c r="N7" t="s">
         <v>213</v>
       </c>
-      <c r="O7" s="15"/>
+      <c r="O7" s="23"/>
     </row>
     <row r="10">
       <c r="A10" s="11" t="s">
@@ -5387,22 +5412,22 @@
       <c r="A12" s="19" t="str">
         <f>'data'!$B$41</f>
       </c>
-      <c r="B12" s="19"/>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="19"/>
+      <c r="B12" s="22"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="22"/>
       <c r="G12" s="19" t="str">
         <f>'data'!$B$40</f>
       </c>
       <c r="I12" s="19" t="str">
         <f>'data'!$B$57</f>
       </c>
-      <c r="J12" s="19"/>
-      <c r="K12" s="19"/>
-      <c r="L12" s="19"/>
-      <c r="M12" s="19"/>
-      <c r="N12" s="19"/>
+      <c r="J12" s="22"/>
+      <c r="K12" s="22"/>
+      <c r="L12" s="22"/>
+      <c r="M12" s="22"/>
+      <c r="N12" s="22"/>
       <c r="O12" s="19" t="str">
         <f>'data'!$B$56</f>
       </c>
@@ -5411,21 +5436,21 @@
       <c r="F14" t="s">
         <v>212</v>
       </c>
-      <c r="G14" s="15"/>
+      <c r="G14" s="23"/>
       <c r="N14" t="s">
         <v>212</v>
       </c>
-      <c r="O14" s="15"/>
+      <c r="O14" s="23"/>
     </row>
     <row r="15">
       <c r="F15" t="s">
         <v>213</v>
       </c>
-      <c r="G15" s="15"/>
+      <c r="G15" s="23"/>
       <c r="N15" t="s">
         <v>213</v>
       </c>
-      <c r="O15" s="15"/>
+      <c r="O15" s="23"/>
     </row>
     <row r="18">
       <c r="A18" s="11" t="s">
@@ -5471,22 +5496,22 @@
       <c r="A20" s="19" t="str">
         <f>'data'!$B$16</f>
       </c>
-      <c r="B20" s="19"/>
-      <c r="C20" s="19"/>
-      <c r="D20" s="19"/>
-      <c r="E20" s="19"/>
-      <c r="F20" s="19"/>
+      <c r="B20" s="22"/>
+      <c r="C20" s="22"/>
+      <c r="D20" s="22"/>
+      <c r="E20" s="22"/>
+      <c r="F20" s="22"/>
       <c r="G20" s="19" t="str">
         <f>'data'!$B$43</f>
       </c>
       <c r="I20" s="19" t="str">
         <f>'data'!$B$60</f>
       </c>
-      <c r="J20" s="19"/>
-      <c r="K20" s="19"/>
-      <c r="L20" s="19"/>
-      <c r="M20" s="19"/>
-      <c r="N20" s="19"/>
+      <c r="J20" s="22"/>
+      <c r="K20" s="22"/>
+      <c r="L20" s="22"/>
+      <c r="M20" s="22"/>
+      <c r="N20" s="22"/>
       <c r="O20" s="19" t="str">
         <f>'data'!$B$81</f>
       </c>
@@ -5495,21 +5520,21 @@
       <c r="F22" t="s">
         <v>212</v>
       </c>
-      <c r="G22" s="15"/>
+      <c r="G22" s="23"/>
       <c r="N22" t="s">
         <v>212</v>
       </c>
-      <c r="O22" s="15"/>
+      <c r="O22" s="23"/>
     </row>
     <row r="23">
       <c r="F23" t="s">
         <v>213</v>
       </c>
-      <c r="G23" s="15"/>
+      <c r="G23" s="23"/>
       <c r="N23" t="s">
         <v>213</v>
       </c>
-      <c r="O23" s="15"/>
+      <c r="O23" s="23"/>
     </row>
     <row r="26">
       <c r="A26" s="11" t="s">
@@ -5555,22 +5580,22 @@
       <c r="A28" s="19" t="str">
         <f>'data'!$B$21</f>
       </c>
-      <c r="B28" s="19"/>
-      <c r="C28" s="19"/>
-      <c r="D28" s="19"/>
-      <c r="E28" s="19"/>
-      <c r="F28" s="19"/>
+      <c r="B28" s="22"/>
+      <c r="C28" s="22"/>
+      <c r="D28" s="22"/>
+      <c r="E28" s="22"/>
+      <c r="F28" s="22"/>
       <c r="G28" s="19" t="str">
         <f>'data'!$B$20</f>
       </c>
       <c r="I28" s="19" t="str">
         <f>'data'!$B$63</f>
       </c>
-      <c r="J28" s="19"/>
-      <c r="K28" s="19"/>
-      <c r="L28" s="19"/>
-      <c r="M28" s="19"/>
-      <c r="N28" s="19"/>
+      <c r="J28" s="22"/>
+      <c r="K28" s="22"/>
+      <c r="L28" s="22"/>
+      <c r="M28" s="22"/>
+      <c r="N28" s="22"/>
       <c r="O28" s="19" t="str">
         <f>'data'!$B$62</f>
       </c>
@@ -5579,21 +5604,21 @@
       <c r="F30" t="s">
         <v>212</v>
       </c>
-      <c r="G30" s="15"/>
+      <c r="G30" s="23"/>
       <c r="N30" t="s">
         <v>212</v>
       </c>
-      <c r="O30" s="15"/>
+      <c r="O30" s="23"/>
     </row>
     <row r="31">
       <c r="F31" t="s">
         <v>213</v>
       </c>
-      <c r="G31" s="15"/>
+      <c r="G31" s="23"/>
       <c r="N31" t="s">
         <v>213</v>
       </c>
-      <c r="O31" s="15"/>
+      <c r="O31" s="23"/>
     </row>
     <row r="34">
       <c r="A34" s="11" t="s">
@@ -5639,22 +5664,22 @@
       <c r="A36" s="19" t="str">
         <f>'data'!$B$24</f>
       </c>
-      <c r="B36" s="19"/>
-      <c r="C36" s="19"/>
-      <c r="D36" s="19"/>
-      <c r="E36" s="19"/>
-      <c r="F36" s="19"/>
+      <c r="B36" s="22"/>
+      <c r="C36" s="22"/>
+      <c r="D36" s="22"/>
+      <c r="E36" s="22"/>
+      <c r="F36" s="22"/>
       <c r="G36" s="19" t="str">
         <f>'data'!$B$23</f>
       </c>
       <c r="I36" s="19" t="str">
         <f>'data'!$B$66</f>
       </c>
-      <c r="J36" s="19"/>
-      <c r="K36" s="19"/>
-      <c r="L36" s="19"/>
-      <c r="M36" s="19"/>
-      <c r="N36" s="19"/>
+      <c r="J36" s="22"/>
+      <c r="K36" s="22"/>
+      <c r="L36" s="22"/>
+      <c r="M36" s="22"/>
+      <c r="N36" s="22"/>
       <c r="O36" s="19" t="str">
         <f>'data'!$B$65</f>
       </c>
@@ -5663,21 +5688,21 @@
       <c r="F38" t="s">
         <v>212</v>
       </c>
-      <c r="G38" s="15"/>
+      <c r="G38" s="23"/>
       <c r="N38" t="s">
         <v>212</v>
       </c>
-      <c r="O38" s="15"/>
+      <c r="O38" s="23"/>
     </row>
     <row r="39">
       <c r="F39" t="s">
         <v>213</v>
       </c>
-      <c r="G39" s="15"/>
+      <c r="G39" s="23"/>
       <c r="N39" t="s">
         <v>213</v>
       </c>
-      <c r="O39" s="15"/>
+      <c r="O39" s="23"/>
     </row>
     <row r="42">
       <c r="A42" s="11" t="s">
@@ -5723,22 +5748,22 @@
       <c r="A44" s="19" t="str">
         <f>'data'!$B$27</f>
       </c>
-      <c r="B44" s="19"/>
-      <c r="C44" s="19"/>
-      <c r="D44" s="19"/>
-      <c r="E44" s="19"/>
-      <c r="F44" s="19"/>
+      <c r="B44" s="22"/>
+      <c r="C44" s="22"/>
+      <c r="D44" s="22"/>
+      <c r="E44" s="22"/>
+      <c r="F44" s="22"/>
       <c r="G44" s="19" t="str">
         <f>'data'!$B$26</f>
       </c>
       <c r="I44" s="19" t="str">
         <f>'data'!$B$4</f>
       </c>
-      <c r="J44" s="19"/>
-      <c r="K44" s="19"/>
-      <c r="L44" s="19"/>
-      <c r="M44" s="19"/>
-      <c r="N44" s="19"/>
+      <c r="J44" s="22"/>
+      <c r="K44" s="22"/>
+      <c r="L44" s="22"/>
+      <c r="M44" s="22"/>
+      <c r="N44" s="22"/>
       <c r="O44" s="19" t="str">
         <f>'data'!$B$68</f>
       </c>
@@ -5747,21 +5772,21 @@
       <c r="F46" t="s">
         <v>212</v>
       </c>
-      <c r="G46" s="15"/>
+      <c r="G46" s="23"/>
       <c r="N46" t="s">
         <v>212</v>
       </c>
-      <c r="O46" s="15"/>
+      <c r="O46" s="23"/>
     </row>
     <row r="47">
       <c r="F47" t="s">
         <v>213</v>
       </c>
-      <c r="G47" s="15"/>
+      <c r="G47" s="23"/>
       <c r="N47" t="s">
         <v>213</v>
       </c>
-      <c r="O47" s="15"/>
+      <c r="O47" s="23"/>
     </row>
     <row r="50">
       <c r="A50" s="11" t="s">
@@ -5807,22 +5832,22 @@
       <c r="A52" s="19" t="str">
         <f>'data'!$B$32</f>
       </c>
-      <c r="B52" s="19"/>
-      <c r="C52" s="19"/>
-      <c r="D52" s="19"/>
-      <c r="E52" s="19"/>
-      <c r="F52" s="19"/>
+      <c r="B52" s="22"/>
+      <c r="C52" s="22"/>
+      <c r="D52" s="22"/>
+      <c r="E52" s="22"/>
+      <c r="F52" s="22"/>
       <c r="G52" s="19" t="str">
         <f>'data'!$B$31</f>
       </c>
       <c r="I52" s="19" t="str">
         <f>'data'!$B$88</f>
       </c>
-      <c r="J52" s="19"/>
-      <c r="K52" s="19"/>
-      <c r="L52" s="19"/>
-      <c r="M52" s="19"/>
-      <c r="N52" s="19"/>
+      <c r="J52" s="22"/>
+      <c r="K52" s="22"/>
+      <c r="L52" s="22"/>
+      <c r="M52" s="22"/>
+      <c r="N52" s="22"/>
       <c r="O52" s="19" t="str">
         <f>'data'!$B$74</f>
       </c>
@@ -5831,21 +5856,21 @@
       <c r="F54" t="s">
         <v>212</v>
       </c>
-      <c r="G54" s="15"/>
+      <c r="G54" s="23"/>
       <c r="N54" t="s">
         <v>212</v>
       </c>
-      <c r="O54" s="15"/>
+      <c r="O54" s="23"/>
     </row>
     <row r="55">
       <c r="F55" t="s">
         <v>213</v>
       </c>
-      <c r="G55" s="15"/>
+      <c r="G55" s="23"/>
       <c r="N55" t="s">
         <v>213</v>
       </c>
-      <c r="O55" s="15"/>
+      <c r="O55" s="23"/>
     </row>
     <row r="58">
       <c r="A58" s="11" t="s">
@@ -5891,22 +5916,22 @@
       <c r="A60" s="19" t="str">
         <f>'data'!$B$35</f>
       </c>
-      <c r="B60" s="19"/>
-      <c r="C60" s="19"/>
-      <c r="D60" s="19"/>
-      <c r="E60" s="19"/>
-      <c r="F60" s="19"/>
+      <c r="B60" s="22"/>
+      <c r="C60" s="22"/>
+      <c r="D60" s="22"/>
+      <c r="E60" s="22"/>
+      <c r="F60" s="22"/>
       <c r="G60" s="19" t="str">
         <f>'data'!$B$5</f>
       </c>
       <c r="I60" s="19" t="str">
         <f>'data'!$B$76</f>
       </c>
-      <c r="J60" s="19"/>
-      <c r="K60" s="19"/>
-      <c r="L60" s="19"/>
-      <c r="M60" s="19"/>
-      <c r="N60" s="19"/>
+      <c r="J60" s="22"/>
+      <c r="K60" s="22"/>
+      <c r="L60" s="22"/>
+      <c r="M60" s="22"/>
+      <c r="N60" s="22"/>
       <c r="O60" s="19" t="str">
         <f>'data'!$B$75</f>
       </c>
@@ -5915,21 +5940,21 @@
       <c r="F62" t="s">
         <v>212</v>
       </c>
-      <c r="G62" s="15"/>
+      <c r="G62" s="23"/>
       <c r="N62" t="s">
         <v>212</v>
       </c>
-      <c r="O62" s="15"/>
+      <c r="O62" s="23"/>
     </row>
     <row r="63">
       <c r="F63" t="s">
         <v>213</v>
       </c>
-      <c r="G63" s="15"/>
+      <c r="G63" s="23"/>
       <c r="N63" t="s">
         <v>213</v>
       </c>
-      <c r="O63" s="15"/>
+      <c r="O63" s="23"/>
     </row>
     <row r="66">
       <c r="A66" s="11" t="s">
@@ -5975,22 +6000,22 @@
       <c r="A68" s="19" t="str">
         <f>'data'!$B$6</f>
       </c>
-      <c r="B68" s="19"/>
-      <c r="C68" s="19"/>
-      <c r="D68" s="19"/>
-      <c r="E68" s="19"/>
-      <c r="F68" s="19"/>
+      <c r="B68" s="22"/>
+      <c r="C68" s="22"/>
+      <c r="D68" s="22"/>
+      <c r="E68" s="22"/>
+      <c r="F68" s="22"/>
       <c r="G68" s="19" t="str">
         <f>'data'!$B$37</f>
       </c>
       <c r="I68" s="19" t="str">
         <f>'data'!$B$79</f>
       </c>
-      <c r="J68" s="19"/>
-      <c r="K68" s="19"/>
-      <c r="L68" s="19"/>
-      <c r="M68" s="19"/>
-      <c r="N68" s="19"/>
+      <c r="J68" s="22"/>
+      <c r="K68" s="22"/>
+      <c r="L68" s="22"/>
+      <c r="M68" s="22"/>
+      <c r="N68" s="22"/>
       <c r="O68" s="19" t="str">
         <f>'data'!$B$78</f>
       </c>
@@ -5999,21 +6024,21 @@
       <c r="F70" t="s">
         <v>212</v>
       </c>
-      <c r="G70" s="15"/>
+      <c r="G70" s="23"/>
       <c r="N70" t="s">
         <v>212</v>
       </c>
-      <c r="O70" s="15"/>
+      <c r="O70" s="23"/>
     </row>
     <row r="71">
       <c r="F71" t="s">
         <v>213</v>
       </c>
-      <c r="G71" s="15"/>
+      <c r="G71" s="23"/>
       <c r="N71" t="s">
         <v>213</v>
       </c>
-      <c r="O71" s="15"/>
+      <c r="O71" s="23"/>
     </row>
     <row r="74">
       <c r="A74" s="11" t="s">
@@ -6059,22 +6084,22 @@
       <c r="A76" s="19" t="str">
         <f>'data'!$B$40</f>
       </c>
-      <c r="B76" s="19"/>
-      <c r="C76" s="19"/>
-      <c r="D76" s="19"/>
-      <c r="E76" s="19"/>
-      <c r="F76" s="19"/>
+      <c r="B76" s="22"/>
+      <c r="C76" s="22"/>
+      <c r="D76" s="22"/>
+      <c r="E76" s="22"/>
+      <c r="F76" s="22"/>
       <c r="G76" s="19" t="str">
         <f>'data'!$B$39</f>
       </c>
       <c r="I76" s="19" t="str">
         <f>'data'!$B$82</f>
       </c>
-      <c r="J76" s="19"/>
-      <c r="K76" s="19"/>
-      <c r="L76" s="19"/>
-      <c r="M76" s="19"/>
-      <c r="N76" s="19"/>
+      <c r="J76" s="22"/>
+      <c r="K76" s="22"/>
+      <c r="L76" s="22"/>
+      <c r="M76" s="22"/>
+      <c r="N76" s="22"/>
       <c r="O76" s="19" t="str">
         <f>'data'!$B$81</f>
       </c>
@@ -6083,21 +6108,21 @@
       <c r="F78" t="s">
         <v>212</v>
       </c>
-      <c r="G78" s="15"/>
+      <c r="G78" s="23"/>
       <c r="N78" t="s">
         <v>212</v>
       </c>
-      <c r="O78" s="15"/>
+      <c r="O78" s="23"/>
     </row>
     <row r="79">
       <c r="F79" t="s">
         <v>213</v>
       </c>
-      <c r="G79" s="15"/>
+      <c r="G79" s="23"/>
       <c r="N79" t="s">
         <v>213</v>
       </c>
-      <c r="O79" s="15"/>
+      <c r="O79" s="23"/>
     </row>
     <row r="82">
       <c r="A82" s="11" t="s">
@@ -6143,22 +6168,22 @@
       <c r="A84" s="19" t="str">
         <f>'data'!$B$43</f>
       </c>
-      <c r="B84" s="19"/>
-      <c r="C84" s="19"/>
-      <c r="D84" s="19"/>
-      <c r="E84" s="19"/>
-      <c r="F84" s="19"/>
+      <c r="B84" s="22"/>
+      <c r="C84" s="22"/>
+      <c r="D84" s="22"/>
+      <c r="E84" s="22"/>
+      <c r="F84" s="22"/>
       <c r="G84" s="19" t="str">
         <f>'data'!$B$42</f>
       </c>
       <c r="I84" s="19" t="str">
         <f>'data'!$B$85</f>
       </c>
-      <c r="J84" s="19"/>
-      <c r="K84" s="19"/>
-      <c r="L84" s="19"/>
-      <c r="M84" s="19"/>
-      <c r="N84" s="19"/>
+      <c r="J84" s="22"/>
+      <c r="K84" s="22"/>
+      <c r="L84" s="22"/>
+      <c r="M84" s="22"/>
+      <c r="N84" s="22"/>
       <c r="O84" s="19" t="str">
         <f>'data'!$B$84</f>
       </c>
@@ -6167,21 +6192,21 @@
       <c r="F86" t="s">
         <v>212</v>
       </c>
-      <c r="G86" s="15"/>
+      <c r="G86" s="23"/>
       <c r="N86" t="s">
         <v>212</v>
       </c>
-      <c r="O86" s="15"/>
+      <c r="O86" s="23"/>
     </row>
     <row r="87">
       <c r="F87" t="s">
         <v>213</v>
       </c>
-      <c r="G87" s="15"/>
+      <c r="G87" s="23"/>
       <c r="N87" t="s">
         <v>213</v>
       </c>
-      <c r="O87" s="15"/>
+      <c r="O87" s="23"/>
     </row>
     <row r="90">
       <c r="A90" s="11" t="s">
@@ -6227,22 +6252,22 @@
       <c r="A92" s="19" t="str">
         <f>'data'!$B$46</f>
       </c>
-      <c r="B92" s="19"/>
-      <c r="C92" s="19"/>
-      <c r="D92" s="19"/>
-      <c r="E92" s="19"/>
-      <c r="F92" s="19"/>
+      <c r="B92" s="22"/>
+      <c r="C92" s="22"/>
+      <c r="D92" s="22"/>
+      <c r="E92" s="22"/>
+      <c r="F92" s="22"/>
       <c r="G92" s="19" t="str">
         <f>'data'!$B$45</f>
       </c>
       <c r="I92" s="19" t="str">
         <f>'data'!$B$88</f>
       </c>
-      <c r="J92" s="19"/>
-      <c r="K92" s="19"/>
-      <c r="L92" s="19"/>
-      <c r="M92" s="19"/>
-      <c r="N92" s="19"/>
+      <c r="J92" s="22"/>
+      <c r="K92" s="22"/>
+      <c r="L92" s="22"/>
+      <c r="M92" s="22"/>
+      <c r="N92" s="22"/>
       <c r="O92" s="19" t="str">
         <f>'data'!$B$87</f>
       </c>
@@ -6251,21 +6276,21 @@
       <c r="F94" t="s">
         <v>212</v>
       </c>
-      <c r="G94" s="15"/>
+      <c r="G94" s="23"/>
       <c r="N94" t="s">
         <v>212</v>
       </c>
-      <c r="O94" s="15"/>
+      <c r="O94" s="23"/>
     </row>
     <row r="95">
       <c r="F95" t="s">
         <v>213</v>
       </c>
-      <c r="G95" s="15"/>
+      <c r="G95" s="23"/>
       <c r="N95" t="s">
         <v>213</v>
       </c>
-      <c r="O95" s="15"/>
+      <c r="O95" s="23"/>
     </row>
     <row r="98">
       <c r="A98" s="11" t="s">
@@ -6311,22 +6336,22 @@
       <c r="A100" s="19" t="str">
         <f>'data'!$B$49</f>
       </c>
-      <c r="B100" s="19"/>
-      <c r="C100" s="19"/>
-      <c r="D100" s="19"/>
-      <c r="E100" s="19"/>
-      <c r="F100" s="19"/>
+      <c r="B100" s="22"/>
+      <c r="C100" s="22"/>
+      <c r="D100" s="22"/>
+      <c r="E100" s="22"/>
+      <c r="F100" s="22"/>
       <c r="G100" s="19" t="str">
         <f>'data'!$B$48</f>
       </c>
       <c r="I100" s="19" t="str">
         <f>'data'!$B$91</f>
       </c>
-      <c r="J100" s="19"/>
-      <c r="K100" s="19"/>
-      <c r="L100" s="19"/>
-      <c r="M100" s="19"/>
-      <c r="N100" s="19"/>
+      <c r="J100" s="22"/>
+      <c r="K100" s="22"/>
+      <c r="L100" s="22"/>
+      <c r="M100" s="22"/>
+      <c r="N100" s="22"/>
       <c r="O100" s="19" t="str">
         <f>'data'!$B$90</f>
       </c>
@@ -6335,21 +6360,21 @@
       <c r="F102" t="s">
         <v>212</v>
       </c>
-      <c r="G102" s="15"/>
+      <c r="G102" s="23"/>
       <c r="N102" t="s">
         <v>212</v>
       </c>
-      <c r="O102" s="15"/>
+      <c r="O102" s="23"/>
     </row>
     <row r="103">
       <c r="F103" t="s">
         <v>213</v>
       </c>
-      <c r="G103" s="15"/>
+      <c r="G103" s="23"/>
       <c r="N103" t="s">
         <v>213</v>
       </c>
-      <c r="O103" s="15"/>
+      <c r="O103" s="23"/>
     </row>
     <row r="106">
       <c r="I106" s="11" t="s">
@@ -6377,11 +6402,11 @@
       <c r="I108" s="19" t="str">
         <f>'data'!$B$5</f>
       </c>
-      <c r="J108" s="19"/>
-      <c r="K108" s="19"/>
-      <c r="L108" s="19"/>
-      <c r="M108" s="19"/>
-      <c r="N108" s="19"/>
+      <c r="J108" s="22"/>
+      <c r="K108" s="22"/>
+      <c r="L108" s="22"/>
+      <c r="M108" s="22"/>
+      <c r="N108" s="22"/>
       <c r="O108" s="19" t="str">
         <f>'data'!$B$93</f>
       </c>
@@ -6390,13 +6415,13 @@
       <c r="N110" t="s">
         <v>212</v>
       </c>
-      <c r="O110" s="15"/>
+      <c r="O110" s="23"/>
     </row>
     <row r="111">
       <c r="N111" t="s">
         <v>213</v>
       </c>
-      <c r="O111" s="15"/>
+      <c r="O111" s="23"/>
     </row>
     <row r="119">
       <c r="A119" s="11" t="s">
@@ -6442,22 +6467,22 @@
       <c r="A121" s="19" t="str">
         <f>'data'!$B$35</f>
       </c>
-      <c r="B121" s="19"/>
-      <c r="C121" s="19"/>
-      <c r="D121" s="19"/>
-      <c r="E121" s="19"/>
-      <c r="F121" s="19"/>
+      <c r="B121" s="22"/>
+      <c r="C121" s="22"/>
+      <c r="D121" s="22"/>
+      <c r="E121" s="22"/>
+      <c r="F121" s="22"/>
       <c r="G121" s="19" t="str">
         <f>'data'!$B$32</f>
       </c>
       <c r="I121" s="19" t="str">
         <f>'data'!$B$51</f>
       </c>
-      <c r="J121" s="19"/>
-      <c r="K121" s="19"/>
-      <c r="L121" s="19"/>
-      <c r="M121" s="19"/>
-      <c r="N121" s="19"/>
+      <c r="J121" s="22"/>
+      <c r="K121" s="22"/>
+      <c r="L121" s="22"/>
+      <c r="M121" s="22"/>
+      <c r="N121" s="22"/>
       <c r="O121" s="19" t="str">
         <f>'data'!$B$50</f>
       </c>
@@ -6466,21 +6491,21 @@
       <c r="F123" t="s">
         <v>212</v>
       </c>
-      <c r="G123" s="15"/>
+      <c r="G123" s="23"/>
       <c r="N123" t="s">
         <v>212</v>
       </c>
-      <c r="O123" s="15"/>
+      <c r="O123" s="23"/>
     </row>
     <row r="124">
       <c r="F124" t="s">
         <v>213</v>
       </c>
-      <c r="G124" s="15"/>
+      <c r="G124" s="23"/>
       <c r="N124" t="s">
         <v>213</v>
       </c>
-      <c r="O124" s="15"/>
+      <c r="O124" s="23"/>
     </row>
     <row r="127">
       <c r="A127" s="11" t="s">
@@ -6526,22 +6551,22 @@
       <c r="A129" s="19" t="str">
         <f>CONCATENATE("M 1 ",G6)</f>
       </c>
-      <c r="B129" s="19"/>
-      <c r="C129" s="19"/>
-      <c r="D129" s="19"/>
-      <c r="E129" s="19"/>
-      <c r="F129" s="19"/>
+      <c r="B129" s="22"/>
+      <c r="C129" s="22"/>
+      <c r="D129" s="22"/>
+      <c r="E129" s="22"/>
+      <c r="F129" s="22"/>
       <c r="G129" s="19" t="str">
         <f>'data'!$B$36</f>
       </c>
       <c r="I129" s="19" t="str">
         <f>CONCATENATE("M 14 ",O6)</f>
       </c>
-      <c r="J129" s="19"/>
-      <c r="K129" s="19"/>
-      <c r="L129" s="19"/>
-      <c r="M129" s="19"/>
-      <c r="N129" s="19"/>
+      <c r="J129" s="22"/>
+      <c r="K129" s="22"/>
+      <c r="L129" s="22"/>
+      <c r="M129" s="22"/>
+      <c r="N129" s="22"/>
       <c r="O129" s="19" t="str">
         <f>'data'!$B$52</f>
       </c>
@@ -6550,21 +6575,21 @@
       <c r="F131" t="s">
         <v>212</v>
       </c>
-      <c r="G131" s="15"/>
+      <c r="G131" s="23"/>
       <c r="N131" t="s">
         <v>212</v>
       </c>
-      <c r="O131" s="15"/>
+      <c r="O131" s="23"/>
     </row>
     <row r="132">
       <c r="F132" t="s">
         <v>213</v>
       </c>
-      <c r="G132" s="15"/>
+      <c r="G132" s="23"/>
       <c r="N132" t="s">
         <v>213</v>
       </c>
-      <c r="O132" s="15"/>
+      <c r="O132" s="23"/>
     </row>
     <row r="135">
       <c r="A135" s="11" t="s">
@@ -6610,22 +6635,22 @@
       <c r="A137" s="19" t="str">
         <f>CONCATENATE("M 2 ",G14)</f>
       </c>
-      <c r="B137" s="19"/>
-      <c r="C137" s="19"/>
-      <c r="D137" s="19"/>
-      <c r="E137" s="19"/>
-      <c r="F137" s="19"/>
+      <c r="B137" s="22"/>
+      <c r="C137" s="22"/>
+      <c r="D137" s="22"/>
+      <c r="E137" s="22"/>
+      <c r="F137" s="22"/>
       <c r="G137" s="19" t="str">
         <f>'data'!$B$39</f>
       </c>
       <c r="I137" s="19" t="str">
         <f>CONCATENATE("M 15 ",O14)</f>
       </c>
-      <c r="J137" s="19"/>
-      <c r="K137" s="19"/>
-      <c r="L137" s="19"/>
-      <c r="M137" s="19"/>
-      <c r="N137" s="19"/>
+      <c r="J137" s="22"/>
+      <c r="K137" s="22"/>
+      <c r="L137" s="22"/>
+      <c r="M137" s="22"/>
+      <c r="N137" s="22"/>
       <c r="O137" s="19" t="str">
         <f>'data'!$B$55</f>
       </c>
@@ -6634,21 +6659,21 @@
       <c r="F139" t="s">
         <v>212</v>
       </c>
-      <c r="G139" s="15"/>
+      <c r="G139" s="23"/>
       <c r="N139" t="s">
         <v>212</v>
       </c>
-      <c r="O139" s="15"/>
+      <c r="O139" s="23"/>
     </row>
     <row r="140">
       <c r="F140" t="s">
         <v>213</v>
       </c>
-      <c r="G140" s="15"/>
+      <c r="G140" s="23"/>
       <c r="N140" t="s">
         <v>213</v>
       </c>
-      <c r="O140" s="15"/>
+      <c r="O140" s="23"/>
     </row>
     <row r="143">
       <c r="A143" s="11" t="s">
@@ -6694,22 +6719,22 @@
       <c r="A145" s="19" t="str">
         <f>CONCATENATE("M 3 ",G22)</f>
       </c>
-      <c r="B145" s="19"/>
-      <c r="C145" s="19"/>
-      <c r="D145" s="19"/>
-      <c r="E145" s="19"/>
-      <c r="F145" s="19"/>
+      <c r="B145" s="22"/>
+      <c r="C145" s="22"/>
+      <c r="D145" s="22"/>
+      <c r="E145" s="22"/>
+      <c r="F145" s="22"/>
       <c r="G145" s="19" t="str">
         <f>'data'!$B$42</f>
       </c>
       <c r="I145" s="19" t="str">
         <f>CONCATENATE("M 16 ",O22)</f>
       </c>
-      <c r="J145" s="19"/>
-      <c r="K145" s="19"/>
-      <c r="L145" s="19"/>
-      <c r="M145" s="19"/>
-      <c r="N145" s="19"/>
+      <c r="J145" s="22"/>
+      <c r="K145" s="22"/>
+      <c r="L145" s="22"/>
+      <c r="M145" s="22"/>
+      <c r="N145" s="22"/>
       <c r="O145" s="19" t="str">
         <f>'data'!$B$58</f>
       </c>
@@ -6718,21 +6743,21 @@
       <c r="F147" t="s">
         <v>212</v>
       </c>
-      <c r="G147" s="15"/>
+      <c r="G147" s="23"/>
       <c r="N147" t="s">
         <v>212</v>
       </c>
-      <c r="O147" s="15"/>
+      <c r="O147" s="23"/>
     </row>
     <row r="148">
       <c r="F148" t="s">
         <v>213</v>
       </c>
-      <c r="G148" s="15"/>
+      <c r="G148" s="23"/>
       <c r="N148" t="s">
         <v>213</v>
       </c>
-      <c r="O148" s="15"/>
+      <c r="O148" s="23"/>
     </row>
     <row r="151">
       <c r="A151" s="11" t="s">
@@ -6778,22 +6803,22 @@
       <c r="A153" s="19" t="str">
         <f>'data'!$B$18</f>
       </c>
-      <c r="B153" s="19"/>
-      <c r="C153" s="19"/>
-      <c r="D153" s="19"/>
-      <c r="E153" s="19"/>
-      <c r="F153" s="19"/>
+      <c r="B153" s="22"/>
+      <c r="C153" s="22"/>
+      <c r="D153" s="22"/>
+      <c r="E153" s="22"/>
+      <c r="F153" s="22"/>
       <c r="G153" s="19" t="str">
         <f>'data'!$B$17</f>
       </c>
       <c r="I153" s="19" t="str">
         <f>CONCATENATE("M 17 ",O30)</f>
       </c>
-      <c r="J153" s="19"/>
-      <c r="K153" s="19"/>
-      <c r="L153" s="19"/>
-      <c r="M153" s="19"/>
-      <c r="N153" s="19"/>
+      <c r="J153" s="22"/>
+      <c r="K153" s="22"/>
+      <c r="L153" s="22"/>
+      <c r="M153" s="22"/>
+      <c r="N153" s="22"/>
       <c r="O153" s="19" t="str">
         <f>'data'!$B$61</f>
       </c>
@@ -6802,21 +6827,21 @@
       <c r="F155" t="s">
         <v>212</v>
       </c>
-      <c r="G155" s="15"/>
+      <c r="G155" s="23"/>
       <c r="N155" t="s">
         <v>212</v>
       </c>
-      <c r="O155" s="15"/>
+      <c r="O155" s="23"/>
     </row>
     <row r="156">
       <c r="F156" t="s">
         <v>213</v>
       </c>
-      <c r="G156" s="15"/>
+      <c r="G156" s="23"/>
       <c r="N156" t="s">
         <v>213</v>
       </c>
-      <c r="O156" s="15"/>
+      <c r="O156" s="23"/>
     </row>
     <row r="159">
       <c r="A159" s="11" t="s">
@@ -6862,22 +6887,22 @@
       <c r="A161" s="19" t="str">
         <f>CONCATENATE("M 4 ",G30)</f>
       </c>
-      <c r="B161" s="19"/>
-      <c r="C161" s="19"/>
-      <c r="D161" s="19"/>
-      <c r="E161" s="19"/>
-      <c r="F161" s="19"/>
+      <c r="B161" s="22"/>
+      <c r="C161" s="22"/>
+      <c r="D161" s="22"/>
+      <c r="E161" s="22"/>
+      <c r="F161" s="22"/>
       <c r="G161" s="19" t="str">
         <f>'data'!$B$30</f>
       </c>
       <c r="I161" s="19" t="str">
         <f>CONCATENATE("M 18 ",O38)</f>
       </c>
-      <c r="J161" s="19"/>
-      <c r="K161" s="19"/>
-      <c r="L161" s="19"/>
-      <c r="M161" s="19"/>
-      <c r="N161" s="19"/>
+      <c r="J161" s="22"/>
+      <c r="K161" s="22"/>
+      <c r="L161" s="22"/>
+      <c r="M161" s="22"/>
+      <c r="N161" s="22"/>
       <c r="O161" s="19" t="str">
         <f>'data'!$B$64</f>
       </c>
@@ -6886,21 +6911,21 @@
       <c r="F163" t="s">
         <v>212</v>
       </c>
-      <c r="G163" s="15"/>
+      <c r="G163" s="23"/>
       <c r="N163" t="s">
         <v>212</v>
       </c>
-      <c r="O163" s="15"/>
+      <c r="O163" s="23"/>
     </row>
     <row r="164">
       <c r="F164" t="s">
         <v>213</v>
       </c>
-      <c r="G164" s="15"/>
+      <c r="G164" s="23"/>
       <c r="N164" t="s">
         <v>213</v>
       </c>
-      <c r="O164" s="15"/>
+      <c r="O164" s="23"/>
     </row>
     <row r="167">
       <c r="A167" s="11" t="s">
@@ -6946,22 +6971,22 @@
       <c r="A169" s="19" t="str">
         <f>CONCATENATE("M 5 ",G38)</f>
       </c>
-      <c r="B169" s="19"/>
-      <c r="C169" s="19"/>
-      <c r="D169" s="19"/>
-      <c r="E169" s="19"/>
-      <c r="F169" s="19"/>
+      <c r="B169" s="22"/>
+      <c r="C169" s="22"/>
+      <c r="D169" s="22"/>
+      <c r="E169" s="22"/>
+      <c r="F169" s="22"/>
       <c r="G169" s="19" t="str">
         <f>'data'!$B$22</f>
       </c>
       <c r="I169" s="19" t="str">
         <f>CONCATENATE("M 19 ",O46)</f>
       </c>
-      <c r="J169" s="19"/>
-      <c r="K169" s="19"/>
-      <c r="L169" s="19"/>
-      <c r="M169" s="19"/>
-      <c r="N169" s="19"/>
+      <c r="J169" s="22"/>
+      <c r="K169" s="22"/>
+      <c r="L169" s="22"/>
+      <c r="M169" s="22"/>
+      <c r="N169" s="22"/>
       <c r="O169" s="19" t="str">
         <f>'data'!$B$67</f>
       </c>
@@ -6970,21 +6995,21 @@
       <c r="F171" t="s">
         <v>212</v>
       </c>
-      <c r="G171" s="15"/>
+      <c r="G171" s="23"/>
       <c r="N171" t="s">
         <v>212</v>
       </c>
-      <c r="O171" s="15"/>
+      <c r="O171" s="23"/>
     </row>
     <row r="172">
       <c r="F172" t="s">
         <v>213</v>
       </c>
-      <c r="G172" s="15"/>
+      <c r="G172" s="23"/>
       <c r="N172" t="s">
         <v>213</v>
       </c>
-      <c r="O172" s="15"/>
+      <c r="O172" s="23"/>
     </row>
     <row r="175">
       <c r="A175" s="11" t="s">
@@ -7030,22 +7055,22 @@
       <c r="A177" s="19" t="str">
         <f>CONCATENATE("M 6 ",G46)</f>
       </c>
-      <c r="B177" s="19"/>
-      <c r="C177" s="19"/>
-      <c r="D177" s="19"/>
-      <c r="E177" s="19"/>
-      <c r="F177" s="19"/>
+      <c r="B177" s="22"/>
+      <c r="C177" s="22"/>
+      <c r="D177" s="22"/>
+      <c r="E177" s="22"/>
+      <c r="F177" s="22"/>
       <c r="G177" s="19" t="str">
         <f>'data'!$B$25</f>
       </c>
       <c r="I177" s="19" t="str">
         <f>CONCATENATE("M 20 ",O54)</f>
       </c>
-      <c r="J177" s="19"/>
-      <c r="K177" s="19"/>
-      <c r="L177" s="19"/>
-      <c r="M177" s="19"/>
-      <c r="N177" s="19"/>
+      <c r="J177" s="22"/>
+      <c r="K177" s="22"/>
+      <c r="L177" s="22"/>
+      <c r="M177" s="22"/>
+      <c r="N177" s="22"/>
       <c r="O177" s="19" t="str">
         <f>'data'!$B$69</f>
       </c>
@@ -7054,21 +7079,21 @@
       <c r="F179" t="s">
         <v>212</v>
       </c>
-      <c r="G179" s="15"/>
+      <c r="G179" s="23"/>
       <c r="N179" t="s">
         <v>212</v>
       </c>
-      <c r="O179" s="15"/>
+      <c r="O179" s="23"/>
     </row>
     <row r="180">
       <c r="F180" t="s">
         <v>213</v>
       </c>
-      <c r="G180" s="15"/>
+      <c r="G180" s="23"/>
       <c r="N180" t="s">
         <v>213</v>
       </c>
-      <c r="O180" s="15"/>
+      <c r="O180" s="23"/>
     </row>
     <row r="183">
       <c r="A183" s="11" t="s">
@@ -7114,22 +7139,22 @@
       <c r="A185" s="19" t="str">
         <f>'data'!$B$29</f>
       </c>
-      <c r="B185" s="19"/>
-      <c r="C185" s="19"/>
-      <c r="D185" s="19"/>
-      <c r="E185" s="19"/>
-      <c r="F185" s="19"/>
+      <c r="B185" s="22"/>
+      <c r="C185" s="22"/>
+      <c r="D185" s="22"/>
+      <c r="E185" s="22"/>
+      <c r="F185" s="22"/>
       <c r="G185" s="19" t="str">
         <f>'data'!$B$28</f>
       </c>
       <c r="I185" s="19" t="str">
         <f>'data'!$B$73</f>
       </c>
-      <c r="J185" s="19"/>
-      <c r="K185" s="19"/>
-      <c r="L185" s="19"/>
-      <c r="M185" s="19"/>
-      <c r="N185" s="19"/>
+      <c r="J185" s="22"/>
+      <c r="K185" s="22"/>
+      <c r="L185" s="22"/>
+      <c r="M185" s="22"/>
+      <c r="N185" s="22"/>
       <c r="O185" s="19" t="str">
         <f>'data'!$B$72</f>
       </c>
@@ -7138,21 +7163,21 @@
       <c r="F187" t="s">
         <v>212</v>
       </c>
-      <c r="G187" s="15"/>
+      <c r="G187" s="23"/>
       <c r="N187" t="s">
         <v>212</v>
       </c>
-      <c r="O187" s="15"/>
+      <c r="O187" s="23"/>
     </row>
     <row r="188">
       <c r="F188" t="s">
         <v>213</v>
       </c>
-      <c r="G188" s="15"/>
+      <c r="G188" s="23"/>
       <c r="N188" t="s">
         <v>213</v>
       </c>
-      <c r="O188" s="15"/>
+      <c r="O188" s="23"/>
     </row>
     <row r="191">
       <c r="A191" s="11" t="s">
@@ -7198,22 +7223,22 @@
       <c r="A193" s="19" t="str">
         <f>CONCATENATE("M 7 ",G54)</f>
       </c>
-      <c r="B193" s="19"/>
-      <c r="C193" s="19"/>
-      <c r="D193" s="19"/>
-      <c r="E193" s="19"/>
-      <c r="F193" s="19"/>
+      <c r="B193" s="22"/>
+      <c r="C193" s="22"/>
+      <c r="D193" s="22"/>
+      <c r="E193" s="22"/>
+      <c r="F193" s="22"/>
       <c r="G193" s="19" t="str">
         <f>'data'!$B$30</f>
       </c>
       <c r="I193" s="19" t="str">
         <f>CONCATENATE("M 21 ",O62)</f>
       </c>
-      <c r="J193" s="19"/>
-      <c r="K193" s="19"/>
-      <c r="L193" s="19"/>
-      <c r="M193" s="19"/>
-      <c r="N193" s="19"/>
+      <c r="J193" s="22"/>
+      <c r="K193" s="22"/>
+      <c r="L193" s="22"/>
+      <c r="M193" s="22"/>
+      <c r="N193" s="22"/>
       <c r="O193" s="19" t="str">
         <f>'data'!$B$74</f>
       </c>
@@ -7222,21 +7247,21 @@
       <c r="F195" t="s">
         <v>212</v>
       </c>
-      <c r="G195" s="15"/>
+      <c r="G195" s="23"/>
       <c r="N195" t="s">
         <v>212</v>
       </c>
-      <c r="O195" s="15"/>
+      <c r="O195" s="23"/>
     </row>
     <row r="196">
       <c r="F196" t="s">
         <v>213</v>
       </c>
-      <c r="G196" s="15"/>
+      <c r="G196" s="23"/>
       <c r="N196" t="s">
         <v>213</v>
       </c>
-      <c r="O196" s="15"/>
+      <c r="O196" s="23"/>
     </row>
     <row r="199">
       <c r="A199" s="11" t="s">
@@ -7282,22 +7307,22 @@
       <c r="A201" s="19" t="str">
         <f>CONCATENATE("M 8 ",G62)</f>
       </c>
-      <c r="B201" s="19"/>
-      <c r="C201" s="19"/>
-      <c r="D201" s="19"/>
-      <c r="E201" s="19"/>
-      <c r="F201" s="19"/>
+      <c r="B201" s="22"/>
+      <c r="C201" s="22"/>
+      <c r="D201" s="22"/>
+      <c r="E201" s="22"/>
+      <c r="F201" s="22"/>
       <c r="G201" s="19" t="str">
         <f>'data'!$B$4</f>
       </c>
       <c r="I201" s="19" t="str">
         <f>CONCATENATE("M 22 ",O70)</f>
       </c>
-      <c r="J201" s="19"/>
-      <c r="K201" s="19"/>
-      <c r="L201" s="19"/>
-      <c r="M201" s="19"/>
-      <c r="N201" s="19"/>
+      <c r="J201" s="22"/>
+      <c r="K201" s="22"/>
+      <c r="L201" s="22"/>
+      <c r="M201" s="22"/>
+      <c r="N201" s="22"/>
       <c r="O201" s="19" t="str">
         <f>'data'!$B$77</f>
       </c>
@@ -7306,21 +7331,21 @@
       <c r="F203" t="s">
         <v>212</v>
       </c>
-      <c r="G203" s="15"/>
+      <c r="G203" s="23"/>
       <c r="N203" t="s">
         <v>212</v>
       </c>
-      <c r="O203" s="15"/>
+      <c r="O203" s="23"/>
     </row>
     <row r="204">
       <c r="F204" t="s">
         <v>213</v>
       </c>
-      <c r="G204" s="15"/>
+      <c r="G204" s="23"/>
       <c r="N204" t="s">
         <v>213</v>
       </c>
-      <c r="O204" s="15"/>
+      <c r="O204" s="23"/>
     </row>
     <row r="207">
       <c r="A207" s="11" t="s">
@@ -7366,22 +7391,22 @@
       <c r="A209" s="19" t="str">
         <f>CONCATENATE("M 9 ",G70)</f>
       </c>
-      <c r="B209" s="19"/>
-      <c r="C209" s="19"/>
-      <c r="D209" s="19"/>
-      <c r="E209" s="19"/>
-      <c r="F209" s="19"/>
+      <c r="B209" s="22"/>
+      <c r="C209" s="22"/>
+      <c r="D209" s="22"/>
+      <c r="E209" s="22"/>
+      <c r="F209" s="22"/>
       <c r="G209" s="19" t="str">
         <f>'data'!$B$36</f>
       </c>
       <c r="I209" s="19" t="str">
         <f>CONCATENATE("M 23 ",O78)</f>
       </c>
-      <c r="J209" s="19"/>
-      <c r="K209" s="19"/>
-      <c r="L209" s="19"/>
-      <c r="M209" s="19"/>
-      <c r="N209" s="19"/>
+      <c r="J209" s="22"/>
+      <c r="K209" s="22"/>
+      <c r="L209" s="22"/>
+      <c r="M209" s="22"/>
+      <c r="N209" s="22"/>
       <c r="O209" s="19" t="str">
         <f>'data'!$B$80</f>
       </c>
@@ -7390,21 +7415,21 @@
       <c r="F211" t="s">
         <v>212</v>
       </c>
-      <c r="G211" s="15"/>
+      <c r="G211" s="23"/>
       <c r="N211" t="s">
         <v>212</v>
       </c>
-      <c r="O211" s="15"/>
+      <c r="O211" s="23"/>
     </row>
     <row r="212">
       <c r="F212" t="s">
         <v>213</v>
       </c>
-      <c r="G212" s="15"/>
+      <c r="G212" s="23"/>
       <c r="N212" t="s">
         <v>213</v>
       </c>
-      <c r="O212" s="15"/>
+      <c r="O212" s="23"/>
     </row>
     <row r="215">
       <c r="A215" s="11" t="s">
@@ -7450,22 +7475,22 @@
       <c r="A217" s="19" t="str">
         <f>CONCATENATE("M 10 ",G78)</f>
       </c>
-      <c r="B217" s="19"/>
-      <c r="C217" s="19"/>
-      <c r="D217" s="19"/>
-      <c r="E217" s="19"/>
-      <c r="F217" s="19"/>
+      <c r="B217" s="22"/>
+      <c r="C217" s="22"/>
+      <c r="D217" s="22"/>
+      <c r="E217" s="22"/>
+      <c r="F217" s="22"/>
       <c r="G217" s="19" t="str">
         <f>'data'!$B$38</f>
       </c>
       <c r="I217" s="19" t="str">
         <f>CONCATENATE("M 24 ",O86)</f>
       </c>
-      <c r="J217" s="19"/>
-      <c r="K217" s="19"/>
-      <c r="L217" s="19"/>
-      <c r="M217" s="19"/>
-      <c r="N217" s="19"/>
+      <c r="J217" s="22"/>
+      <c r="K217" s="22"/>
+      <c r="L217" s="22"/>
+      <c r="M217" s="22"/>
+      <c r="N217" s="22"/>
       <c r="O217" s="19" t="str">
         <f>'data'!$B$83</f>
       </c>
@@ -7474,21 +7499,21 @@
       <c r="F219" t="s">
         <v>212</v>
       </c>
-      <c r="G219" s="15"/>
+      <c r="G219" s="23"/>
       <c r="N219" t="s">
         <v>212</v>
       </c>
-      <c r="O219" s="15"/>
+      <c r="O219" s="23"/>
     </row>
     <row r="220">
       <c r="F220" t="s">
         <v>213</v>
       </c>
-      <c r="G220" s="15"/>
+      <c r="G220" s="23"/>
       <c r="N220" t="s">
         <v>213</v>
       </c>
-      <c r="O220" s="15"/>
+      <c r="O220" s="23"/>
     </row>
     <row r="223">
       <c r="A223" s="11" t="s">
@@ -7534,22 +7559,22 @@
       <c r="A225" s="19" t="str">
         <f>CONCATENATE("M 11 ",G86)</f>
       </c>
-      <c r="B225" s="19"/>
-      <c r="C225" s="19"/>
-      <c r="D225" s="19"/>
-      <c r="E225" s="19"/>
-      <c r="F225" s="19"/>
+      <c r="B225" s="22"/>
+      <c r="C225" s="22"/>
+      <c r="D225" s="22"/>
+      <c r="E225" s="22"/>
+      <c r="F225" s="22"/>
       <c r="G225" s="19" t="str">
         <f>'data'!$B$41</f>
       </c>
       <c r="I225" s="19" t="str">
         <f>CONCATENATE("M 25 ",O94)</f>
       </c>
-      <c r="J225" s="19"/>
-      <c r="K225" s="19"/>
-      <c r="L225" s="19"/>
-      <c r="M225" s="19"/>
-      <c r="N225" s="19"/>
+      <c r="J225" s="22"/>
+      <c r="K225" s="22"/>
+      <c r="L225" s="22"/>
+      <c r="M225" s="22"/>
+      <c r="N225" s="22"/>
       <c r="O225" s="19" t="str">
         <f>'data'!$B$86</f>
       </c>
@@ -7558,21 +7583,21 @@
       <c r="F227" t="s">
         <v>212</v>
       </c>
-      <c r="G227" s="15"/>
+      <c r="G227" s="23"/>
       <c r="N227" t="s">
         <v>212</v>
       </c>
-      <c r="O227" s="15"/>
+      <c r="O227" s="23"/>
     </row>
     <row r="228">
       <c r="F228" t="s">
         <v>213</v>
       </c>
-      <c r="G228" s="15"/>
+      <c r="G228" s="23"/>
       <c r="N228" t="s">
         <v>213</v>
       </c>
-      <c r="O228" s="15"/>
+      <c r="O228" s="23"/>
     </row>
     <row r="231">
       <c r="A231" s="11" t="s">
@@ -7618,22 +7643,22 @@
       <c r="A233" s="19" t="str">
         <f>CONCATENATE("M 12 ",G94)</f>
       </c>
-      <c r="B233" s="19"/>
-      <c r="C233" s="19"/>
-      <c r="D233" s="19"/>
-      <c r="E233" s="19"/>
-      <c r="F233" s="19"/>
+      <c r="B233" s="22"/>
+      <c r="C233" s="22"/>
+      <c r="D233" s="22"/>
+      <c r="E233" s="22"/>
+      <c r="F233" s="22"/>
       <c r="G233" s="19" t="str">
         <f>'data'!$B$44</f>
       </c>
       <c r="I233" s="19" t="str">
         <f>CONCATENATE("M 26 ",O102)</f>
       </c>
-      <c r="J233" s="19"/>
-      <c r="K233" s="19"/>
-      <c r="L233" s="19"/>
-      <c r="M233" s="19"/>
-      <c r="N233" s="19"/>
+      <c r="J233" s="22"/>
+      <c r="K233" s="22"/>
+      <c r="L233" s="22"/>
+      <c r="M233" s="22"/>
+      <c r="N233" s="22"/>
       <c r="O233" s="19" t="str">
         <f>'data'!$B$89</f>
       </c>
@@ -7642,21 +7667,21 @@
       <c r="F235" t="s">
         <v>212</v>
       </c>
-      <c r="G235" s="15"/>
+      <c r="G235" s="23"/>
       <c r="N235" t="s">
         <v>212</v>
       </c>
-      <c r="O235" s="15"/>
+      <c r="O235" s="23"/>
     </row>
     <row r="236">
       <c r="F236" t="s">
         <v>213</v>
       </c>
-      <c r="G236" s="15"/>
+      <c r="G236" s="23"/>
       <c r="N236" t="s">
         <v>213</v>
       </c>
-      <c r="O236" s="15"/>
+      <c r="O236" s="23"/>
     </row>
     <row r="239">
       <c r="A239" s="11" t="s">
@@ -7702,22 +7727,22 @@
       <c r="A241" s="19" t="str">
         <f>CONCATENATE("M 13 ",G102)</f>
       </c>
-      <c r="B241" s="19"/>
-      <c r="C241" s="19"/>
-      <c r="D241" s="19"/>
-      <c r="E241" s="19"/>
-      <c r="F241" s="19"/>
+      <c r="B241" s="22"/>
+      <c r="C241" s="22"/>
+      <c r="D241" s="22"/>
+      <c r="E241" s="22"/>
+      <c r="F241" s="22"/>
       <c r="G241" s="19" t="str">
         <f>'data'!$B$47</f>
       </c>
       <c r="I241" s="19" t="str">
         <f>CONCATENATE("M 27 ",O110)</f>
       </c>
-      <c r="J241" s="19"/>
-      <c r="K241" s="19"/>
-      <c r="L241" s="19"/>
-      <c r="M241" s="19"/>
-      <c r="N241" s="19"/>
+      <c r="J241" s="22"/>
+      <c r="K241" s="22"/>
+      <c r="L241" s="22"/>
+      <c r="M241" s="22"/>
+      <c r="N241" s="22"/>
       <c r="O241" s="19" t="str">
         <f>'data'!$B$92</f>
       </c>
@@ -7726,21 +7751,21 @@
       <c r="F243" t="s">
         <v>212</v>
       </c>
-      <c r="G243" s="15"/>
+      <c r="G243" s="23"/>
       <c r="N243" t="s">
         <v>212</v>
       </c>
-      <c r="O243" s="15"/>
+      <c r="O243" s="23"/>
     </row>
     <row r="244">
       <c r="F244" t="s">
         <v>213</v>
       </c>
-      <c r="G244" s="15"/>
+      <c r="G244" s="23"/>
       <c r="N244" t="s">
         <v>213</v>
       </c>
-      <c r="O244" s="15"/>
+      <c r="O244" s="23"/>
     </row>
     <row r="252">
       <c r="A252" s="11" t="s">
@@ -7786,22 +7811,22 @@
       <c r="A254" s="19" t="str">
         <f>CONCATENATE("M 29 ",G131)</f>
       </c>
-      <c r="B254" s="19"/>
-      <c r="C254" s="19"/>
-      <c r="D254" s="19"/>
-      <c r="E254" s="19"/>
-      <c r="F254" s="19"/>
+      <c r="B254" s="22"/>
+      <c r="C254" s="22"/>
+      <c r="D254" s="22"/>
+      <c r="E254" s="22"/>
+      <c r="F254" s="22"/>
       <c r="G254" s="19" t="str">
         <f>CONCATENATE("M 28 ",G123)</f>
       </c>
       <c r="I254" s="19" t="str">
         <f>CONCATENATE("M 45 ",O131)</f>
       </c>
-      <c r="J254" s="19"/>
-      <c r="K254" s="19"/>
-      <c r="L254" s="19"/>
-      <c r="M254" s="19"/>
-      <c r="N254" s="19"/>
+      <c r="J254" s="22"/>
+      <c r="K254" s="22"/>
+      <c r="L254" s="22"/>
+      <c r="M254" s="22"/>
+      <c r="N254" s="22"/>
       <c r="O254" s="19" t="str">
         <f>CONCATENATE("M 44 ",O123)</f>
       </c>
@@ -7810,21 +7835,21 @@
       <c r="F256" t="s">
         <v>212</v>
       </c>
-      <c r="G256" s="15"/>
+      <c r="G256" s="23"/>
       <c r="N256" t="s">
         <v>212</v>
       </c>
-      <c r="O256" s="15"/>
+      <c r="O256" s="23"/>
     </row>
     <row r="257">
       <c r="F257" t="s">
         <v>213</v>
       </c>
-      <c r="G257" s="15"/>
+      <c r="G257" s="23"/>
       <c r="N257" t="s">
         <v>213</v>
       </c>
-      <c r="O257" s="15"/>
+      <c r="O257" s="23"/>
     </row>
     <row r="260">
       <c r="A260" s="11" t="s">
@@ -7870,22 +7895,22 @@
       <c r="A262" s="19" t="str">
         <f>CONCATENATE("M 31 ",G147)</f>
       </c>
-      <c r="B262" s="19"/>
-      <c r="C262" s="19"/>
-      <c r="D262" s="19"/>
-      <c r="E262" s="19"/>
-      <c r="F262" s="19"/>
+      <c r="B262" s="22"/>
+      <c r="C262" s="22"/>
+      <c r="D262" s="22"/>
+      <c r="E262" s="22"/>
+      <c r="F262" s="22"/>
       <c r="G262" s="19" t="str">
         <f>CONCATENATE("M 30 ",G139)</f>
       </c>
       <c r="I262" s="19" t="str">
         <f>CONCATENATE("M 47 ",O147)</f>
       </c>
-      <c r="J262" s="19"/>
-      <c r="K262" s="19"/>
-      <c r="L262" s="19"/>
-      <c r="M262" s="19"/>
-      <c r="N262" s="19"/>
+      <c r="J262" s="22"/>
+      <c r="K262" s="22"/>
+      <c r="L262" s="22"/>
+      <c r="M262" s="22"/>
+      <c r="N262" s="22"/>
       <c r="O262" s="19" t="str">
         <f>CONCATENATE("M 46 ",O139)</f>
       </c>
@@ -7894,21 +7919,21 @@
       <c r="F264" t="s">
         <v>212</v>
       </c>
-      <c r="G264" s="15"/>
+      <c r="G264" s="23"/>
       <c r="N264" t="s">
         <v>212</v>
       </c>
-      <c r="O264" s="15"/>
+      <c r="O264" s="23"/>
     </row>
     <row r="265">
       <c r="F265" t="s">
         <v>213</v>
       </c>
-      <c r="G265" s="15"/>
+      <c r="G265" s="23"/>
       <c r="N265" t="s">
         <v>213</v>
       </c>
-      <c r="O265" s="15"/>
+      <c r="O265" s="23"/>
     </row>
     <row r="268">
       <c r="A268" s="11" t="s">
@@ -7954,22 +7979,22 @@
       <c r="A270" s="19" t="str">
         <f>CONCATENATE("M 33 ",G163)</f>
       </c>
-      <c r="B270" s="19"/>
-      <c r="C270" s="19"/>
-      <c r="D270" s="19"/>
-      <c r="E270" s="19"/>
-      <c r="F270" s="19"/>
+      <c r="B270" s="22"/>
+      <c r="C270" s="22"/>
+      <c r="D270" s="22"/>
+      <c r="E270" s="22"/>
+      <c r="F270" s="22"/>
       <c r="G270" s="19" t="str">
         <f>CONCATENATE("M 32 ",G155)</f>
       </c>
       <c r="I270" s="19" t="str">
         <f>CONCATENATE("M 49 ",O163)</f>
       </c>
-      <c r="J270" s="19"/>
-      <c r="K270" s="19"/>
-      <c r="L270" s="19"/>
-      <c r="M270" s="19"/>
-      <c r="N270" s="19"/>
+      <c r="J270" s="22"/>
+      <c r="K270" s="22"/>
+      <c r="L270" s="22"/>
+      <c r="M270" s="22"/>
+      <c r="N270" s="22"/>
       <c r="O270" s="19" t="str">
         <f>CONCATENATE("M 48 ",O155)</f>
       </c>
@@ -7978,21 +8003,21 @@
       <c r="F272" t="s">
         <v>212</v>
       </c>
-      <c r="G272" s="15"/>
+      <c r="G272" s="23"/>
       <c r="N272" t="s">
         <v>212</v>
       </c>
-      <c r="O272" s="15"/>
+      <c r="O272" s="23"/>
     </row>
     <row r="273">
       <c r="F273" t="s">
         <v>213</v>
       </c>
-      <c r="G273" s="15"/>
+      <c r="G273" s="23"/>
       <c r="N273" t="s">
         <v>213</v>
       </c>
-      <c r="O273" s="15"/>
+      <c r="O273" s="23"/>
     </row>
     <row r="276">
       <c r="A276" s="11" t="s">
@@ -8038,22 +8063,22 @@
       <c r="A278" s="19" t="str">
         <f>CONCATENATE("M 35 ",G179)</f>
       </c>
-      <c r="B278" s="19"/>
-      <c r="C278" s="19"/>
-      <c r="D278" s="19"/>
-      <c r="E278" s="19"/>
-      <c r="F278" s="19"/>
+      <c r="B278" s="22"/>
+      <c r="C278" s="22"/>
+      <c r="D278" s="22"/>
+      <c r="E278" s="22"/>
+      <c r="F278" s="22"/>
       <c r="G278" s="19" t="str">
         <f>CONCATENATE("M 34 ",G171)</f>
       </c>
       <c r="I278" s="19" t="str">
         <f>CONCATENATE("M 51 ",O179)</f>
       </c>
-      <c r="J278" s="19"/>
-      <c r="K278" s="19"/>
-      <c r="L278" s="19"/>
-      <c r="M278" s="19"/>
-      <c r="N278" s="19"/>
+      <c r="J278" s="22"/>
+      <c r="K278" s="22"/>
+      <c r="L278" s="22"/>
+      <c r="M278" s="22"/>
+      <c r="N278" s="22"/>
       <c r="O278" s="19" t="str">
         <f>CONCATENATE("M 50 ",O171)</f>
       </c>
@@ -8062,21 +8087,21 @@
       <c r="F280" t="s">
         <v>212</v>
       </c>
-      <c r="G280" s="15"/>
+      <c r="G280" s="23"/>
       <c r="N280" t="s">
         <v>212</v>
       </c>
-      <c r="O280" s="15"/>
+      <c r="O280" s="23"/>
     </row>
     <row r="281">
       <c r="F281" t="s">
         <v>213</v>
       </c>
-      <c r="G281" s="15"/>
+      <c r="G281" s="23"/>
       <c r="N281" t="s">
         <v>213</v>
       </c>
-      <c r="O281" s="15"/>
+      <c r="O281" s="23"/>
     </row>
     <row r="284">
       <c r="A284" s="11" t="s">
@@ -8122,22 +8147,22 @@
       <c r="A286" s="19" t="str">
         <f>CONCATENATE("M 37 ",G195)</f>
       </c>
-      <c r="B286" s="19"/>
-      <c r="C286" s="19"/>
-      <c r="D286" s="19"/>
-      <c r="E286" s="19"/>
-      <c r="F286" s="19"/>
+      <c r="B286" s="22"/>
+      <c r="C286" s="22"/>
+      <c r="D286" s="22"/>
+      <c r="E286" s="22"/>
+      <c r="F286" s="22"/>
       <c r="G286" s="19" t="str">
         <f>CONCATENATE("M 36 ",G187)</f>
       </c>
       <c r="I286" s="19" t="str">
         <f>CONCATENATE("M 53 ",O195)</f>
       </c>
-      <c r="J286" s="19"/>
-      <c r="K286" s="19"/>
-      <c r="L286" s="19"/>
-      <c r="M286" s="19"/>
-      <c r="N286" s="19"/>
+      <c r="J286" s="22"/>
+      <c r="K286" s="22"/>
+      <c r="L286" s="22"/>
+      <c r="M286" s="22"/>
+      <c r="N286" s="22"/>
       <c r="O286" s="19" t="str">
         <f>CONCATENATE("M 52 ",O187)</f>
       </c>
@@ -8146,21 +8171,21 @@
       <c r="F288" t="s">
         <v>212</v>
       </c>
-      <c r="G288" s="15"/>
+      <c r="G288" s="23"/>
       <c r="N288" t="s">
         <v>212</v>
       </c>
-      <c r="O288" s="15"/>
+      <c r="O288" s="23"/>
     </row>
     <row r="289">
       <c r="F289" t="s">
         <v>213</v>
       </c>
-      <c r="G289" s="15"/>
+      <c r="G289" s="23"/>
       <c r="N289" t="s">
         <v>213</v>
       </c>
-      <c r="O289" s="15"/>
+      <c r="O289" s="23"/>
     </row>
     <row r="292">
       <c r="A292" s="11" t="s">
@@ -8206,22 +8231,22 @@
       <c r="A294" s="19" t="str">
         <f>CONCATENATE("M 39 ",G211)</f>
       </c>
-      <c r="B294" s="19"/>
-      <c r="C294" s="19"/>
-      <c r="D294" s="19"/>
-      <c r="E294" s="19"/>
-      <c r="F294" s="19"/>
+      <c r="B294" s="22"/>
+      <c r="C294" s="22"/>
+      <c r="D294" s="22"/>
+      <c r="E294" s="22"/>
+      <c r="F294" s="22"/>
       <c r="G294" s="19" t="str">
         <f>CONCATENATE("M 38 ",G203)</f>
       </c>
       <c r="I294" s="19" t="str">
         <f>CONCATENATE("M 55 ",O211)</f>
       </c>
-      <c r="J294" s="19"/>
-      <c r="K294" s="19"/>
-      <c r="L294" s="19"/>
-      <c r="M294" s="19"/>
-      <c r="N294" s="19"/>
+      <c r="J294" s="22"/>
+      <c r="K294" s="22"/>
+      <c r="L294" s="22"/>
+      <c r="M294" s="22"/>
+      <c r="N294" s="22"/>
       <c r="O294" s="19" t="str">
         <f>CONCATENATE("M 54 ",O203)</f>
       </c>
@@ -8230,21 +8255,21 @@
       <c r="F296" t="s">
         <v>212</v>
       </c>
-      <c r="G296" s="15"/>
+      <c r="G296" s="23"/>
       <c r="N296" t="s">
         <v>212</v>
       </c>
-      <c r="O296" s="15"/>
+      <c r="O296" s="23"/>
     </row>
     <row r="297">
       <c r="F297" t="s">
         <v>213</v>
       </c>
-      <c r="G297" s="15"/>
+      <c r="G297" s="23"/>
       <c r="N297" t="s">
         <v>213</v>
       </c>
-      <c r="O297" s="15"/>
+      <c r="O297" s="23"/>
     </row>
     <row r="300">
       <c r="A300" s="11" t="s">
@@ -8290,22 +8315,22 @@
       <c r="A302" s="19" t="str">
         <f>CONCATENATE("M 41 ",G227)</f>
       </c>
-      <c r="B302" s="19"/>
-      <c r="C302" s="19"/>
-      <c r="D302" s="19"/>
-      <c r="E302" s="19"/>
-      <c r="F302" s="19"/>
+      <c r="B302" s="22"/>
+      <c r="C302" s="22"/>
+      <c r="D302" s="22"/>
+      <c r="E302" s="22"/>
+      <c r="F302" s="22"/>
       <c r="G302" s="19" t="str">
         <f>CONCATENATE("M 40 ",G219)</f>
       </c>
       <c r="I302" s="19" t="str">
         <f>CONCATENATE("M 57 ",O227)</f>
       </c>
-      <c r="J302" s="19"/>
-      <c r="K302" s="19"/>
-      <c r="L302" s="19"/>
-      <c r="M302" s="19"/>
-      <c r="N302" s="19"/>
+      <c r="J302" s="22"/>
+      <c r="K302" s="22"/>
+      <c r="L302" s="22"/>
+      <c r="M302" s="22"/>
+      <c r="N302" s="22"/>
       <c r="O302" s="19" t="str">
         <f>CONCATENATE("M 56 ",O219)</f>
       </c>
@@ -8314,21 +8339,21 @@
       <c r="F304" t="s">
         <v>212</v>
       </c>
-      <c r="G304" s="15"/>
+      <c r="G304" s="23"/>
       <c r="N304" t="s">
         <v>212</v>
       </c>
-      <c r="O304" s="15"/>
+      <c r="O304" s="23"/>
     </row>
     <row r="305">
       <c r="F305" t="s">
         <v>213</v>
       </c>
-      <c r="G305" s="15"/>
+      <c r="G305" s="23"/>
       <c r="N305" t="s">
         <v>213</v>
       </c>
-      <c r="O305" s="15"/>
+      <c r="O305" s="23"/>
     </row>
     <row r="308">
       <c r="A308" s="11" t="s">
@@ -8374,22 +8399,22 @@
       <c r="A310" s="19" t="str">
         <f>CONCATENATE("M 43 ",G243)</f>
       </c>
-      <c r="B310" s="19"/>
-      <c r="C310" s="19"/>
-      <c r="D310" s="19"/>
-      <c r="E310" s="19"/>
-      <c r="F310" s="19"/>
+      <c r="B310" s="22"/>
+      <c r="C310" s="22"/>
+      <c r="D310" s="22"/>
+      <c r="E310" s="22"/>
+      <c r="F310" s="22"/>
       <c r="G310" s="19" t="str">
         <f>CONCATENATE("M 42 ",G235)</f>
       </c>
       <c r="I310" s="19" t="str">
         <f>CONCATENATE("M 59 ",O243)</f>
       </c>
-      <c r="J310" s="19"/>
-      <c r="K310" s="19"/>
-      <c r="L310" s="19"/>
-      <c r="M310" s="19"/>
-      <c r="N310" s="19"/>
+      <c r="J310" s="22"/>
+      <c r="K310" s="22"/>
+      <c r="L310" s="22"/>
+      <c r="M310" s="22"/>
+      <c r="N310" s="22"/>
       <c r="O310" s="19" t="str">
         <f>CONCATENATE("M 58 ",O235)</f>
       </c>
@@ -8398,21 +8423,21 @@
       <c r="F312" t="s">
         <v>212</v>
       </c>
-      <c r="G312" s="15"/>
+      <c r="G312" s="23"/>
       <c r="N312" t="s">
         <v>212</v>
       </c>
-      <c r="O312" s="15"/>
+      <c r="O312" s="23"/>
     </row>
     <row r="313">
       <c r="F313" t="s">
         <v>213</v>
       </c>
-      <c r="G313" s="15"/>
+      <c r="G313" s="23"/>
       <c r="N313" t="s">
         <v>213</v>
       </c>
-      <c r="O313" s="15"/>
+      <c r="O313" s="23"/>
     </row>
     <row r="321">
       <c r="A321" s="11" t="s">
@@ -8458,22 +8483,22 @@
       <c r="A323" s="19" t="str">
         <f>CONCATENATE("M 61 ",G264)</f>
       </c>
-      <c r="B323" s="19"/>
-      <c r="C323" s="19"/>
-      <c r="D323" s="19"/>
-      <c r="E323" s="19"/>
-      <c r="F323" s="19"/>
+      <c r="B323" s="22"/>
+      <c r="C323" s="22"/>
+      <c r="D323" s="22"/>
+      <c r="E323" s="22"/>
+      <c r="F323" s="22"/>
       <c r="G323" s="19" t="str">
         <f>CONCATENATE("M 60 ",G256)</f>
       </c>
       <c r="I323" s="19" t="str">
         <f>CONCATENATE("M 69 ",O264)</f>
       </c>
-      <c r="J323" s="19"/>
-      <c r="K323" s="19"/>
-      <c r="L323" s="19"/>
-      <c r="M323" s="19"/>
-      <c r="N323" s="19"/>
+      <c r="J323" s="22"/>
+      <c r="K323" s="22"/>
+      <c r="L323" s="22"/>
+      <c r="M323" s="22"/>
+      <c r="N323" s="22"/>
       <c r="O323" s="19" t="str">
         <f>CONCATENATE("M 68 ",O256)</f>
       </c>
@@ -8482,21 +8507,21 @@
       <c r="F325" t="s">
         <v>212</v>
       </c>
-      <c r="G325" s="15"/>
+      <c r="G325" s="23"/>
       <c r="N325" t="s">
         <v>212</v>
       </c>
-      <c r="O325" s="15"/>
+      <c r="O325" s="23"/>
     </row>
     <row r="326">
       <c r="F326" t="s">
         <v>213</v>
       </c>
-      <c r="G326" s="15"/>
+      <c r="G326" s="23"/>
       <c r="N326" t="s">
         <v>213</v>
       </c>
-      <c r="O326" s="15"/>
+      <c r="O326" s="23"/>
     </row>
     <row r="329">
       <c r="A329" s="11" t="s">
@@ -8542,22 +8567,22 @@
       <c r="A331" s="19" t="str">
         <f>CONCATENATE("M 63 ",G280)</f>
       </c>
-      <c r="B331" s="19"/>
-      <c r="C331" s="19"/>
-      <c r="D331" s="19"/>
-      <c r="E331" s="19"/>
-      <c r="F331" s="19"/>
+      <c r="B331" s="22"/>
+      <c r="C331" s="22"/>
+      <c r="D331" s="22"/>
+      <c r="E331" s="22"/>
+      <c r="F331" s="22"/>
       <c r="G331" s="19" t="str">
         <f>CONCATENATE("M 62 ",G272)</f>
       </c>
       <c r="I331" s="19" t="str">
         <f>CONCATENATE("M 71 ",O280)</f>
       </c>
-      <c r="J331" s="19"/>
-      <c r="K331" s="19"/>
-      <c r="L331" s="19"/>
-      <c r="M331" s="19"/>
-      <c r="N331" s="19"/>
+      <c r="J331" s="22"/>
+      <c r="K331" s="22"/>
+      <c r="L331" s="22"/>
+      <c r="M331" s="22"/>
+      <c r="N331" s="22"/>
       <c r="O331" s="19" t="str">
         <f>CONCATENATE("M 70 ",O272)</f>
       </c>
@@ -8566,21 +8591,21 @@
       <c r="F333" t="s">
         <v>212</v>
       </c>
-      <c r="G333" s="15"/>
+      <c r="G333" s="23"/>
       <c r="N333" t="s">
         <v>212</v>
       </c>
-      <c r="O333" s="15"/>
+      <c r="O333" s="23"/>
     </row>
     <row r="334">
       <c r="F334" t="s">
         <v>213</v>
       </c>
-      <c r="G334" s="15"/>
+      <c r="G334" s="23"/>
       <c r="N334" t="s">
         <v>213</v>
       </c>
-      <c r="O334" s="15"/>
+      <c r="O334" s="23"/>
     </row>
     <row r="337">
       <c r="A337" s="11" t="s">
@@ -8626,22 +8651,22 @@
       <c r="A339" s="19" t="str">
         <f>CONCATENATE("M 65 ",G296)</f>
       </c>
-      <c r="B339" s="19"/>
-      <c r="C339" s="19"/>
-      <c r="D339" s="19"/>
-      <c r="E339" s="19"/>
-      <c r="F339" s="19"/>
+      <c r="B339" s="22"/>
+      <c r="C339" s="22"/>
+      <c r="D339" s="22"/>
+      <c r="E339" s="22"/>
+      <c r="F339" s="22"/>
       <c r="G339" s="19" t="str">
         <f>CONCATENATE("M 64 ",G288)</f>
       </c>
       <c r="I339" s="19" t="str">
         <f>CONCATENATE("M 73 ",O296)</f>
       </c>
-      <c r="J339" s="19"/>
-      <c r="K339" s="19"/>
-      <c r="L339" s="19"/>
-      <c r="M339" s="19"/>
-      <c r="N339" s="19"/>
+      <c r="J339" s="22"/>
+      <c r="K339" s="22"/>
+      <c r="L339" s="22"/>
+      <c r="M339" s="22"/>
+      <c r="N339" s="22"/>
       <c r="O339" s="19" t="str">
         <f>CONCATENATE("M 72 ",O288)</f>
       </c>
@@ -8650,21 +8675,21 @@
       <c r="F341" t="s">
         <v>212</v>
       </c>
-      <c r="G341" s="15"/>
+      <c r="G341" s="23"/>
       <c r="N341" t="s">
         <v>212</v>
       </c>
-      <c r="O341" s="15"/>
+      <c r="O341" s="23"/>
     </row>
     <row r="342">
       <c r="F342" t="s">
         <v>213</v>
       </c>
-      <c r="G342" s="15"/>
+      <c r="G342" s="23"/>
       <c r="N342" t="s">
         <v>213</v>
       </c>
-      <c r="O342" s="15"/>
+      <c r="O342" s="23"/>
     </row>
     <row r="345">
       <c r="A345" s="11" t="s">
@@ -8710,22 +8735,22 @@
       <c r="A347" s="19" t="str">
         <f>CONCATENATE("M 67 ",G312)</f>
       </c>
-      <c r="B347" s="19"/>
-      <c r="C347" s="19"/>
-      <c r="D347" s="19"/>
-      <c r="E347" s="19"/>
-      <c r="F347" s="19"/>
+      <c r="B347" s="22"/>
+      <c r="C347" s="22"/>
+      <c r="D347" s="22"/>
+      <c r="E347" s="22"/>
+      <c r="F347" s="22"/>
       <c r="G347" s="19" t="str">
         <f>CONCATENATE("M 66 ",G304)</f>
       </c>
       <c r="I347" s="19" t="str">
         <f>CONCATENATE("M 75 ",O312)</f>
       </c>
-      <c r="J347" s="19"/>
-      <c r="K347" s="19"/>
-      <c r="L347" s="19"/>
-      <c r="M347" s="19"/>
-      <c r="N347" s="19"/>
+      <c r="J347" s="22"/>
+      <c r="K347" s="22"/>
+      <c r="L347" s="22"/>
+      <c r="M347" s="22"/>
+      <c r="N347" s="22"/>
       <c r="O347" s="19" t="str">
         <f>CONCATENATE("M 74 ",O304)</f>
       </c>
@@ -8734,21 +8759,21 @@
       <c r="F349" t="s">
         <v>212</v>
       </c>
-      <c r="G349" s="15"/>
+      <c r="G349" s="23"/>
       <c r="N349" t="s">
         <v>212</v>
       </c>
-      <c r="O349" s="15"/>
+      <c r="O349" s="23"/>
     </row>
     <row r="350">
       <c r="F350" t="s">
         <v>213</v>
       </c>
-      <c r="G350" s="15"/>
+      <c r="G350" s="23"/>
       <c r="N350" t="s">
         <v>213</v>
       </c>
-      <c r="O350" s="15"/>
+      <c r="O350" s="23"/>
     </row>
     <row r="358">
       <c r="A358" s="11" t="s">
@@ -8794,22 +8819,22 @@
       <c r="A360" s="19" t="str">
         <f>CONCATENATE("M 77 ",G333)</f>
       </c>
-      <c r="B360" s="19"/>
-      <c r="C360" s="19"/>
-      <c r="D360" s="19"/>
-      <c r="E360" s="19"/>
-      <c r="F360" s="19"/>
+      <c r="B360" s="22"/>
+      <c r="C360" s="22"/>
+      <c r="D360" s="22"/>
+      <c r="E360" s="22"/>
+      <c r="F360" s="22"/>
       <c r="G360" s="19" t="str">
         <f>CONCATENATE("M 76 ",G325)</f>
       </c>
       <c r="I360" s="19" t="str">
         <f>CONCATENATE("M 81 ",O333)</f>
       </c>
-      <c r="J360" s="19"/>
-      <c r="K360" s="19"/>
-      <c r="L360" s="19"/>
-      <c r="M360" s="19"/>
-      <c r="N360" s="19"/>
+      <c r="J360" s="22"/>
+      <c r="K360" s="22"/>
+      <c r="L360" s="22"/>
+      <c r="M360" s="22"/>
+      <c r="N360" s="22"/>
       <c r="O360" s="19" t="str">
         <f>CONCATENATE("M 80 ",O325)</f>
       </c>
@@ -8818,21 +8843,21 @@
       <c r="F362" t="s">
         <v>212</v>
       </c>
-      <c r="G362" s="15"/>
+      <c r="G362" s="23"/>
       <c r="N362" t="s">
         <v>212</v>
       </c>
-      <c r="O362" s="15"/>
+      <c r="O362" s="23"/>
     </row>
     <row r="363">
       <c r="F363" t="s">
         <v>213</v>
       </c>
-      <c r="G363" s="15"/>
+      <c r="G363" s="23"/>
       <c r="N363" t="s">
         <v>213</v>
       </c>
-      <c r="O363" s="15"/>
+      <c r="O363" s="23"/>
     </row>
     <row r="366">
       <c r="A366" s="11" t="s">
@@ -8878,22 +8903,22 @@
       <c r="A368" s="19" t="str">
         <f>CONCATENATE("M 79 ",G349)</f>
       </c>
-      <c r="B368" s="19"/>
-      <c r="C368" s="19"/>
-      <c r="D368" s="19"/>
-      <c r="E368" s="19"/>
-      <c r="F368" s="19"/>
+      <c r="B368" s="22"/>
+      <c r="C368" s="22"/>
+      <c r="D368" s="22"/>
+      <c r="E368" s="22"/>
+      <c r="F368" s="22"/>
       <c r="G368" s="19" t="str">
         <f>CONCATENATE("M 78 ",G341)</f>
       </c>
       <c r="I368" s="19" t="str">
         <f>CONCATENATE("M 83 ",O349)</f>
       </c>
-      <c r="J368" s="19"/>
-      <c r="K368" s="19"/>
-      <c r="L368" s="19"/>
-      <c r="M368" s="19"/>
-      <c r="N368" s="19"/>
+      <c r="J368" s="22"/>
+      <c r="K368" s="22"/>
+      <c r="L368" s="22"/>
+      <c r="M368" s="22"/>
+      <c r="N368" s="22"/>
       <c r="O368" s="19" t="str">
         <f>CONCATENATE("M 82 ",O341)</f>
       </c>
@@ -8902,21 +8927,21 @@
       <c r="F370" t="s">
         <v>212</v>
       </c>
-      <c r="G370" s="15"/>
+      <c r="G370" s="23"/>
       <c r="N370" t="s">
         <v>212</v>
       </c>
-      <c r="O370" s="15"/>
+      <c r="O370" s="23"/>
     </row>
     <row r="371">
       <c r="F371" t="s">
         <v>213</v>
       </c>
-      <c r="G371" s="15"/>
+      <c r="G371" s="23"/>
       <c r="N371" t="s">
         <v>213</v>
       </c>
-      <c r="O371" s="15"/>
+      <c r="O371" s="23"/>
     </row>
     <row r="379">
       <c r="A379" s="11" t="s">
@@ -8962,22 +8987,22 @@
       <c r="A381" s="19" t="str">
         <f>CONCATENATE("M 85 ",G370)</f>
       </c>
-      <c r="B381" s="19"/>
-      <c r="C381" s="19"/>
-      <c r="D381" s="19"/>
-      <c r="E381" s="19"/>
-      <c r="F381" s="19"/>
+      <c r="B381" s="22"/>
+      <c r="C381" s="22"/>
+      <c r="D381" s="22"/>
+      <c r="E381" s="22"/>
+      <c r="F381" s="22"/>
       <c r="G381" s="19" t="str">
         <f>CONCATENATE("M 84 ",G362)</f>
       </c>
       <c r="I381" s="19" t="str">
         <f>CONCATENATE("M 87 ",O370)</f>
       </c>
-      <c r="J381" s="19"/>
-      <c r="K381" s="19"/>
-      <c r="L381" s="19"/>
-      <c r="M381" s="19"/>
-      <c r="N381" s="19"/>
+      <c r="J381" s="22"/>
+      <c r="K381" s="22"/>
+      <c r="L381" s="22"/>
+      <c r="M381" s="22"/>
+      <c r="N381" s="22"/>
       <c r="O381" s="19" t="str">
         <f>CONCATENATE("M 86 ",O362)</f>
       </c>
@@ -8986,21 +9011,21 @@
       <c r="F383" t="s">
         <v>212</v>
       </c>
-      <c r="G383" s="15"/>
+      <c r="G383" s="23"/>
       <c r="N383" t="s">
         <v>212</v>
       </c>
-      <c r="O383" s="15"/>
+      <c r="O383" s="23"/>
     </row>
     <row r="384">
       <c r="F384" t="s">
         <v>213</v>
       </c>
-      <c r="G384" s="15"/>
+      <c r="G384" s="23"/>
       <c r="N384" t="s">
         <v>213</v>
       </c>
-      <c r="O384" s="15"/>
+      <c r="O384" s="23"/>
     </row>
     <row r="392">
       <c r="A392" s="11" t="s">
@@ -9028,11 +9053,11 @@
       <c r="A394" s="19" t="str">
         <f>CONCATENATE("M 89 ",O383)</f>
       </c>
-      <c r="B394" s="19"/>
-      <c r="C394" s="19"/>
-      <c r="D394" s="19"/>
-      <c r="E394" s="19"/>
-      <c r="F394" s="19"/>
+      <c r="B394" s="22"/>
+      <c r="C394" s="22"/>
+      <c r="D394" s="22"/>
+      <c r="E394" s="22"/>
+      <c r="F394" s="22"/>
       <c r="G394" s="19" t="str">
         <f>CONCATENATE("M 88 ",G383)</f>
       </c>
@@ -9041,15 +9066,16 @@
       <c r="F396" t="s">
         <v>212</v>
       </c>
-      <c r="G396" s="15"/>
+      <c r="G396" s="23"/>
     </row>
     <row r="397">
       <c r="F397" t="s">
         <v>213</v>
       </c>
-      <c r="G397" s="15"/>
+      <c r="G397" s="23"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="true" objects="true" scenarios="true" formatCells="true" formatColumns="true" formatRows="true" insertColumns="true" insertRows="true" insertHyperlinks="true" deleteColumns="true" deleteRows="true" selectLockedCells="false" sort="true" autoFilter="true" pivotTables="true" selectUnlockedCells="false"/>
   <mergeCells count="92">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="I1:O1"/>
@@ -9380,6 +9406,7 @@
       <c r="E35" s="12"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="true" objects="true" scenarios="true" formatCells="true" formatColumns="true" formatRows="true" insertColumns="true" insertRows="true" insertHyperlinks="true" deleteColumns="true" deleteRows="true" selectLockedCells="false" sort="true" autoFilter="true" pivotTables="true" selectUnlockedCells="false"/>
   <mergeCells count="1">
     <mergeCell ref="A1:P1"/>
   </mergeCells>
@@ -9603,6 +9630,7 @@
       <c r="E35" s="12"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="true" objects="true" scenarios="true" formatCells="true" formatColumns="true" formatRows="true" insertColumns="true" insertRows="true" insertHyperlinks="true" deleteColumns="true" deleteRows="true" selectLockedCells="false" sort="true" autoFilter="true" pivotTables="true" selectUnlockedCells="false"/>
   <mergeCells count="1">
     <mergeCell ref="A1:P1"/>
   </mergeCells>

</xml_diff>

<commit_message>
feat: implement state overrides and normalize competition data for the web API
</commit_message>
<xml_diff>
--- a/playoffs-example-large-seeded.xlsx
+++ b/playoffs-example-large-seeded.xlsx
@@ -24,7 +24,7 @@
   <definedNames>
     <definedName localSheetId="11" name="_xlnm.Print_Area">'Names to Print A'!$A$1:$B$46</definedName>
     <definedName localSheetId="12" name="_xlnm.Print_Area">'Names to Print B'!$A$1:$B$45</definedName>
-    <definedName localSheetId="2" name="_xlnm.Print_Area">'Elimination Matches'!$A$1:$O$404</definedName>
+    <definedName localSheetId="2" name="_xlnm.Print_Area">'Elimination Matches'!$A$1:$P$404</definedName>
   </definedNames>
   <calcPr calcId="122211"/>
 </workbook>
@@ -4183,7 +4183,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="18" t="str">
-        <f>data!D3</f>
+        <f>'data'!D3</f>
       </c>
     </row>
     <row r="2" ht="270" customHeight="true">
@@ -4191,7 +4191,7 @@
         <v>4</v>
       </c>
       <c r="B2" s="18" t="str">
-        <f>data!D7</f>
+        <f>'data'!D7</f>
       </c>
     </row>
     <row r="3" ht="270" customHeight="true">
@@ -4199,7 +4199,7 @@
         <v>5</v>
       </c>
       <c r="B3" s="18" t="str">
-        <f>data!D8</f>
+        <f>'data'!D8</f>
       </c>
     </row>
     <row r="4" ht="270" customHeight="true">
@@ -4207,7 +4207,7 @@
         <v>6</v>
       </c>
       <c r="B4" s="18" t="str">
-        <f>data!D9</f>
+        <f>'data'!D9</f>
       </c>
     </row>
     <row r="5" ht="270" customHeight="true">
@@ -4215,7 +4215,7 @@
         <v>7</v>
       </c>
       <c r="B5" s="18" t="str">
-        <f>data!D10</f>
+        <f>'data'!D10</f>
       </c>
     </row>
     <row r="6" ht="270" customHeight="true">
@@ -4223,7 +4223,7 @@
         <v>8</v>
       </c>
       <c r="B6" s="18" t="str">
-        <f>data!D11</f>
+        <f>'data'!D11</f>
       </c>
     </row>
     <row r="7" ht="270" customHeight="true">
@@ -4231,7 +4231,7 @@
         <v>9</v>
       </c>
       <c r="B7" s="18" t="str">
-        <f>data!D12</f>
+        <f>'data'!D12</f>
       </c>
     </row>
     <row r="8" ht="270" customHeight="true">
@@ -4239,7 +4239,7 @@
         <v>10</v>
       </c>
       <c r="B8" s="18" t="str">
-        <f>data!D13</f>
+        <f>'data'!D13</f>
       </c>
     </row>
     <row r="9" ht="270" customHeight="true">
@@ -4247,7 +4247,7 @@
         <v>11</v>
       </c>
       <c r="B9" s="18" t="str">
-        <f>data!D14</f>
+        <f>'data'!D14</f>
       </c>
     </row>
     <row r="10" ht="270" customHeight="true">
@@ -4255,7 +4255,7 @@
         <v>12</v>
       </c>
       <c r="B10" s="18" t="str">
-        <f>data!D15</f>
+        <f>'data'!D15</f>
       </c>
     </row>
     <row r="11" ht="270" customHeight="true">
@@ -4263,7 +4263,7 @@
         <v>13</v>
       </c>
       <c r="B11" s="18" t="str">
-        <f>data!D16</f>
+        <f>'data'!D16</f>
       </c>
     </row>
     <row r="12" ht="270" customHeight="true">
@@ -4271,7 +4271,7 @@
         <v>14</v>
       </c>
       <c r="B12" s="18" t="str">
-        <f>data!D17</f>
+        <f>'data'!D17</f>
       </c>
     </row>
     <row r="13" ht="270" customHeight="true">
@@ -4279,7 +4279,7 @@
         <v>15</v>
       </c>
       <c r="B13" s="18" t="str">
-        <f>data!D18</f>
+        <f>'data'!D18</f>
       </c>
     </row>
     <row r="14" ht="270" customHeight="true">
@@ -4287,7 +4287,7 @@
         <v>16</v>
       </c>
       <c r="B14" s="18" t="str">
-        <f>data!D19</f>
+        <f>'data'!D19</f>
       </c>
     </row>
     <row r="15" ht="270" customHeight="true">
@@ -4295,7 +4295,7 @@
         <v>17</v>
       </c>
       <c r="B15" s="18" t="str">
-        <f>data!D20</f>
+        <f>'data'!D20</f>
       </c>
     </row>
     <row r="16" ht="270" customHeight="true">
@@ -4303,7 +4303,7 @@
         <v>18</v>
       </c>
       <c r="B16" s="18" t="str">
-        <f>data!D21</f>
+        <f>'data'!D21</f>
       </c>
     </row>
     <row r="17" ht="270" customHeight="true">
@@ -4311,7 +4311,7 @@
         <v>19</v>
       </c>
       <c r="B17" s="18" t="str">
-        <f>data!D22</f>
+        <f>'data'!D22</f>
       </c>
     </row>
     <row r="18" ht="270" customHeight="true">
@@ -4319,7 +4319,7 @@
         <v>20</v>
       </c>
       <c r="B18" s="18" t="str">
-        <f>data!D23</f>
+        <f>'data'!D23</f>
       </c>
     </row>
     <row r="19" ht="270" customHeight="true">
@@ -4327,7 +4327,7 @@
         <v>21</v>
       </c>
       <c r="B19" s="18" t="str">
-        <f>data!D24</f>
+        <f>'data'!D24</f>
       </c>
     </row>
     <row r="20" ht="270" customHeight="true">
@@ -4335,7 +4335,7 @@
         <v>22</v>
       </c>
       <c r="B20" s="18" t="str">
-        <f>data!D25</f>
+        <f>'data'!D25</f>
       </c>
     </row>
     <row r="21" ht="270" customHeight="true">
@@ -4343,7 +4343,7 @@
         <v>23</v>
       </c>
       <c r="B21" s="18" t="str">
-        <f>data!D26</f>
+        <f>'data'!D26</f>
       </c>
     </row>
     <row r="22" ht="270" customHeight="true">
@@ -4351,7 +4351,7 @@
         <v>24</v>
       </c>
       <c r="B22" s="18" t="str">
-        <f>data!D27</f>
+        <f>'data'!D27</f>
       </c>
     </row>
     <row r="23" ht="270" customHeight="true">
@@ -4359,7 +4359,7 @@
         <v>25</v>
       </c>
       <c r="B23" s="18" t="str">
-        <f>data!D28</f>
+        <f>'data'!D28</f>
       </c>
     </row>
     <row r="24" ht="270" customHeight="true">
@@ -4367,7 +4367,7 @@
         <v>26</v>
       </c>
       <c r="B24" s="18" t="str">
-        <f>data!D29</f>
+        <f>'data'!D29</f>
       </c>
     </row>
     <row r="25" ht="270" customHeight="true">
@@ -4375,7 +4375,7 @@
         <v>27</v>
       </c>
       <c r="B25" s="18" t="str">
-        <f>data!D30</f>
+        <f>'data'!D30</f>
       </c>
     </row>
     <row r="26" ht="270" customHeight="true">
@@ -4383,7 +4383,7 @@
         <v>28</v>
       </c>
       <c r="B26" s="18" t="str">
-        <f>data!D31</f>
+        <f>'data'!D31</f>
       </c>
     </row>
     <row r="27" ht="270" customHeight="true">
@@ -4391,7 +4391,7 @@
         <v>29</v>
       </c>
       <c r="B27" s="18" t="str">
-        <f>data!D32</f>
+        <f>'data'!D32</f>
       </c>
     </row>
     <row r="28" ht="270" customHeight="true">
@@ -4399,7 +4399,7 @@
         <v>30</v>
       </c>
       <c r="B28" s="18" t="str">
-        <f>data!D33</f>
+        <f>'data'!D33</f>
       </c>
     </row>
     <row r="29" ht="270" customHeight="true">
@@ -4407,7 +4407,7 @@
         <v>31</v>
       </c>
       <c r="B29" s="18" t="str">
-        <f>data!D34</f>
+        <f>'data'!D34</f>
       </c>
     </row>
     <row r="30" ht="270" customHeight="true">
@@ -4415,7 +4415,7 @@
         <v>32</v>
       </c>
       <c r="B30" s="18" t="str">
-        <f>data!D35</f>
+        <f>'data'!D35</f>
       </c>
     </row>
     <row r="31" ht="270" customHeight="true">
@@ -4423,7 +4423,7 @@
         <v>33</v>
       </c>
       <c r="B31" s="18" t="str">
-        <f>data!D36</f>
+        <f>'data'!D36</f>
       </c>
     </row>
     <row r="32" ht="270" customHeight="true">
@@ -4431,7 +4431,7 @@
         <v>34</v>
       </c>
       <c r="B32" s="18" t="str">
-        <f>data!D37</f>
+        <f>'data'!D37</f>
       </c>
     </row>
     <row r="33" ht="270" customHeight="true">
@@ -4439,7 +4439,7 @@
         <v>3</v>
       </c>
       <c r="B33" s="18" t="str">
-        <f>data!D6</f>
+        <f>'data'!D6</f>
       </c>
     </row>
     <row r="34" ht="270" customHeight="true">
@@ -4447,7 +4447,7 @@
         <v>35</v>
       </c>
       <c r="B34" s="18" t="str">
-        <f>data!D38</f>
+        <f>'data'!D38</f>
       </c>
     </row>
     <row r="35" ht="270" customHeight="true">
@@ -4455,7 +4455,7 @@
         <v>36</v>
       </c>
       <c r="B35" s="18" t="str">
-        <f>data!D39</f>
+        <f>'data'!D39</f>
       </c>
     </row>
     <row r="36" ht="270" customHeight="true">
@@ -4463,7 +4463,7 @@
         <v>37</v>
       </c>
       <c r="B36" s="18" t="str">
-        <f>data!D40</f>
+        <f>'data'!D40</f>
       </c>
     </row>
     <row r="37" ht="270" customHeight="true">
@@ -4471,7 +4471,7 @@
         <v>38</v>
       </c>
       <c r="B37" s="18" t="str">
-        <f>data!D41</f>
+        <f>'data'!D41</f>
       </c>
     </row>
     <row r="38" ht="270" customHeight="true">
@@ -4479,7 +4479,7 @@
         <v>39</v>
       </c>
       <c r="B38" s="18" t="str">
-        <f>data!D42</f>
+        <f>'data'!D42</f>
       </c>
     </row>
     <row r="39" ht="270" customHeight="true">
@@ -4487,7 +4487,7 @@
         <v>40</v>
       </c>
       <c r="B39" s="18" t="str">
-        <f>data!D43</f>
+        <f>'data'!D43</f>
       </c>
     </row>
     <row r="40" ht="270" customHeight="true">
@@ -4495,7 +4495,7 @@
         <v>41</v>
       </c>
       <c r="B40" s="18" t="str">
-        <f>data!D44</f>
+        <f>'data'!D44</f>
       </c>
     </row>
     <row r="41" ht="270" customHeight="true">
@@ -4503,7 +4503,7 @@
         <v>42</v>
       </c>
       <c r="B41" s="18" t="str">
-        <f>data!D45</f>
+        <f>'data'!D45</f>
       </c>
     </row>
     <row r="42" ht="270" customHeight="true">
@@ -4511,7 +4511,7 @@
         <v>43</v>
       </c>
       <c r="B42" s="18" t="str">
-        <f>data!D46</f>
+        <f>'data'!D46</f>
       </c>
     </row>
     <row r="43" ht="270" customHeight="true">
@@ -4519,7 +4519,7 @@
         <v>44</v>
       </c>
       <c r="B43" s="18" t="str">
-        <f>data!D47</f>
+        <f>'data'!D47</f>
       </c>
     </row>
     <row r="44" ht="270" customHeight="true">
@@ -4527,7 +4527,7 @@
         <v>45</v>
       </c>
       <c r="B44" s="18" t="str">
-        <f>data!D48</f>
+        <f>'data'!D48</f>
       </c>
     </row>
     <row r="45" ht="270" customHeight="true">
@@ -4535,7 +4535,7 @@
         <v>46</v>
       </c>
       <c r="B45" s="18" t="str">
-        <f>data!D49</f>
+        <f>'data'!D49</f>
       </c>
     </row>
     <row r="46" ht="270" customHeight="true">
@@ -4543,7 +4543,7 @@
         <v>47</v>
       </c>
       <c r="B46" s="18" t="str">
-        <f>data!D50</f>
+        <f>'data'!D50</f>
       </c>
     </row>
   </sheetData>
@@ -4584,7 +4584,7 @@
         <v>48</v>
       </c>
       <c r="B1" s="18" t="str">
-        <f>data!D51</f>
+        <f>'data'!D51</f>
       </c>
     </row>
     <row r="2" ht="270" customHeight="true">
@@ -4592,7 +4592,7 @@
         <v>49</v>
       </c>
       <c r="B2" s="18" t="str">
-        <f>data!D52</f>
+        <f>'data'!D52</f>
       </c>
     </row>
     <row r="3" ht="270" customHeight="true">
@@ -4600,7 +4600,7 @@
         <v>50</v>
       </c>
       <c r="B3" s="18" t="str">
-        <f>data!D53</f>
+        <f>'data'!D53</f>
       </c>
     </row>
     <row r="4" ht="270" customHeight="true">
@@ -4608,7 +4608,7 @@
         <v>51</v>
       </c>
       <c r="B4" s="18" t="str">
-        <f>data!D54</f>
+        <f>'data'!D54</f>
       </c>
     </row>
     <row r="5" ht="270" customHeight="true">
@@ -4616,7 +4616,7 @@
         <v>52</v>
       </c>
       <c r="B5" s="18" t="str">
-        <f>data!D55</f>
+        <f>'data'!D55</f>
       </c>
     </row>
     <row r="6" ht="270" customHeight="true">
@@ -4624,7 +4624,7 @@
         <v>53</v>
       </c>
       <c r="B6" s="18" t="str">
-        <f>data!D56</f>
+        <f>'data'!D56</f>
       </c>
     </row>
     <row r="7" ht="270" customHeight="true">
@@ -4632,7 +4632,7 @@
         <v>54</v>
       </c>
       <c r="B7" s="18" t="str">
-        <f>data!D57</f>
+        <f>'data'!D57</f>
       </c>
     </row>
     <row r="8" ht="270" customHeight="true">
@@ -4640,7 +4640,7 @@
         <v>55</v>
       </c>
       <c r="B8" s="18" t="str">
-        <f>data!D58</f>
+        <f>'data'!D58</f>
       </c>
     </row>
     <row r="9" ht="270" customHeight="true">
@@ -4648,7 +4648,7 @@
         <v>56</v>
       </c>
       <c r="B9" s="18" t="str">
-        <f>data!D59</f>
+        <f>'data'!D59</f>
       </c>
     </row>
     <row r="10" ht="270" customHeight="true">
@@ -4656,7 +4656,7 @@
         <v>57</v>
       </c>
       <c r="B10" s="18" t="str">
-        <f>data!D60</f>
+        <f>'data'!D60</f>
       </c>
     </row>
     <row r="11" ht="270" customHeight="true">
@@ -4664,7 +4664,7 @@
         <v>58</v>
       </c>
       <c r="B11" s="18" t="str">
-        <f>data!D61</f>
+        <f>'data'!D61</f>
       </c>
     </row>
     <row r="12" ht="270" customHeight="true">
@@ -4672,7 +4672,7 @@
         <v>59</v>
       </c>
       <c r="B12" s="18" t="str">
-        <f>data!D62</f>
+        <f>'data'!D62</f>
       </c>
     </row>
     <row r="13" ht="270" customHeight="true">
@@ -4680,7 +4680,7 @@
         <v>60</v>
       </c>
       <c r="B13" s="18" t="str">
-        <f>data!D63</f>
+        <f>'data'!D63</f>
       </c>
     </row>
     <row r="14" ht="270" customHeight="true">
@@ -4688,7 +4688,7 @@
         <v>61</v>
       </c>
       <c r="B14" s="18" t="str">
-        <f>data!D64</f>
+        <f>'data'!D64</f>
       </c>
     </row>
     <row r="15" ht="270" customHeight="true">
@@ -4696,7 +4696,7 @@
         <v>62</v>
       </c>
       <c r="B15" s="18" t="str">
-        <f>data!D65</f>
+        <f>'data'!D65</f>
       </c>
     </row>
     <row r="16" ht="270" customHeight="true">
@@ -4704,7 +4704,7 @@
         <v>63</v>
       </c>
       <c r="B16" s="18" t="str">
-        <f>data!D66</f>
+        <f>'data'!D66</f>
       </c>
     </row>
     <row r="17" ht="270" customHeight="true">
@@ -4712,7 +4712,7 @@
         <v>64</v>
       </c>
       <c r="B17" s="18" t="str">
-        <f>data!D67</f>
+        <f>'data'!D67</f>
       </c>
     </row>
     <row r="18" ht="270" customHeight="true">
@@ -4720,7 +4720,7 @@
         <v>65</v>
       </c>
       <c r="B18" s="18" t="str">
-        <f>data!D68</f>
+        <f>'data'!D68</f>
       </c>
     </row>
     <row r="19" ht="270" customHeight="true">
@@ -4728,7 +4728,7 @@
         <v>1</v>
       </c>
       <c r="B19" s="18" t="str">
-        <f>data!D4</f>
+        <f>'data'!D4</f>
       </c>
     </row>
     <row r="20" ht="270" customHeight="true">
@@ -4736,7 +4736,7 @@
         <v>66</v>
       </c>
       <c r="B20" s="18" t="str">
-        <f>data!D69</f>
+        <f>'data'!D69</f>
       </c>
     </row>
     <row r="21" ht="270" customHeight="true">
@@ -4744,7 +4744,7 @@
         <v>67</v>
       </c>
       <c r="B21" s="18" t="str">
-        <f>data!D70</f>
+        <f>'data'!D70</f>
       </c>
     </row>
     <row r="22" ht="270" customHeight="true">
@@ -4752,7 +4752,7 @@
         <v>68</v>
       </c>
       <c r="B22" s="18" t="str">
-        <f>data!D71</f>
+        <f>'data'!D71</f>
       </c>
     </row>
     <row r="23" ht="270" customHeight="true">
@@ -4760,7 +4760,7 @@
         <v>69</v>
       </c>
       <c r="B23" s="18" t="str">
-        <f>data!D72</f>
+        <f>'data'!D72</f>
       </c>
     </row>
     <row r="24" ht="270" customHeight="true">
@@ -4768,7 +4768,7 @@
         <v>70</v>
       </c>
       <c r="B24" s="18" t="str">
-        <f>data!D73</f>
+        <f>'data'!D73</f>
       </c>
     </row>
     <row r="25" ht="270" customHeight="true">
@@ -4776,7 +4776,7 @@
         <v>71</v>
       </c>
       <c r="B25" s="18" t="str">
-        <f>data!D74</f>
+        <f>'data'!D74</f>
       </c>
     </row>
     <row r="26" ht="270" customHeight="true">
@@ -4784,7 +4784,7 @@
         <v>72</v>
       </c>
       <c r="B26" s="18" t="str">
-        <f>data!D75</f>
+        <f>'data'!D75</f>
       </c>
     </row>
     <row r="27" ht="270" customHeight="true">
@@ -4792,7 +4792,7 @@
         <v>73</v>
       </c>
       <c r="B27" s="18" t="str">
-        <f>data!D76</f>
+        <f>'data'!D76</f>
       </c>
     </row>
     <row r="28" ht="270" customHeight="true">
@@ -4800,7 +4800,7 @@
         <v>74</v>
       </c>
       <c r="B28" s="18" t="str">
-        <f>data!D77</f>
+        <f>'data'!D77</f>
       </c>
     </row>
     <row r="29" ht="270" customHeight="true">
@@ -4808,7 +4808,7 @@
         <v>75</v>
       </c>
       <c r="B29" s="18" t="str">
-        <f>data!D78</f>
+        <f>'data'!D78</f>
       </c>
     </row>
     <row r="30" ht="270" customHeight="true">
@@ -4816,7 +4816,7 @@
         <v>76</v>
       </c>
       <c r="B30" s="18" t="str">
-        <f>data!D79</f>
+        <f>'data'!D79</f>
       </c>
     </row>
     <row r="31" ht="270" customHeight="true">
@@ -4824,7 +4824,7 @@
         <v>77</v>
       </c>
       <c r="B31" s="18" t="str">
-        <f>data!D80</f>
+        <f>'data'!D80</f>
       </c>
     </row>
     <row r="32" ht="270" customHeight="true">
@@ -4832,7 +4832,7 @@
         <v>78</v>
       </c>
       <c r="B32" s="18" t="str">
-        <f>data!D81</f>
+        <f>'data'!D81</f>
       </c>
     </row>
     <row r="33" ht="270" customHeight="true">
@@ -4840,7 +4840,7 @@
         <v>79</v>
       </c>
       <c r="B33" s="18" t="str">
-        <f>data!D82</f>
+        <f>'data'!D82</f>
       </c>
     </row>
     <row r="34" ht="270" customHeight="true">
@@ -4848,7 +4848,7 @@
         <v>80</v>
       </c>
       <c r="B34" s="18" t="str">
-        <f>data!D83</f>
+        <f>'data'!D83</f>
       </c>
     </row>
     <row r="35" ht="270" customHeight="true">
@@ -4856,7 +4856,7 @@
         <v>81</v>
       </c>
       <c r="B35" s="18" t="str">
-        <f>data!D84</f>
+        <f>'data'!D84</f>
       </c>
     </row>
     <row r="36" ht="270" customHeight="true">
@@ -4864,7 +4864,7 @@
         <v>82</v>
       </c>
       <c r="B36" s="18" t="str">
-        <f>data!D85</f>
+        <f>'data'!D85</f>
       </c>
     </row>
     <row r="37" ht="270" customHeight="true">
@@ -4872,7 +4872,7 @@
         <v>83</v>
       </c>
       <c r="B37" s="18" t="str">
-        <f>data!D86</f>
+        <f>'data'!D86</f>
       </c>
     </row>
     <row r="38" ht="270" customHeight="true">
@@ -4880,7 +4880,7 @@
         <v>84</v>
       </c>
       <c r="B38" s="18" t="str">
-        <f>data!D87</f>
+        <f>'data'!D87</f>
       </c>
     </row>
     <row r="39" ht="270" customHeight="true">
@@ -4888,7 +4888,7 @@
         <v>85</v>
       </c>
       <c r="B39" s="18" t="str">
-        <f>data!D88</f>
+        <f>'data'!D88</f>
       </c>
     </row>
     <row r="40" ht="270" customHeight="true">
@@ -4896,7 +4896,7 @@
         <v>86</v>
       </c>
       <c r="B40" s="18" t="str">
-        <f>data!D89</f>
+        <f>'data'!D89</f>
       </c>
     </row>
     <row r="41" ht="270" customHeight="true">
@@ -4904,7 +4904,7 @@
         <v>87</v>
       </c>
       <c r="B41" s="18" t="str">
-        <f>data!D90</f>
+        <f>'data'!D90</f>
       </c>
     </row>
     <row r="42" ht="270" customHeight="true">
@@ -4912,7 +4912,7 @@
         <v>88</v>
       </c>
       <c r="B42" s="18" t="str">
-        <f>data!D91</f>
+        <f>'data'!D91</f>
       </c>
     </row>
     <row r="43" ht="270" customHeight="true">
@@ -4920,7 +4920,7 @@
         <v>89</v>
       </c>
       <c r="B43" s="18" t="str">
-        <f>data!D92</f>
+        <f>'data'!D92</f>
       </c>
     </row>
     <row r="44" ht="270" customHeight="true">
@@ -4928,7 +4928,7 @@
         <v>90</v>
       </c>
       <c r="B44" s="18" t="str">
-        <f>data!D93</f>
+        <f>'data'!D93</f>
       </c>
     </row>
     <row r="45" ht="270" customHeight="true">
@@ -4936,7 +4936,7 @@
         <v>2</v>
       </c>
       <c r="B45" s="18" t="str">
-        <f>data!D5</f>
+        <f>'data'!D5</f>
       </c>
     </row>
   </sheetData>
@@ -5249,19 +5249,14 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col customWidth="true" max="1" min="1" width="30"/>
-    <col customWidth="true" max="3" min="2" width="5"/>
-    <col customWidth="true" max="4" min="4" width="3"/>
-    <col customWidth="true" max="6" min="5" width="5"/>
+    <col customWidth="true" max="6" min="2" width="5"/>
     <col customWidth="true" max="7" min="7" width="30"/>
     <col customWidth="true" max="8" min="8" width="5"/>
     <col customWidth="true" max="9" min="9" width="30"/>
-    <col customWidth="true" max="11" min="10" width="5"/>
-    <col customWidth="true" max="12" min="12" width="3"/>
-    <col customWidth="true" max="14" min="13" width="5"/>
+    <col customWidth="true" max="14" min="10" width="5"/>
     <col customWidth="true" max="15" min="15" width="30"/>
-    <col customWidth="true" max="18" min="16" width="5"/>
-    <col customWidth="true" max="19" min="19" width="30"/>
-    <col customWidth="true" max="20" min="20" width="2"/>
+    <col customWidth="true" max="16" min="16" width="5"/>
+    <col customWidth="true" max="20" min="17" width="10.83"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
chore: regenerate example workbooks
Regenerated via `make examples` after the Excel clipping fix (ShrinkToFit,
narrower Tags column, print area) and the playoffs-only Data sheet's
"Number" -> "Draw order" column A rename, both of which change bytes in
every tracked example workbook.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/playoffs-example-large-seeded.xlsx
+++ b/playoffs-example-large-seeded.xlsx
@@ -74,7 +74,7 @@
     <t/>
   </si>
   <si>
-    <t>Number</t>
+    <t>Draw order</t>
   </si>
   <si>
     <t>Player Name</t>
@@ -1469,7 +1469,7 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" shrinkToFit="true" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
@@ -1808,7 +1808,7 @@
     </row>
     <row r="3">
       <c r="A3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B3" t="s">
         <v>17</v>
@@ -1825,7 +1825,7 @@
     </row>
     <row r="4">
       <c r="A4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B4" t="s">
         <v>21</v>
@@ -1842,7 +1842,7 @@
     </row>
     <row r="5">
       <c r="A5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B5" t="s">
         <v>25</v>
@@ -1859,7 +1859,7 @@
     </row>
     <row r="6">
       <c r="A6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B6" t="s">
         <v>29</v>
@@ -1876,7 +1876,7 @@
     </row>
     <row r="7">
       <c r="A7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B7" t="s">
         <v>33</v>
@@ -1893,7 +1893,7 @@
     </row>
     <row r="8">
       <c r="A8">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B8" t="s">
         <v>37</v>
@@ -1910,7 +1910,7 @@
     </row>
     <row r="9">
       <c r="A9">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B9" t="s">
         <v>40</v>
@@ -1927,7 +1927,7 @@
     </row>
     <row r="10">
       <c r="A10">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B10" t="s">
         <v>43</v>
@@ -1944,7 +1944,7 @@
     </row>
     <row r="11">
       <c r="A11">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B11" t="s">
         <v>46</v>
@@ -1961,7 +1961,7 @@
     </row>
     <row r="12">
       <c r="A12">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B12" t="s">
         <v>49</v>
@@ -1978,7 +1978,7 @@
     </row>
     <row r="13">
       <c r="A13">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B13" t="s">
         <v>52</v>
@@ -1995,7 +1995,7 @@
     </row>
     <row r="14">
       <c r="A14">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B14" t="s">
         <v>55</v>
@@ -2012,7 +2012,7 @@
     </row>
     <row r="15">
       <c r="A15">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B15" t="s">
         <v>58</v>
@@ -2029,7 +2029,7 @@
     </row>
     <row r="16">
       <c r="A16">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B16" t="s">
         <v>61</v>
@@ -2046,7 +2046,7 @@
     </row>
     <row r="17">
       <c r="A17">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B17" t="s">
         <v>64</v>
@@ -2063,7 +2063,7 @@
     </row>
     <row r="18">
       <c r="A18">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B18" t="s">
         <v>67</v>
@@ -2080,7 +2080,7 @@
     </row>
     <row r="19">
       <c r="A19">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B19" t="s">
         <v>70</v>
@@ -2097,7 +2097,7 @@
     </row>
     <row r="20">
       <c r="A20">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B20" t="s">
         <v>73</v>
@@ -2114,7 +2114,7 @@
     </row>
     <row r="21">
       <c r="A21">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B21" t="s">
         <v>76</v>
@@ -2131,7 +2131,7 @@
     </row>
     <row r="22">
       <c r="A22">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B22" t="s">
         <v>79</v>
@@ -2148,7 +2148,7 @@
     </row>
     <row r="23">
       <c r="A23">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B23" t="s">
         <v>82</v>
@@ -2165,7 +2165,7 @@
     </row>
     <row r="24">
       <c r="A24">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B24" t="s">
         <v>85</v>
@@ -2182,7 +2182,7 @@
     </row>
     <row r="25">
       <c r="A25">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B25" t="s">
         <v>89</v>
@@ -2199,7 +2199,7 @@
     </row>
     <row r="26">
       <c r="A26">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B26" t="s">
         <v>93</v>
@@ -2216,7 +2216,7 @@
     </row>
     <row r="27">
       <c r="A27">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B27" t="s">
         <v>97</v>
@@ -2233,7 +2233,7 @@
     </row>
     <row r="28">
       <c r="A28">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B28" t="s">
         <v>101</v>
@@ -2250,7 +2250,7 @@
     </row>
     <row r="29">
       <c r="A29">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B29" t="s">
         <v>105</v>
@@ -2267,7 +2267,7 @@
     </row>
     <row r="30">
       <c r="A30">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B30" t="s">
         <v>108</v>
@@ -2284,7 +2284,7 @@
     </row>
     <row r="31">
       <c r="A31">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B31" t="s">
         <v>110</v>
@@ -2301,7 +2301,7 @@
     </row>
     <row r="32">
       <c r="A32">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B32" t="s">
         <v>113</v>
@@ -2318,7 +2318,7 @@
     </row>
     <row r="33">
       <c r="A33">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B33" t="s">
         <v>115</v>
@@ -2335,7 +2335,7 @@
     </row>
     <row r="34">
       <c r="A34">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B34" t="s">
         <v>117</v>
@@ -2352,7 +2352,7 @@
     </row>
     <row r="35">
       <c r="A35">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B35" t="s">
         <v>119</v>
@@ -2369,7 +2369,7 @@
     </row>
     <row r="36">
       <c r="A36">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B36" t="s">
         <v>121</v>
@@ -2386,7 +2386,7 @@
     </row>
     <row r="37">
       <c r="A37">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B37" t="s">
         <v>123</v>
@@ -2403,7 +2403,7 @@
     </row>
     <row r="38">
       <c r="A38">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B38" t="s">
         <v>125</v>
@@ -2420,7 +2420,7 @@
     </row>
     <row r="39">
       <c r="A39">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B39" t="s">
         <v>127</v>
@@ -2437,7 +2437,7 @@
     </row>
     <row r="40">
       <c r="A40">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B40" t="s">
         <v>129</v>
@@ -2454,7 +2454,7 @@
     </row>
     <row r="41">
       <c r="A41">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B41" t="s">
         <v>131</v>
@@ -2471,7 +2471,7 @@
     </row>
     <row r="42">
       <c r="A42">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B42" t="s">
         <v>133</v>
@@ -2488,7 +2488,7 @@
     </row>
     <row r="43">
       <c r="A43">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B43" t="s">
         <v>135</v>
@@ -2505,7 +2505,7 @@
     </row>
     <row r="44">
       <c r="A44">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B44" t="s">
         <v>137</v>
@@ -2522,7 +2522,7 @@
     </row>
     <row r="45">
       <c r="A45">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B45" t="s">
         <v>140</v>
@@ -2539,7 +2539,7 @@
     </row>
     <row r="46">
       <c r="A46">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B46" t="s">
         <v>143</v>
@@ -2556,7 +2556,7 @@
     </row>
     <row r="47">
       <c r="A47">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B47" t="s">
         <v>146</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="48">
       <c r="A48">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B48" t="s">
         <v>149</v>
@@ -2590,7 +2590,7 @@
     </row>
     <row r="49">
       <c r="A49">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B49" t="s">
         <v>152</v>
@@ -2607,7 +2607,7 @@
     </row>
     <row r="50">
       <c r="A50">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B50" t="s">
         <v>155</v>
@@ -2624,7 +2624,7 @@
     </row>
     <row r="51">
       <c r="A51">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B51" t="s">
         <v>158</v>
@@ -2641,7 +2641,7 @@
     </row>
     <row r="52">
       <c r="A52">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B52" t="s">
         <v>161</v>
@@ -2658,7 +2658,7 @@
     </row>
     <row r="53">
       <c r="A53">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B53" t="s">
         <v>164</v>
@@ -2675,7 +2675,7 @@
     </row>
     <row r="54">
       <c r="A54">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B54" t="s">
         <v>167</v>
@@ -2692,7 +2692,7 @@
     </row>
     <row r="55">
       <c r="A55">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B55" t="s">
         <v>171</v>
@@ -2709,7 +2709,7 @@
     </row>
     <row r="56">
       <c r="A56">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B56" t="s">
         <v>175</v>
@@ -2726,7 +2726,7 @@
     </row>
     <row r="57">
       <c r="A57">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B57" t="s">
         <v>179</v>
@@ -2743,7 +2743,7 @@
     </row>
     <row r="58">
       <c r="A58">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B58" t="s">
         <v>183</v>
@@ -2760,7 +2760,7 @@
     </row>
     <row r="59">
       <c r="A59">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B59" t="s">
         <v>187</v>
@@ -2777,7 +2777,7 @@
     </row>
     <row r="60">
       <c r="A60">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B60" t="s">
         <v>191</v>
@@ -2794,7 +2794,7 @@
     </row>
     <row r="61">
       <c r="A61">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B61" t="s">
         <v>195</v>
@@ -2811,7 +2811,7 @@
     </row>
     <row r="62">
       <c r="A62">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B62" t="s">
         <v>199</v>
@@ -2828,7 +2828,7 @@
     </row>
     <row r="63">
       <c r="A63">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B63" t="s">
         <v>203</v>
@@ -2845,7 +2845,7 @@
     </row>
     <row r="64">
       <c r="A64">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B64" t="s">
         <v>207</v>
@@ -2862,7 +2862,7 @@
     </row>
     <row r="65">
       <c r="A65">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B65" t="s">
         <v>211</v>
@@ -2879,7 +2879,7 @@
     </row>
     <row r="66">
       <c r="A66">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B66" t="s">
         <v>215</v>
@@ -2896,7 +2896,7 @@
     </row>
     <row r="67">
       <c r="A67">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B67" t="s">
         <v>219</v>
@@ -2913,7 +2913,7 @@
     </row>
     <row r="68">
       <c r="A68">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B68" t="s">
         <v>223</v>
@@ -2930,7 +2930,7 @@
     </row>
     <row r="69">
       <c r="A69">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B69" t="s">
         <v>226</v>
@@ -2947,7 +2947,7 @@
     </row>
     <row r="70">
       <c r="A70">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B70" t="s">
         <v>229</v>
@@ -2964,7 +2964,7 @@
     </row>
     <row r="71">
       <c r="A71">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B71" t="s">
         <v>232</v>
@@ -2981,7 +2981,7 @@
     </row>
     <row r="72">
       <c r="A72">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B72" t="s">
         <v>235</v>
@@ -2998,7 +2998,7 @@
     </row>
     <row r="73">
       <c r="A73">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B73" t="s">
         <v>238</v>
@@ -3015,7 +3015,7 @@
     </row>
     <row r="74">
       <c r="A74">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B74" t="s">
         <v>241</v>
@@ -3032,7 +3032,7 @@
     </row>
     <row r="75">
       <c r="A75">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B75" t="s">
         <v>243</v>
@@ -3049,7 +3049,7 @@
     </row>
     <row r="76">
       <c r="A76">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B76" t="s">
         <v>246</v>
@@ -3066,7 +3066,7 @@
     </row>
     <row r="77">
       <c r="A77">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B77" t="s">
         <v>249</v>
@@ -3083,7 +3083,7 @@
     </row>
     <row r="78">
       <c r="A78">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B78" t="s">
         <v>252</v>
@@ -3100,7 +3100,7 @@
     </row>
     <row r="79">
       <c r="A79">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B79" t="s">
         <v>255</v>
@@ -3117,7 +3117,7 @@
     </row>
     <row r="80">
       <c r="A80">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B80" t="s">
         <v>258</v>
@@ -3134,7 +3134,7 @@
     </row>
     <row r="81">
       <c r="A81">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B81" t="s">
         <v>261</v>
@@ -3151,7 +3151,7 @@
     </row>
     <row r="82">
       <c r="A82">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B82" t="s">
         <v>263</v>
@@ -3168,7 +3168,7 @@
     </row>
     <row r="83">
       <c r="A83">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B83" t="s">
         <v>266</v>
@@ -3185,7 +3185,7 @@
     </row>
     <row r="84">
       <c r="A84">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B84" t="s">
         <v>269</v>
@@ -3202,7 +3202,7 @@
     </row>
     <row r="85">
       <c r="A85">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B85" t="s">
         <v>272</v>
@@ -3219,7 +3219,7 @@
     </row>
     <row r="86">
       <c r="A86">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B86" t="s">
         <v>275</v>
@@ -3236,7 +3236,7 @@
     </row>
     <row r="87">
       <c r="A87">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B87" t="s">
         <v>278</v>
@@ -3253,7 +3253,7 @@
     </row>
     <row r="88">
       <c r="A88">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B88" t="s">
         <v>281</v>
@@ -3270,7 +3270,7 @@
     </row>
     <row r="89">
       <c r="A89">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B89" t="s">
         <v>283</v>
@@ -3287,7 +3287,7 @@
     </row>
     <row r="90">
       <c r="A90">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B90" t="s">
         <v>286</v>
@@ -3304,7 +3304,7 @@
     </row>
     <row r="91">
       <c r="A91">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B91" t="s">
         <v>289</v>
@@ -3321,7 +3321,7 @@
     </row>
     <row r="92">
       <c r="A92">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B92" t="s">
         <v>292</v>
@@ -3338,7 +3338,7 @@
     </row>
     <row r="93">
       <c r="A93">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B93" t="s">
         <v>295</v>

</xml_diff>

<commit_message>
chore(examples): regenerate example workbooks after the bc-drwx draw fixes
make examples run against the final state of this PR. The seed/dojo/pool
fixes (items 1-10) change placement for some of these committed rosters
(dojo-tree meeting-round scoring, dojo string normalization, wrapped-seed
placement, pool-size remainder spread, pool naming, the tier-d exchange
guard); the workbooks are regenerated to match. mock_data_small_3_teams.csv
was also fixed in an earlier commit (item 10: it lacked a dojo column),
which changes pools-example-small-3-teams.xlsx's roster too.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/playoffs-example-large-seeded.xlsx
+++ b/playoffs-example-large-seeded.xlsx
@@ -2838,7 +2838,7 @@
     </row>
     <row r="5">
       <c r="C5" s="16" t="s">
-        <v>77</v>
+        <v>126</v>
       </c>
     </row>
     <row r="6">
@@ -2849,7 +2849,7 @@
     </row>
     <row r="7">
       <c r="C7" s="16" t="s">
-        <v>79</v>
+        <v>120</v>
       </c>
       <c r="D7" s="15"/>
       <c r="E7" s="12"/>
@@ -2915,7 +2915,7 @@
     </row>
     <row r="19">
       <c r="C19" s="16" t="s">
-        <v>18</v>
+        <v>141</v>
       </c>
       <c r="D19" s="15"/>
       <c r="E19" s="12"/>
@@ -2950,7 +2950,7 @@
     </row>
     <row r="25">
       <c r="C25" s="16" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="G25" s="12"/>
       <c r="H25" s="14"/>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="9">
       <c r="C9" s="16" t="s">
-        <v>106</v>
+        <v>38</v>
       </c>
       <c r="G9" s="12"/>
       <c r="H9" s="14"/>
@@ -3101,7 +3101,7 @@
     </row>
     <row r="11">
       <c r="C11" s="16" t="s">
-        <v>40</v>
+        <v>164</v>
       </c>
       <c r="D11" s="15"/>
       <c r="E11" s="12"/>
@@ -3121,7 +3121,7 @@
       <c r="C14" s="16"/>
       <c r="D14" s="16"/>
       <c r="E14" s="16" t="s">
-        <v>42</v>
+        <v>147</v>
       </c>
       <c r="I14" s="12"/>
       <c r="K14" s="12"/>
@@ -3142,7 +3142,7 @@
     </row>
     <row r="17">
       <c r="C17" s="16" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="G17" s="12"/>
       <c r="K17" s="12"/>
@@ -3158,7 +3158,7 @@
     </row>
     <row r="19">
       <c r="C19" s="16" t="s">
-        <v>46</v>
+        <v>201</v>
       </c>
       <c r="D19" s="15"/>
       <c r="E19" s="12"/>
@@ -3265,7 +3265,7 @@
     </row>
     <row r="35">
       <c r="C35" s="16" t="s">
-        <v>38</v>
+        <v>106</v>
       </c>
       <c r="D35" s="15"/>
       <c r="E35" s="12"/>
@@ -3406,7 +3406,7 @@
       <c r="C22" s="16"/>
       <c r="D22" s="16"/>
       <c r="E22" s="16" t="s">
-        <v>120</v>
+        <v>38</v>
       </c>
       <c r="K22" s="12"/>
     </row>
@@ -3423,7 +3423,7 @@
     </row>
     <row r="25">
       <c r="C25" s="16" t="s">
-        <v>123</v>
+        <v>52</v>
       </c>
       <c r="G25" s="12"/>
       <c r="H25" s="14"/>
@@ -3442,7 +3442,7 @@
     </row>
     <row r="27">
       <c r="C27" s="16" t="s">
-        <v>126</v>
+        <v>30</v>
       </c>
       <c r="D27" s="15"/>
       <c r="E27" s="12"/>
@@ -3463,7 +3463,7 @@
       <c r="C30" s="16"/>
       <c r="D30" s="16"/>
       <c r="E30" s="16" t="s">
-        <v>129</v>
+        <v>34</v>
       </c>
       <c r="I30" s="12"/>
     </row>
@@ -3481,7 +3481,7 @@
     </row>
     <row r="33">
       <c r="C33" s="16" t="s">
-        <v>132</v>
+        <v>36</v>
       </c>
       <c r="G33" s="12"/>
     </row>
@@ -3495,7 +3495,7 @@
     </row>
     <row r="35">
       <c r="C35" s="16" t="s">
-        <v>60</v>
+        <v>135</v>
       </c>
       <c r="D35" s="15"/>
       <c r="E35" s="12"/>
@@ -3543,7 +3543,7 @@
       <c r="C6" s="16"/>
       <c r="D6" s="16"/>
       <c r="E6" s="16" t="s">
-        <v>138</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7">
@@ -3557,7 +3557,7 @@
     </row>
     <row r="9">
       <c r="C9" s="16" t="s">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="G9" s="12"/>
       <c r="H9" s="14"/>
@@ -3574,7 +3574,7 @@
     </row>
     <row r="11">
       <c r="C11" s="16" t="s">
-        <v>62</v>
+        <v>144</v>
       </c>
       <c r="D11" s="15"/>
       <c r="E11" s="12"/>
@@ -3594,7 +3594,7 @@
       <c r="C14" s="16"/>
       <c r="D14" s="16"/>
       <c r="E14" s="16" t="s">
-        <v>36</v>
+        <v>181</v>
       </c>
       <c r="I14" s="12"/>
       <c r="K14" s="12"/>
@@ -3666,7 +3666,7 @@
     </row>
     <row r="25">
       <c r="C25" s="16" t="s">
-        <v>158</v>
+        <v>62</v>
       </c>
       <c r="G25" s="12"/>
       <c r="H25" s="14"/>
@@ -3724,7 +3724,7 @@
     </row>
     <row r="33">
       <c r="C33" s="16" t="s">
-        <v>190</v>
+        <v>162</v>
       </c>
       <c r="G33" s="12"/>
     </row>
@@ -3915,7 +3915,7 @@
     </row>
     <row r="27">
       <c r="C27" s="16" t="s">
-        <v>52</v>
+        <v>32</v>
       </c>
       <c r="D27" s="15"/>
       <c r="E27" s="12"/>
@@ -3936,7 +3936,7 @@
       <c r="C30" s="16"/>
       <c r="D30" s="16"/>
       <c r="E30" s="16" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="I30" s="12"/>
     </row>
@@ -3954,7 +3954,7 @@
     </row>
     <row r="33">
       <c r="C33" s="16" t="s">
-        <v>46</v>
+        <v>132</v>
       </c>
       <c r="G33" s="12"/>
     </row>
@@ -3968,7 +3968,7 @@
     </row>
     <row r="35">
       <c r="C35" s="16" t="s">
-        <v>38</v>
+        <v>184</v>
       </c>
       <c r="D35" s="15"/>
       <c r="E35" s="12"/>
@@ -4016,7 +4016,7 @@
       <c r="C6" s="16"/>
       <c r="D6" s="16"/>
       <c r="E6" s="16" t="s">
-        <v>40</v>
+        <v>186</v>
       </c>
     </row>
     <row r="7">
@@ -4030,7 +4030,7 @@
     </row>
     <row r="9">
       <c r="C9" s="16" t="s">
-        <v>32</v>
+        <v>188</v>
       </c>
       <c r="G9" s="12"/>
       <c r="H9" s="14"/>
@@ -4047,7 +4047,7 @@
     </row>
     <row r="11">
       <c r="C11" s="16" t="s">
-        <v>162</v>
+        <v>24</v>
       </c>
       <c r="D11" s="15"/>
       <c r="E11" s="12"/>
@@ -4067,7 +4067,7 @@
       <c r="C14" s="16"/>
       <c r="D14" s="16"/>
       <c r="E14" s="16" t="s">
-        <v>30</v>
+        <v>192</v>
       </c>
       <c r="I14" s="12"/>
       <c r="K14" s="12"/>
@@ -4088,7 +4088,7 @@
     </row>
     <row r="17">
       <c r="C17" s="16" t="s">
-        <v>44</v>
+        <v>194</v>
       </c>
       <c r="G17" s="12"/>
       <c r="K17" s="12"/>
@@ -4104,7 +4104,7 @@
     </row>
     <row r="19">
       <c r="C19" s="16" t="s">
-        <v>164</v>
+        <v>40</v>
       </c>
       <c r="D19" s="15"/>
       <c r="E19" s="12"/>
@@ -4139,7 +4139,7 @@
     </row>
     <row r="25">
       <c r="C25" s="16" t="s">
-        <v>199</v>
+        <v>44</v>
       </c>
       <c r="G25" s="12"/>
       <c r="H25" s="14"/>
@@ -4158,7 +4158,7 @@
     </row>
     <row r="27">
       <c r="C27" s="16" t="s">
-        <v>201</v>
+        <v>46</v>
       </c>
       <c r="D27" s="15"/>
       <c r="E27" s="12"/>
@@ -4244,74 +4244,74 @@
     </row>
     <row r="2" ht="270" customHeight="true">
       <c r="A2" s="17">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B2" s="18" t="str">
-        <f>'data'!D26</f>
+        <f>'data'!D28</f>
       </c>
     </row>
     <row r="3" ht="270" customHeight="true">
       <c r="A3" s="17">
-        <v>24</v>
+        <v>76</v>
       </c>
       <c r="B3" s="18" t="str">
-        <f>'data'!D27</f>
+        <f>'data'!D79</f>
       </c>
     </row>
     <row r="4" ht="270" customHeight="true">
       <c r="A4" s="17">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="B4" s="18" t="str">
-        <f>'data'!D62</f>
+        <f>'data'!D58</f>
       </c>
     </row>
     <row r="5" ht="270" customHeight="true">
       <c r="A5" s="17">
-        <v>22</v>
+        <v>56</v>
       </c>
       <c r="B5" s="18" t="str">
-        <f>'data'!D25</f>
+        <f>'data'!D59</f>
       </c>
     </row>
     <row r="6" ht="270" customHeight="true">
       <c r="A6" s="17">
-        <v>79</v>
+        <v>26</v>
       </c>
       <c r="B6" s="18" t="str">
-        <f>'data'!D82</f>
+        <f>'data'!D29</f>
       </c>
     </row>
     <row r="7" ht="270" customHeight="true">
       <c r="A7" s="17">
-        <v>80</v>
+        <v>9</v>
       </c>
       <c r="B7" s="18" t="str">
-        <f>'data'!D83</f>
+        <f>'data'!D12</f>
       </c>
     </row>
     <row r="8" ht="270" customHeight="true">
       <c r="A8" s="17">
-        <v>31</v>
+        <v>58</v>
       </c>
       <c r="B8" s="18" t="str">
-        <f>'data'!D34</f>
+        <f>'data'!D61</f>
       </c>
     </row>
     <row r="9" ht="270" customHeight="true">
       <c r="A9" s="17">
-        <v>77</v>
+        <v>11</v>
       </c>
       <c r="B9" s="18" t="str">
-        <f>'data'!D80</f>
+        <f>'data'!D14</f>
       </c>
     </row>
     <row r="10" ht="270" customHeight="true">
       <c r="A10" s="17">
-        <v>78</v>
+        <v>12</v>
       </c>
       <c r="B10" s="18" t="str">
-        <f>'data'!D81</f>
+        <f>'data'!D15</f>
       </c>
     </row>
     <row r="11" ht="270" customHeight="true">
@@ -4332,18 +4332,18 @@
     </row>
     <row r="13" ht="270" customHeight="true">
       <c r="A13" s="17">
-        <v>76</v>
+        <v>53</v>
       </c>
       <c r="B13" s="18" t="str">
-        <f>'data'!D79</f>
+        <f>'data'!D56</f>
       </c>
     </row>
     <row r="14" ht="270" customHeight="true">
       <c r="A14" s="17">
-        <v>16</v>
+        <v>82</v>
       </c>
       <c r="B14" s="18" t="str">
-        <f>'data'!D19</f>
+        <f>'data'!D85</f>
       </c>
     </row>
     <row r="15" ht="270" customHeight="true">
@@ -4364,18 +4364,18 @@
     </row>
     <row r="17" ht="270" customHeight="true">
       <c r="A17" s="17">
-        <v>57</v>
+        <v>19</v>
       </c>
       <c r="B17" s="18" t="str">
-        <f>'data'!D60</f>
+        <f>'data'!D22</f>
       </c>
     </row>
     <row r="18" ht="270" customHeight="true">
       <c r="A18" s="17">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="B18" s="18" t="str">
-        <f>'data'!D63</f>
+        <f>'data'!D68</f>
       </c>
     </row>
     <row r="19" ht="270" customHeight="true">
@@ -4388,42 +4388,42 @@
     </row>
     <row r="20" ht="270" customHeight="true">
       <c r="A20" s="17">
-        <v>61</v>
+        <v>22</v>
       </c>
       <c r="B20" s="18" t="str">
-        <f>'data'!D64</f>
+        <f>'data'!D25</f>
       </c>
     </row>
     <row r="21" ht="270" customHeight="true">
       <c r="A21" s="17">
-        <v>83</v>
+        <v>23</v>
       </c>
       <c r="B21" s="18" t="str">
-        <f>'data'!D86</f>
+        <f>'data'!D26</f>
       </c>
     </row>
     <row r="22" ht="270" customHeight="true">
       <c r="A22" s="17">
-        <v>81</v>
+        <v>24</v>
       </c>
       <c r="B22" s="18" t="str">
-        <f>'data'!D84</f>
+        <f>'data'!D27</f>
       </c>
     </row>
     <row r="23" ht="270" customHeight="true">
       <c r="A23" s="17">
-        <v>25</v>
+        <v>54</v>
       </c>
       <c r="B23" s="18" t="str">
-        <f>'data'!D28</f>
+        <f>'data'!D57</f>
       </c>
     </row>
     <row r="24" ht="270" customHeight="true">
       <c r="A24" s="17">
-        <v>26</v>
+        <v>52</v>
       </c>
       <c r="B24" s="18" t="str">
-        <f>'data'!D29</f>
+        <f>'data'!D55</f>
       </c>
     </row>
     <row r="25" ht="270" customHeight="true">
@@ -4444,10 +4444,10 @@
     </row>
     <row r="27" ht="270" customHeight="true">
       <c r="A27" s="17">
-        <v>29</v>
+        <v>59</v>
       </c>
       <c r="B27" s="18" t="str">
-        <f>'data'!D32</f>
+        <f>'data'!D62</f>
       </c>
     </row>
     <row r="28" ht="270" customHeight="true">
@@ -4460,10 +4460,10 @@
     </row>
     <row r="29" ht="270" customHeight="true">
       <c r="A29" s="17">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="B29" s="18" t="str">
-        <f>'data'!D13</f>
+        <f>'data'!D19</f>
       </c>
     </row>
     <row r="30" ht="270" customHeight="true">
@@ -4508,42 +4508,42 @@
     </row>
     <row r="35" ht="270" customHeight="true">
       <c r="A35" s="17">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="B35" s="18" t="str">
-        <f>'data'!D49</f>
+        <f>'data'!D39</f>
       </c>
     </row>
     <row r="36" ht="270" customHeight="true">
       <c r="A36" s="17">
-        <v>37</v>
+        <v>85</v>
       </c>
       <c r="B36" s="18" t="str">
-        <f>'data'!D40</f>
+        <f>'data'!D88</f>
       </c>
     </row>
     <row r="37" ht="270" customHeight="true">
       <c r="A37" s="17">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="B37" s="18" t="str">
-        <f>'data'!D41</f>
+        <f>'data'!D64</f>
       </c>
     </row>
     <row r="38" ht="270" customHeight="true">
       <c r="A38" s="17">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B38" s="18" t="str">
-        <f>'data'!D87</f>
+        <f>'data'!D90</f>
       </c>
     </row>
     <row r="39" ht="270" customHeight="true">
       <c r="A39" s="17">
-        <v>40</v>
+        <v>88</v>
       </c>
       <c r="B39" s="18" t="str">
-        <f>'data'!D43</f>
+        <f>'data'!D91</f>
       </c>
     </row>
     <row r="40" ht="270" customHeight="true">
@@ -4588,10 +4588,10 @@
     </row>
     <row r="45" ht="270" customHeight="true">
       <c r="A45" s="17">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="B45" s="18" t="str">
-        <f>'data'!D39</f>
+        <f>'data'!D49</f>
       </c>
     </row>
     <row r="46" ht="270" customHeight="true">
@@ -4669,82 +4669,82 @@
     </row>
     <row r="5" ht="270" customHeight="true">
       <c r="A5" s="17">
-        <v>52</v>
+        <v>8</v>
       </c>
       <c r="B5" s="18" t="str">
-        <f>'data'!D55</f>
+        <f>'data'!D11</f>
       </c>
     </row>
     <row r="6" ht="270" customHeight="true">
       <c r="A6" s="17">
-        <v>53</v>
+        <v>15</v>
       </c>
       <c r="B6" s="18" t="str">
-        <f>'data'!D56</f>
+        <f>'data'!D18</f>
       </c>
     </row>
     <row r="7" ht="270" customHeight="true">
       <c r="A7" s="17">
-        <v>54</v>
+        <v>4</v>
       </c>
       <c r="B7" s="18" t="str">
-        <f>'data'!D57</f>
+        <f>'data'!D7</f>
       </c>
     </row>
     <row r="8" ht="270" customHeight="true">
       <c r="A8" s="17">
-        <v>55</v>
+        <v>6</v>
       </c>
       <c r="B8" s="18" t="str">
-        <f>'data'!D58</f>
+        <f>'data'!D9</f>
       </c>
     </row>
     <row r="9" ht="270" customHeight="true">
       <c r="A9" s="17">
-        <v>56</v>
+        <v>7</v>
       </c>
       <c r="B9" s="18" t="str">
-        <f>'data'!D59</f>
+        <f>'data'!D10</f>
       </c>
     </row>
     <row r="10" ht="270" customHeight="true">
       <c r="A10" s="17">
-        <v>19</v>
+        <v>57</v>
       </c>
       <c r="B10" s="18" t="str">
-        <f>'data'!D22</f>
+        <f>'data'!D60</f>
       </c>
     </row>
     <row r="11" ht="270" customHeight="true">
       <c r="A11" s="17">
-        <v>58</v>
+        <v>10</v>
       </c>
       <c r="B11" s="18" t="str">
-        <f>'data'!D61</f>
+        <f>'data'!D13</f>
       </c>
     </row>
     <row r="12" ht="270" customHeight="true">
       <c r="A12" s="17">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="B12" s="18" t="str">
-        <f>'data'!D9</f>
+        <f>'data'!D32</f>
       </c>
     </row>
     <row r="13" ht="270" customHeight="true">
       <c r="A13" s="17">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="B13" s="18" t="str">
-        <f>'data'!D23</f>
+        <f>'data'!D63</f>
       </c>
     </row>
     <row r="14" ht="270" customHeight="true">
       <c r="A14" s="17">
-        <v>7</v>
+        <v>77</v>
       </c>
       <c r="B14" s="18" t="str">
-        <f>'data'!D10</f>
+        <f>'data'!D80</f>
       </c>
     </row>
     <row r="15" ht="270" customHeight="true">
@@ -4773,10 +4773,10 @@
     </row>
     <row r="18" ht="270" customHeight="true">
       <c r="A18" s="17">
-        <v>65</v>
+        <v>20</v>
       </c>
       <c r="B18" s="18" t="str">
-        <f>'data'!D68</f>
+        <f>'data'!D23</f>
       </c>
     </row>
     <row r="19" ht="270" customHeight="true">
@@ -4797,10 +4797,10 @@
     </row>
     <row r="21" ht="270" customHeight="true">
       <c r="A21" s="17">
-        <v>82</v>
+        <v>71</v>
       </c>
       <c r="B21" s="18" t="str">
-        <f>'data'!D85</f>
+        <f>'data'!D74</f>
       </c>
     </row>
     <row r="22" ht="270" customHeight="true">
@@ -4829,10 +4829,10 @@
     </row>
     <row r="25" ht="270" customHeight="true">
       <c r="A25" s="17">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B25" s="18" t="str">
-        <f>'data'!D74</f>
+        <f>'data'!D70</f>
       </c>
     </row>
     <row r="26" ht="270" customHeight="true">
@@ -4869,82 +4869,82 @@
     </row>
     <row r="30" ht="270" customHeight="true">
       <c r="A30" s="17">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="B30" s="18" t="str">
-        <f>'data'!D18</f>
+        <f>'data'!D8</f>
       </c>
     </row>
     <row r="31" ht="270" customHeight="true">
       <c r="A31" s="17">
-        <v>11</v>
+        <v>38</v>
       </c>
       <c r="B31" s="18" t="str">
-        <f>'data'!D14</f>
+        <f>'data'!D41</f>
       </c>
     </row>
     <row r="32" ht="270" customHeight="true">
       <c r="A32" s="17">
-        <v>12</v>
+        <v>78</v>
       </c>
       <c r="B32" s="18" t="str">
-        <f>'data'!D15</f>
+        <f>'data'!D81</f>
       </c>
     </row>
     <row r="33" ht="270" customHeight="true">
       <c r="A33" s="17">
-        <v>8</v>
+        <v>79</v>
       </c>
       <c r="B33" s="18" t="str">
-        <f>'data'!D11</f>
+        <f>'data'!D82</f>
       </c>
     </row>
     <row r="34" ht="270" customHeight="true">
       <c r="A34" s="17">
-        <v>9</v>
+        <v>80</v>
       </c>
       <c r="B34" s="18" t="str">
-        <f>'data'!D12</f>
+        <f>'data'!D83</f>
       </c>
     </row>
     <row r="35" ht="270" customHeight="true">
       <c r="A35" s="17">
-        <v>5</v>
+        <v>81</v>
       </c>
       <c r="B35" s="18" t="str">
-        <f>'data'!D8</f>
+        <f>'data'!D84</f>
       </c>
     </row>
     <row r="36" ht="270" customHeight="true">
       <c r="A36" s="17">
-        <v>67</v>
+        <v>31</v>
       </c>
       <c r="B36" s="18" t="str">
-        <f>'data'!D70</f>
+        <f>'data'!D34</f>
       </c>
     </row>
     <row r="37" ht="270" customHeight="true">
       <c r="A37" s="17">
-        <v>4</v>
+        <v>83</v>
       </c>
       <c r="B37" s="18" t="str">
-        <f>'data'!D7</f>
+        <f>'data'!D86</f>
       </c>
     </row>
     <row r="38" ht="270" customHeight="true">
       <c r="A38" s="17">
-        <v>39</v>
+        <v>84</v>
       </c>
       <c r="B38" s="18" t="str">
-        <f>'data'!D42</f>
+        <f>'data'!D87</f>
       </c>
     </row>
     <row r="39" ht="270" customHeight="true">
       <c r="A39" s="17">
-        <v>85</v>
+        <v>37</v>
       </c>
       <c r="B39" s="18" t="str">
-        <f>'data'!D88</f>
+        <f>'data'!D40</f>
       </c>
     </row>
     <row r="40" ht="270" customHeight="true">
@@ -4957,18 +4957,18 @@
     </row>
     <row r="41" ht="270" customHeight="true">
       <c r="A41" s="17">
-        <v>87</v>
+        <v>39</v>
       </c>
       <c r="B41" s="18" t="str">
-        <f>'data'!D90</f>
+        <f>'data'!D42</f>
       </c>
     </row>
     <row r="42" ht="270" customHeight="true">
       <c r="A42" s="17">
-        <v>88</v>
+        <v>40</v>
       </c>
       <c r="B42" s="18" t="str">
-        <f>'data'!D91</f>
+        <f>'data'!D43</f>
       </c>
     </row>
     <row r="43" ht="270" customHeight="true">
@@ -5377,7 +5377,7 @@
     </row>
     <row r="4">
       <c r="A4" s="19" t="str">
-        <f>'data'!$B$26</f>
+        <f>'data'!$B$28</f>
       </c>
       <c r="B4" s="22"/>
       <c r="C4" s="22"/>
@@ -5461,7 +5461,7 @@
     </row>
     <row r="12">
       <c r="A12" s="19" t="str">
-        <f>'data'!$B$25</f>
+        <f>'data'!$B$81</f>
       </c>
       <c r="B12" s="22"/>
       <c r="C12" s="22"/>
@@ -5469,7 +5469,7 @@
       <c r="E12" s="22"/>
       <c r="F12" s="22"/>
       <c r="G12" s="19" t="str">
-        <f>'data'!$B$62</f>
+        <f>'data'!$B$58</f>
       </c>
       <c r="I12" s="19" t="str">
         <f>'data'!$B$54</f>
@@ -5545,7 +5545,7 @@
     </row>
     <row r="20">
       <c r="A20" s="19" t="str">
-        <f>'data'!$B$5</f>
+        <f>'data'!$B$61</f>
       </c>
       <c r="B20" s="22"/>
       <c r="C20" s="22"/>
@@ -5553,10 +5553,10 @@
       <c r="E20" s="22"/>
       <c r="F20" s="22"/>
       <c r="G20" s="19" t="str">
-        <f>'data'!$B$83</f>
+        <f>'data'!$B$40</f>
       </c>
       <c r="I20" s="19" t="str">
-        <f>'data'!$B$57</f>
+        <f>'data'!$B$7</f>
       </c>
       <c r="J20" s="22"/>
       <c r="K20" s="22"/>
@@ -5564,7 +5564,7 @@
       <c r="M20" s="22"/>
       <c r="N20" s="22"/>
       <c r="O20" s="19" t="str">
-        <f>'data'!$B$56</f>
+        <f>'data'!$B$18</f>
       </c>
     </row>
     <row r="22">
@@ -5637,10 +5637,10 @@
       <c r="E28" s="22"/>
       <c r="F28" s="22"/>
       <c r="G28" s="19" t="str">
-        <f>'data'!$B$59</f>
+        <f>'data'!$B$43</f>
       </c>
       <c r="I28" s="19" t="str">
-        <f>'data'!$B$22</f>
+        <f>'data'!$B$60</f>
       </c>
       <c r="J28" s="22"/>
       <c r="K28" s="22"/>
@@ -5648,7 +5648,7 @@
       <c r="M28" s="22"/>
       <c r="N28" s="22"/>
       <c r="O28" s="19" t="str">
-        <f>'data'!$B$59</f>
+        <f>'data'!$B$10</f>
       </c>
     </row>
     <row r="30">
@@ -5713,7 +5713,7 @@
     </row>
     <row r="36">
       <c r="A36" s="19" t="str">
-        <f>'data'!$B$79</f>
+        <f>'data'!$B$56</f>
       </c>
       <c r="B36" s="22"/>
       <c r="C36" s="22"/>
@@ -5724,7 +5724,7 @@
         <f>'data'!$B$17</f>
       </c>
       <c r="I36" s="19" t="str">
-        <f>'data'!$B$23</f>
+        <f>'data'!$B$63</f>
       </c>
       <c r="J36" s="22"/>
       <c r="K36" s="22"/>
@@ -5732,7 +5732,7 @@
       <c r="M36" s="22"/>
       <c r="N36" s="22"/>
       <c r="O36" s="19" t="str">
-        <f>'data'!$B$9</f>
+        <f>'data'!$B$32</f>
       </c>
     </row>
     <row r="38">
@@ -5889,7 +5889,7 @@
       <c r="E52" s="22"/>
       <c r="F52" s="22"/>
       <c r="G52" s="19" t="str">
-        <f>'data'!$B$63</f>
+        <f>'data'!$B$68</f>
       </c>
       <c r="I52" s="19" t="str">
         <f>'data'!$B$4</f>
@@ -5900,7 +5900,7 @@
       <c r="M52" s="22"/>
       <c r="N52" s="22"/>
       <c r="O52" s="19" t="str">
-        <f>'data'!$B$68</f>
+        <f>'data'!$B$23</f>
       </c>
     </row>
     <row r="54">
@@ -5965,7 +5965,7 @@
     </row>
     <row r="60">
       <c r="A60" s="19" t="str">
-        <f>'data'!$B$84</f>
+        <f>'data'!$B$27</f>
       </c>
       <c r="B60" s="22"/>
       <c r="C60" s="22"/>
@@ -5973,10 +5973,10 @@
       <c r="E60" s="22"/>
       <c r="F60" s="22"/>
       <c r="G60" s="19" t="str">
-        <f>'data'!$B$86</f>
+        <f>'data'!$B$26</f>
       </c>
       <c r="I60" s="19" t="str">
-        <f>'data'!$B$88</f>
+        <f>'data'!$B$71</f>
       </c>
       <c r="J60" s="22"/>
       <c r="K60" s="22"/>
@@ -5984,7 +5984,7 @@
       <c r="M60" s="22"/>
       <c r="N60" s="22"/>
       <c r="O60" s="19" t="str">
-        <f>'data'!$B$85</f>
+        <f>'data'!$B$70</f>
       </c>
     </row>
     <row r="62">
@@ -6049,7 +6049,7 @@
     </row>
     <row r="68">
       <c r="A68" s="19" t="str">
-        <f>'data'!$B$29</f>
+        <f>'data'!$B$55</f>
       </c>
       <c r="B68" s="22"/>
       <c r="C68" s="22"/>
@@ -6057,7 +6057,7 @@
       <c r="E68" s="22"/>
       <c r="F68" s="22"/>
       <c r="G68" s="19" t="str">
-        <f>'data'!$B$28</f>
+        <f>'data'!$B$57</f>
       </c>
       <c r="I68" s="19" t="str">
         <f>'data'!$B$73</f>
@@ -6133,7 +6133,7 @@
     </row>
     <row r="76">
       <c r="A76" s="19" t="str">
-        <f>'data'!$B$32</f>
+        <f>'data'!$B$62</f>
       </c>
       <c r="B76" s="22"/>
       <c r="C76" s="22"/>
@@ -6225,10 +6225,10 @@
       <c r="E84" s="22"/>
       <c r="F84" s="22"/>
       <c r="G84" s="19" t="str">
-        <f>'data'!$B$41</f>
+        <f>'data'!$B$19</f>
       </c>
       <c r="I84" s="19" t="str">
-        <f>'data'!$B$18</f>
+        <f>'data'!$B$8</f>
       </c>
       <c r="J84" s="22"/>
       <c r="K84" s="22"/>
@@ -6312,7 +6312,7 @@
         <f>'data'!$B$9</f>
       </c>
       <c r="I92" s="19" t="str">
-        <f>'data'!$B$11</f>
+        <f>'data'!$B$82</f>
       </c>
       <c r="J92" s="22"/>
       <c r="K92" s="22"/>
@@ -6320,7 +6320,7 @@
       <c r="M92" s="22"/>
       <c r="N92" s="22"/>
       <c r="O92" s="19" t="str">
-        <f>'data'!$B$15</f>
+        <f>'data'!$B$81</f>
       </c>
     </row>
     <row r="94">
@@ -6385,7 +6385,7 @@
     </row>
     <row r="100">
       <c r="A100" s="19" t="str">
-        <f>'data'!$B$12</f>
+        <f>'data'!$B$71</f>
       </c>
       <c r="B100" s="22"/>
       <c r="C100" s="22"/>
@@ -6393,10 +6393,10 @@
       <c r="E100" s="22"/>
       <c r="F100" s="22"/>
       <c r="G100" s="19" t="str">
-        <f>'data'!$B$49</f>
+        <f>'data'!$B$11</f>
       </c>
       <c r="I100" s="19" t="str">
-        <f>'data'!$B$70</f>
+        <f>'data'!$B$5</f>
       </c>
       <c r="J100" s="22"/>
       <c r="K100" s="22"/>
@@ -6404,7 +6404,7 @@
       <c r="M100" s="22"/>
       <c r="N100" s="22"/>
       <c r="O100" s="19" t="str">
-        <f>'data'!$B$8</f>
+        <f>'data'!$B$84</f>
       </c>
     </row>
     <row r="102">
@@ -6469,7 +6469,7 @@
     </row>
     <row r="108">
       <c r="A108" s="19" t="str">
-        <f>'data'!$B$15</f>
+        <f>'data'!$B$91</f>
       </c>
       <c r="B108" s="22"/>
       <c r="C108" s="22"/>
@@ -6477,10 +6477,10 @@
       <c r="E108" s="22"/>
       <c r="F108" s="22"/>
       <c r="G108" s="19" t="str">
-        <f>'data'!$B$87</f>
+        <f>'data'!$B$90</f>
       </c>
       <c r="I108" s="19" t="str">
-        <f>'data'!$B$88</f>
+        <f>'data'!$B$40</f>
       </c>
       <c r="J108" s="22"/>
       <c r="K108" s="22"/>
@@ -6488,7 +6488,7 @@
       <c r="M108" s="22"/>
       <c r="N108" s="22"/>
       <c r="O108" s="19" t="str">
-        <f>'data'!$B$42</f>
+        <f>'data'!$B$87</f>
       </c>
     </row>
     <row r="110">
@@ -6564,7 +6564,7 @@
         <f>'data'!$B$45</f>
       </c>
       <c r="I116" s="19" t="str">
-        <f>'data'!$B$91</f>
+        <f>'data'!$B$43</f>
       </c>
       <c r="J116" s="22"/>
       <c r="K116" s="22"/>
@@ -6572,7 +6572,7 @@
       <c r="M116" s="22"/>
       <c r="N116" s="22"/>
       <c r="O116" s="19" t="str">
-        <f>'data'!$B$90</f>
+        <f>'data'!$B$42</f>
       </c>
     </row>
     <row r="118">
@@ -6637,7 +6637,7 @@
     </row>
     <row r="124">
       <c r="A124" s="19" t="str">
-        <f>'data'!$B$11</f>
+        <f>'data'!$B$49</f>
       </c>
       <c r="B124" s="22"/>
       <c r="C124" s="22"/>
@@ -6729,7 +6729,7 @@
       <c r="E137" s="22"/>
       <c r="F137" s="22"/>
       <c r="G137" s="19" t="str">
-        <f>'data'!$B$27</f>
+        <f>'data'!$B$79</f>
       </c>
       <c r="I137" s="19" t="str">
         <f>CONCATENATE("M 18 ",O14)</f>
@@ -6813,7 +6813,7 @@
       <c r="E145" s="22"/>
       <c r="F145" s="22"/>
       <c r="G145" s="19" t="str">
-        <f>'data'!$B$82</f>
+        <f>'data'!$B$29</f>
       </c>
       <c r="I145" s="19" t="str">
         <f>CONCATENATE("M 19 ",O22)</f>
@@ -6824,7 +6824,7 @@
       <c r="M145" s="22"/>
       <c r="N145" s="22"/>
       <c r="O145" s="19" t="str">
-        <f>'data'!$B$55</f>
+        <f>'data'!$B$11</f>
       </c>
     </row>
     <row r="147">
@@ -6897,7 +6897,7 @@
       <c r="E153" s="22"/>
       <c r="F153" s="22"/>
       <c r="G153" s="19" t="str">
-        <f>'data'!$B$80</f>
+        <f>'data'!$B$42</f>
       </c>
       <c r="I153" s="19" t="str">
         <f>CONCATENATE("M 20 ",O30)</f>
@@ -6908,7 +6908,7 @@
       <c r="M153" s="22"/>
       <c r="N153" s="22"/>
       <c r="O153" s="19" t="str">
-        <f>'data'!$B$58</f>
+        <f>'data'!$B$9</f>
       </c>
     </row>
     <row r="155">
@@ -6981,7 +6981,7 @@
       <c r="E161" s="22"/>
       <c r="F161" s="22"/>
       <c r="G161" s="19" t="str">
-        <f>'data'!$B$30</f>
+        <f>'data'!$B$85</f>
       </c>
       <c r="I161" s="19" t="str">
         <f>CONCATENATE("M 21 ",O38)</f>
@@ -6992,7 +6992,7 @@
       <c r="M161" s="22"/>
       <c r="N161" s="22"/>
       <c r="O161" s="19" t="str">
-        <f>'data'!$B$61</f>
+        <f>'data'!$B$41</f>
       </c>
     </row>
     <row r="163">
@@ -7065,7 +7065,7 @@
       <c r="E169" s="22"/>
       <c r="F169" s="22"/>
       <c r="G169" s="19" t="str">
-        <f>'data'!$B$60</f>
+        <f>'data'!$B$22</f>
       </c>
       <c r="I169" s="19" t="str">
         <f>CONCATENATE("M 22 ",O46)</f>
@@ -7076,7 +7076,7 @@
       <c r="M169" s="22"/>
       <c r="N169" s="22"/>
       <c r="O169" s="19" t="str">
-        <f>'data'!$B$10</f>
+        <f>'data'!$B$80</f>
       </c>
     </row>
     <row r="171">
@@ -7149,7 +7149,7 @@
       <c r="E177" s="22"/>
       <c r="F177" s="22"/>
       <c r="G177" s="19" t="str">
-        <f>'data'!$B$64</f>
+        <f>'data'!$B$25</f>
       </c>
       <c r="I177" s="19" t="str">
         <f>CONCATENATE("M 23 ",O54)</f>
@@ -7233,7 +7233,7 @@
       <c r="E185" s="22"/>
       <c r="F185" s="22"/>
       <c r="G185" s="19" t="str">
-        <f>'data'!$B$30</f>
+        <f>'data'!$B$19</f>
       </c>
       <c r="I185" s="19" t="str">
         <f>CONCATENATE("M 24 ",O62)</f>
@@ -7496,7 +7496,7 @@
       <c r="M209" s="22"/>
       <c r="N209" s="22"/>
       <c r="O209" s="19" t="str">
-        <f>'data'!$B$42</f>
+        <f>'data'!$B$41</f>
       </c>
     </row>
     <row r="211">
@@ -7569,7 +7569,7 @@
       <c r="E217" s="22"/>
       <c r="F217" s="22"/>
       <c r="G217" s="19" t="str">
-        <f>'data'!$B$41</f>
+        <f>'data'!$B$64</f>
       </c>
       <c r="I217" s="19" t="str">
         <f>CONCATENATE("M 29 ",O102)</f>
@@ -7580,7 +7580,7 @@
       <c r="M217" s="22"/>
       <c r="N217" s="22"/>
       <c r="O217" s="19" t="str">
-        <f>'data'!$B$12</f>
+        <f>'data'!$B$83</f>
       </c>
     </row>
     <row r="219">
@@ -7664,7 +7664,7 @@
       <c r="M225" s="22"/>
       <c r="N225" s="22"/>
       <c r="O225" s="19" t="str">
-        <f>'data'!$B$7</f>
+        <f>'data'!$B$86</f>
       </c>
     </row>
     <row r="227">
@@ -9282,7 +9282,7 @@
     </row>
     <row r="7">
       <c r="C7" s="16" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="D7" s="15"/>
       <c r="E7" s="12"/>
@@ -9311,7 +9311,7 @@
       <c r="C14" s="16"/>
       <c r="D14" s="16"/>
       <c r="E14" s="16" t="s">
-        <v>74</v>
+        <v>179</v>
       </c>
       <c r="I14" s="12"/>
       <c r="K14" s="12"/>
@@ -9332,7 +9332,7 @@
     </row>
     <row r="17">
       <c r="C17" s="16" t="s">
-        <v>141</v>
+        <v>129</v>
       </c>
       <c r="G17" s="12"/>
       <c r="K17" s="12"/>
@@ -9348,7 +9348,7 @@
     </row>
     <row r="19">
       <c r="C19" s="16" t="s">
-        <v>68</v>
+        <v>132</v>
       </c>
       <c r="D19" s="15"/>
       <c r="E19" s="12"/>
@@ -9366,7 +9366,7 @@
       <c r="C22" s="16"/>
       <c r="D22" s="16"/>
       <c r="E22" s="16" t="s">
-        <v>184</v>
+        <v>79</v>
       </c>
       <c r="K22" s="12"/>
     </row>
@@ -9383,7 +9383,7 @@
     </row>
     <row r="25">
       <c r="C25" s="16" t="s">
-        <v>186</v>
+        <v>40</v>
       </c>
       <c r="G25" s="12"/>
       <c r="H25" s="14"/>
@@ -9402,7 +9402,7 @@
     </row>
     <row r="27">
       <c r="C27" s="16" t="s">
-        <v>24</v>
+        <v>138</v>
       </c>
       <c r="D27" s="15"/>
       <c r="E27" s="12"/>
@@ -9423,7 +9423,7 @@
       <c r="C30" s="16"/>
       <c r="D30" s="16"/>
       <c r="E30" s="16" t="s">
-        <v>181</v>
+        <v>44</v>
       </c>
       <c r="I30" s="12"/>
     </row>
@@ -9441,7 +9441,7 @@
     </row>
     <row r="33">
       <c r="C33" s="16" t="s">
-        <v>132</v>
+        <v>46</v>
       </c>
       <c r="G33" s="12"/>
     </row>
@@ -9512,7 +9512,7 @@
     </row>
     <row r="7">
       <c r="C7" s="16" t="s">
-        <v>179</v>
+        <v>123</v>
       </c>
       <c r="D7" s="15"/>
       <c r="E7" s="12"/>
@@ -9541,7 +9541,7 @@
       <c r="C14" s="16"/>
       <c r="D14" s="16"/>
       <c r="E14" s="16" t="s">
-        <v>54</v>
+        <v>190</v>
       </c>
       <c r="I14" s="12"/>
       <c r="K14" s="12"/>
@@ -9596,7 +9596,7 @@
       <c r="C22" s="16"/>
       <c r="D22" s="16"/>
       <c r="E22" s="16" t="s">
-        <v>135</v>
+        <v>60</v>
       </c>
       <c r="K22" s="12"/>
     </row>
@@ -9613,7 +9613,7 @@
     </row>
     <row r="25">
       <c r="C25" s="16" t="s">
-        <v>144</v>
+        <v>158</v>
       </c>
       <c r="G25" s="12"/>
       <c r="H25" s="14"/>
@@ -9653,7 +9653,7 @@
       <c r="C30" s="16"/>
       <c r="D30" s="16"/>
       <c r="E30" s="16" t="s">
-        <v>147</v>
+        <v>68</v>
       </c>
       <c r="I30" s="12"/>
     </row>
@@ -9671,7 +9671,7 @@
     </row>
     <row r="33">
       <c r="C33" s="16" t="s">
-        <v>192</v>
+        <v>71</v>
       </c>
       <c r="G33" s="12"/>
     </row>
@@ -9685,7 +9685,7 @@
     </row>
     <row r="35">
       <c r="C35" s="16" t="s">
-        <v>188</v>
+        <v>74</v>
       </c>
       <c r="D35" s="15"/>
       <c r="E35" s="12"/>

</xml_diff>

<commit_message>
chore(examples): regenerate the example workbooks for the fixed Names to Print widths
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/playoffs-example-large-seeded.xlsx
+++ b/playoffs-example-large-seeded.xlsx
@@ -1472,7 +1472,7 @@
       <alignment horizontal="center" shrinkToFit="true" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" shrinkToFit="true" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
@@ -4782,8 +4782,8 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>
   <cols>
-    <col customWidth="true" max="1" min="1" width="30"/>
-    <col customWidth="true" max="2" min="2" width="160"/>
+    <col customWidth="true" max="1" min="1" width="40"/>
+    <col customWidth="true" max="2" min="2" width="140"/>
   </cols>
   <sheetData>
     <row r="1" ht="270" customHeight="true">
@@ -5183,8 +5183,8 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>
   <cols>
-    <col customWidth="true" max="1" min="1" width="30"/>
-    <col customWidth="true" max="2" min="2" width="160"/>
+    <col customWidth="true" max="1" min="1" width="40"/>
+    <col customWidth="true" max="2" min="2" width="140"/>
   </cols>
   <sheetData>
     <row r="1" ht="270" customHeight="true">

</xml_diff>